<commit_message>
Expand Day1 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -15905,11 +15905,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -15917,48 +15917,191 @@
     <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:3">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ACGO名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>模板综合双优学生</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>模板题和非模板综合题都表现突出</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>基础扎实迁移待提升学生</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>模板题较稳，综合题优化和迁移还需加强</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>模板稳定难题突破不足学生</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>基础题完成较好，难题突破和部分分策略不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>思维突出模板待稳学生</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>非模板题有想法，模板和代码稳定性不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>思路正确细节失分学生</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>大方向能判断，细节和检查习惯导致失分</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>观察题表现较好学生</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>规律观察类题目表现较好，复杂实现仍需练习</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>部分分意识较好学生</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>能争取部分分，完整解法和稳定性还需提升</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>模板掌握不均学生</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>部分模板会，树上/图论/DP等模块存在断点</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>综合题畏难学生</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>基础题可完成一部分，综合题容易放弃或停顿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>模板基础和代码实现都需要优先补强</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -25277,11 +25420,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="54" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -25289,7 +25432,7 @@
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="70" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -25344,15 +25487,15 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="76" customHeight="1">
+    <row r="2" ht="92" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Day1 主要进行开班梳理与综合摸底：上午复习并串讲提高组常见算法模板，帮助学生回顾并查集、树状数组、树上问题、动态规划、最短路等基础能力；下午进行模板题与综合题结合的摸底测试，测试内容既包含默认应掌握的模板题，也包含需要现场观察、分析和优化的综合题；晚上围绕测试进行讲解、补题和错题复盘。</t>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A类学生</t>
+          <t>模板综合双优学生</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -25392,24 +25535,24 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>A类学生在今日摸底中整体表现突出，基础模板题完成度高，能够较稳定地写出常见算法模板，并在代码实现中保持较好的准确率。面对非模板综合题时，能够主动观察题目性质，尝试从数据范围、特殊情况和可优化方向入手分析问题，具备较强的独立思考能力。后续建议继续保持模板熟练度，同时在综合题中加强检查习惯，避免因细节失误影响最终得分。</t>
+          <t>孩子今天的整体表现非常稳定，基础模板题完成度高，说明常见算法框架掌握得比较扎实；在后面的综合题中，也能主动观察题目条件，尝试从规律、数据范围和特殊情况入手推进思路。比较难得的是，孩子不是只会套固定方法，而是能把学过的知识迁移到新题里。后续建议继续保持这种做题节奏，同时在提交前多留一点时间检查边界和细节，争取把会做的分数拿得更稳。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="76" customHeight="1">
+    <row r="3" ht="92" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Day1 主要进行开班梳理与综合摸底：上午复习并串讲提高组常见算法模板，帮助学生回顾并查集、树状数组、树上问题、动态规划、最短路等基础能力；下午进行模板题与综合题结合的摸底测试，测试内容既包含默认应掌握的模板题，也包含需要现场观察、分析和优化的综合题；晚上围绕测试进行讲解、补题和错题复盘。</t>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B类学生</t>
+          <t>基础扎实迁移待提升学生</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -25419,12 +25562,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -25444,39 +25587,39 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>B类学生今日整体表现较稳定，基础模板题大多能够完成，说明前期常见算法框架已有一定掌握；但在实现细节和题型迁移上仍需要加强，遇到非模板综合题时容易停留在直观做法，进一步优化和总结规律的能力还需要训练。后续建议重点巩固模板题的熟练度，补题时多复盘“为什么这样优化”，逐步提升从已学知识迁移到新题的能力。</t>
+          <t>孩子今天在基础模板题上的表现比较稳，能够看出前期知识点不是空着的，常见题型有一定熟练度。遇到综合题时，孩子能写出一部分思路，但从基础做法继续往优化方向推进时还会有些卡顿。这个阶段最需要训练的不是单纯多记模板，而是学会判断“这道题为什么能优化”。后续补题时建议多复盘思路变化过程，把会做的基础题转化成更强的综合解题能力。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="76" customHeight="1">
+    <row r="4" ht="92" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Day1 主要进行开班梳理与综合摸底：上午复习并串讲提高组常见算法模板，帮助学生回顾并查集、树状数组、树上问题、动态规划、最短路等基础能力；下午进行模板题与综合题结合的摸底测试，测试内容既包含默认应掌握的模板题，也包含需要现场观察、分析和优化的综合题；晚上围绕测试进行讲解、补题和错题复盘。</t>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C类学生</t>
+          <t>模板稳定难题突破不足学生</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -25496,16 +25639,380 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C类学生今日主要目标是完成基础摸底和查漏补缺。从测试情况看，模板题中仍有部分知识点不够熟练，代码实现容易出现漏条件、边界处理不清或调试时间较长的问题；面对综合题时，独立分析难度较大，需要更多提示才能推进。后续建议先把基础模板补扎实，优先完成并查集、树状数组、动态规划和图论基础题的订正与默写，再逐步尝试综合题中的简单部分分。</t>
+          <t>孩子今天基础部分完成得不错，固定方法类题目基本能够进入状态，说明课堂中学过的核心内容有吸收。但在难度提升的综合题上，孩子容易等到完整思路再动手，导致可拿的部分分没有充分争取。竞赛测试中，能把简单分、部分分先拿到非常重要。后续建议训练分层做题意识：先完成确定会做的部分，再逐步尝试优化和突破难点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>思维突出模板待稳学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在综合题中的思维亮点比较明显，遇到新题时愿意观察规律，也能提出一些有价值的方向，说明孩子的思考能力是不错的。不过基础模板题和代码实现的稳定性还需要加强，有些分数并不是不会想，而是卡在固定写法、边界处理或调试细节上。后续建议把常见模板练到更熟，减少基础实现带来的消耗，这样孩子的思维优势才能在考试中更好地转化成分数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>思路正确细节失分学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天不少题目的大方向是能判断出来的，说明理解能力并不弱，但在代码细节上还不够稳，例如边界、数组范围、初始化、输出格式等位置容易出现小问题。这类失分比较可惜，因为它不是完全不会，而是最后实现和检查环节没有守住。后续建议养成写完后自查样例、边界和特殊情况的习惯，尤其是模板题要做到又快又准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>观察题表现较好学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天在需要观察规律的题目上表现不错，能够从样例和题目条件中找到一些突破口，这说明孩子并不是机械做题，具备一定的分析意识。相对来说，涉及较复杂数据结构或树上处理的题目会更吃力一些，代码实现也容易变慢。后续建议保持这种观察和归纳能力，同时补强基础算法实现，让思路和代码能够更顺畅地连接起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>部分分意识较好学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天在不会完整解决的题目上，能够尝试从简单情况或部分数据入手，这是一个很好的竞赛习惯。虽然目前完整解法和代码稳定性还需要提升，但愿意先拿可拿的分，说明孩子已经开始建立考试策略。后续建议在补题时把“部分分做法”和“满分做法”放在一起对比，理解每一步优化解决了什么问题，这样进步会更明显。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>模板掌握不均学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天的表现能看出有些基础内容是掌握的，但不同模块之间不太均衡：熟悉的题型可以推进，不熟悉的模板就容易卡住，代码实现也会受到影响。Day1 的摸底很适合暴露这类问题，因为它覆盖了多个基础方向。后续建议不要急着刷难题，先把薄弱模板逐个补齐，尤其要把常见写法、适用场景和易错点整理清楚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>综合题畏难学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天在基础题上能完成一部分内容，但一遇到题面较长或条件较多的综合题，就容易出现停顿，不太敢继续拆解。其实这类题不一定要一开始就想出完整做法，可以先从样例、特殊情况和小数据入手。后续老师会引导孩子把复杂题拆成几个小问题来处理，也建议孩子补题时先写出自己能想到的部分，不要因为暂时没有满分思路就直接放弃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day1 主要进行开班梳理与综合摸底：上午完成开班说明、CSP-S复赛题型总结、S组一等奖得分情况分析，并结合典型真题感受复赛题目的难度差异；同时梳理历年高频考点和冲刺一等需要具备的能力。下午进行摸底考试，内容包含基础模板题和4道综合测试题，用于了解学生当前模板掌握、代码实现和综合分析能力；晚上进行测试讲解与补题。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天主要完成了基础摸底，也暴露出一些需要优先补强的地方。当前阶段基础模板还不够熟练，写代码时容易在步骤、变量和边界处理上花较多时间；综合题独立推进难度也比较大。后续建议先把基础题订正到位，尤其是固定方法类题目要反复练到能独立写出，再逐步尝试综合题中的简单部分。只要基础补起来，后面的训练会顺很多。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
       <formula1>'名单'!$A:$A</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Day2-Day4 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -15909,7 +15909,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -16441,6 +16441,176 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>真题综合性较强，基础分析和代码都需补强</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>特殊性质把握优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>能快速抓住题目关键性质，并将其转化为简洁做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>关键转化能力较强学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>能把题目条件转成数学式、可达状态或区间统计问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>数学规律敏感学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>对总和变化、奇偶/大小关系、最高位等规律比较敏感。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>排序二分应用较好学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>能想到排序、二分、双指针等优化方式处理统计类问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>树上问题理解较好学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>对树上距离、追赶、路径覆盖等题有思路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>位运算题有亮点学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>异或、二进制最高位等题目有想法，但实现复杂度较高。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>特殊性质能看出但落码不稳学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>能发现部分性质，但代码实现和边界处理影响得分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>暴力到正解过渡不足学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>能写暴力或部分分，难以继续利用特殊性质优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>部分分与特殊数据意识较好学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>能根据特殊性质、小数据或简化情况争取部分分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>性质题适应待加强学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>题目条件较复杂时，不太会主动寻找关键性质。</t>
         </is>
       </c>
     </row>
@@ -30747,646 +30917,797 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.125" customWidth="1"/>
-    <col min="2" max="3" width="15.5833333333333" customWidth="1"/>
-    <col min="4" max="4" width="24.125" customWidth="1"/>
-    <col min="5" max="5" width="22.75" customWidth="1"/>
-    <col min="6" max="9" width="25.875" customWidth="1"/>
-    <col min="10" max="10" width="51.3666666666667" customWidth="1"/>
-    <col min="11" max="11" width="14.25" customWidth="1"/>
-    <col min="12" max="12" width="61.25"/>
-    <col min="13" max="13" width="120.75" customWidth="1"/>
-    <col min="14" max="14" width="119.75"/>
-    <col min="15" max="15" width="76.875" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:15">
-      <c r="A1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="55" t="s">
-        <v>374</v>
-      </c>
-      <c r="E1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>18</v>
-      </c>
-      <c r="J1" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="55" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" s="55" t="s">
-        <v>374</v>
-      </c>
-      <c r="N1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="O1" s="55" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="2" ht="162.75" customHeight="1" spans="1:15">
-      <c r="A2" s="120" t="s">
-        <v>375</v>
-      </c>
-      <c r="B2" s="139" t="s">
-        <v>167</v>
-      </c>
-      <c r="C2" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="D2" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="E2" s="108" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="108" t="s">
-        <v>201</v>
-      </c>
-      <c r="J2" s="120" t="str">
-        <f>A$2&amp;""&amp;SUBSTITUTE(IF(OR(C2="A",C2="A-",C2="A+"),L$2,IF(OR(C2="B",C2="B-",C2="B+"),L$3,L$4)),"【xx】",B2)&amp;""&amp;SUBSTITUTE(IF(OR(D2="A",D2="A-",D2="A+"),N$2,IF(OR(D2="B",D2="B-",D2="B+"),N$3,N$4)),"【xx】",B2)&amp;""&amp;SUBSTITUTE(IF(OR(E2="A",E2="A-",E2="A+"),M$2,IF(OR(E2="B",E2="B-",E2="B+"),M$3,M$4)),"【xx】",B2)&amp;""&amp;SUBSTITUTE(IF(OR(F2="A",F2="A-",F2="A+"),O$2,IF(OR(F2="B",F2="B-",F2="B+"),O$3,O$4)),"【xx】",B2)</f>
-        <v>今天选讲了提高组的真题，重点讲解了在面对冗长代码时如何通过模块化拆分、封装函数来保持逻辑清晰，并介绍了哈希这一高效优化技巧，帮助同学们在解决字符串及模拟问题时更加得心应手。葛义同学课堂积极度良好。能够参与互动，跟上课堂节奏，表现出学习热情。葛义在本次测试中表现不错，葛义能够解决基础的问题，在做其他题目时能够去获取部分分数，在面对中等题的时候，也能能够分析出问题的类型，但是孩子对于普及组二分 or 双指针的使用不是很熟练，实现代码的时候遇到了困难，需要加强基础算法的熟练度，继续加油。后续会通过不断练习来提高算法优化技巧的熟练度。</v>
-      </c>
-      <c r="K2" s="55">
-        <f>IF(D2="A",1,0)*30+IF(D2="B",1,0)*20+IF(D2="C",1,0)*10+IF(E2="A",1,0)*30+IF(E2="B",1,0)*20+IF(E2="C",1,0)*10+IF(F2="A",1,0)*30+IF(F2="B",1,0)*20+IF(F2="C",1,0)*10</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="55" t="s">
-        <v>376</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="N2" s="55" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:15">
-      <c r="J3" s="120"/>
-      <c r="L3" s="55" t="s">
-        <v>379</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="N3" s="199" t="s">
-        <v>381</v>
-      </c>
-      <c r="O3" s="55" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:15">
-      <c r="J4" s="120"/>
-      <c r="L4" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="M4" s="55" t="s">
-        <v>384</v>
-      </c>
-      <c r="N4" s="199"/>
-      <c r="O4" s="55" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:15">
-      <c r="J5" s="120"/>
-    </row>
-    <row r="6" customHeight="1" spans="1:15">
-      <c r="J6" s="120"/>
-    </row>
-    <row r="7" customHeight="1" spans="1:15">
-      <c r="J7" s="120"/>
-    </row>
-    <row r="8" customHeight="1" spans="1:15">
-      <c r="J8" s="120"/>
-    </row>
-    <row r="9" ht="203.25" customHeight="1" spans="1:15">
-      <c r="B9" s="180" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="G9" s="131" t="s">
-        <v>385</v>
-      </c>
-      <c r="H9" s="131" t="s">
-        <v>386</v>
-      </c>
-      <c r="I9" s="131" t="s">
-        <v>387</v>
-      </c>
-      <c r="J9" s="200" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="10" ht="203.25" customHeight="1" spans="1:15">
-      <c r="B10" s="180" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="E10" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="G10" s="131" t="s">
-        <v>389</v>
-      </c>
-      <c r="H10" s="131" t="s">
-        <v>390</v>
-      </c>
-      <c r="I10" s="131" t="s">
-        <v>391</v>
-      </c>
-      <c r="J10" s="200" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="11" ht="189.75" customHeight="1" spans="1:15">
-      <c r="B11" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="G11" s="131" t="s">
-        <v>393</v>
-      </c>
-      <c r="H11" s="131" t="s">
-        <v>394</v>
-      </c>
-      <c r="I11" s="131" t="s">
-        <v>395</v>
-      </c>
-      <c r="J11" s="200" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="12" ht="203.25" customHeight="1" spans="1:15">
-      <c r="B12" s="180" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="132" t="s">
-        <v>397</v>
-      </c>
-      <c r="H12" s="132" t="s">
-        <v>398</v>
-      </c>
-      <c r="I12" s="131" t="s">
-        <v>399</v>
-      </c>
-      <c r="J12" s="200" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="13" ht="189.75" customHeight="1" spans="1:15">
-      <c r="B13" s="180" t="s">
-        <v>95</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="132" t="s">
-        <v>401</v>
-      </c>
-      <c r="H13" s="131" t="s">
-        <v>402</v>
-      </c>
-      <c r="I13" s="131" t="s">
-        <v>324</v>
-      </c>
-      <c r="J13" s="200" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="14" ht="135.75" customHeight="1" spans="1:15">
-      <c r="B14" s="180" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" s="131" t="s">
-        <v>404</v>
-      </c>
-      <c r="H14" s="131" t="s">
-        <v>405</v>
-      </c>
-      <c r="I14" s="131" t="s">
-        <v>406</v>
-      </c>
-      <c r="J14" s="200" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="15" ht="189.75" customHeight="1" spans="1:15">
-      <c r="B15" s="180" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="G15" s="132" t="s">
-        <v>408</v>
-      </c>
-      <c r="H15" s="131" t="s">
-        <v>409</v>
-      </c>
-      <c r="I15" s="131" t="s">
-        <v>410</v>
-      </c>
-      <c r="J15" s="200" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="16" ht="189.75" customHeight="1" spans="1:15">
-      <c r="B16" s="180" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="132" t="s">
-        <v>412</v>
-      </c>
-      <c r="H16" s="131" t="s">
-        <v>413</v>
-      </c>
-      <c r="I16" s="131" t="s">
-        <v>414</v>
-      </c>
-      <c r="J16" s="200" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="17" ht="162.75" customHeight="1" spans="1:14">
-      <c r="B17" s="180" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="G17" s="132" t="s">
-        <v>416</v>
-      </c>
-      <c r="H17" s="132" t="s">
-        <v>417</v>
-      </c>
-      <c r="I17" s="131" t="s">
-        <v>418</v>
-      </c>
-      <c r="J17" s="200" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="18" ht="162.75" customHeight="1" spans="1:14">
-      <c r="B18" s="180" t="s">
-        <v>100</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="131" t="s">
-        <v>420</v>
-      </c>
-      <c r="H18" s="131" t="s">
-        <v>421</v>
-      </c>
-      <c r="I18" s="131" t="s">
-        <v>422</v>
-      </c>
-      <c r="J18" s="200" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="19" ht="189.75" customHeight="1" spans="1:14">
-      <c r="B19" s="180" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E19" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="135" t="s">
-        <v>33</v>
-      </c>
-      <c r="G19" s="132" t="s">
-        <v>424</v>
-      </c>
-      <c r="H19" s="132" t="s">
-        <v>425</v>
-      </c>
-      <c r="I19" s="132" t="s">
-        <v>426</v>
-      </c>
-      <c r="J19" s="200" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="20" ht="162.75" customHeight="1" spans="1:14">
-      <c r="B20" s="180" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E20" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="135" t="s">
-        <v>33</v>
-      </c>
-      <c r="G20" s="131" t="s">
-        <v>428</v>
-      </c>
-      <c r="H20" s="131" t="s">
-        <v>429</v>
-      </c>
-      <c r="I20" s="131" t="s">
-        <v>430</v>
-      </c>
-      <c r="J20" s="200" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="21" ht="122.25" customHeight="1" spans="1:14">
-      <c r="B21" s="180" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="F21" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="132" t="s">
-        <v>432</v>
-      </c>
-      <c r="H21" s="131" t="s">
-        <v>433</v>
-      </c>
-      <c r="I21" s="131" t="s">
-        <v>434</v>
-      </c>
-      <c r="J21" s="200" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="22" customHeight="1" spans="1:14">
-      <c r="B22" s="180" t="s">
-        <v>110</v>
-      </c>
-      <c r="C22" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F22" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="G22" s="131" t="s">
-        <v>436</v>
-      </c>
-      <c r="H22" s="131" t="s">
-        <v>437</v>
-      </c>
-      <c r="I22" s="131" t="s">
-        <v>438</v>
-      </c>
-      <c r="J22" s="55" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="23" ht="315" customHeight="1" spans="1:14">
-      <c r="B23" s="180" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="F23" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="G23" s="132" t="s">
-        <v>440</v>
-      </c>
-      <c r="H23" s="132" t="s">
-        <v>441</v>
-      </c>
-      <c r="I23" s="131" t="s">
-        <v>442</v>
-      </c>
-      <c r="J23" s="56" t="s">
-        <v>443</v>
-      </c>
-      <c r="M23" s="55" t="s">
-        <v>444</v>
-      </c>
-      <c r="N23" s="55" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="24" ht="27.75" customHeight="1" spans="1:14">
-      <c r="B24" s="180" t="s">
-        <v>79</v>
-      </c>
-      <c r="C24" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D24" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E24" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="F24" s="135" t="s">
-        <v>293</v>
-      </c>
-      <c r="G24" s="131" t="s">
-        <v>446</v>
-      </c>
-      <c r="H24" s="131" t="s">
-        <v>447</v>
-      </c>
-      <c r="I24" s="131" t="s">
-        <v>448</v>
-      </c>
-      <c r="J24" s="56" t="s">
-        <v>449</v>
-      </c>
-      <c r="M24" s="55" t="s">
-        <v>450</v>
-      </c>
-      <c r="N24" s="55" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="25" customHeight="1" spans="1:14">
-      <c r="M25" s="55" t="s">
-        <v>452</v>
-      </c>
-      <c r="N25" s="55" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="31" customHeight="1" spans="1:14">
-      <c r="A31" s="56" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="37" ht="52.5" customHeight="1"/>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>课程内容</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>反思</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>反馈结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>特殊性质把握优秀学生</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>孩子今天在“从特殊性质出发”的训练中表现突出，能比较快地发现题目隐藏的关键规律，并把复杂操作转化成更简单的判断或计算。面对综合题时，孩子不是停留在表面模拟，而是会主动思考哪些条件真正影响答案。后续建议继续保持这种分析习惯，同时在写代码时加强边界和数据范围检查，争取让好思路更稳定地拿到分数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>关键转化能力较强学生</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>孩子今天在题目转化方面表现不错，能够尝试把原本复杂的描述转成更清晰的数学关系或状态关系，比如从操作条件中提取出真正需要维护的量。这类能力对复赛非常重要。后续需要加强的是把转化后的思路完整落实到代码中，尤其注意排序、二分、集合维护等实现细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="92" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>数学规律敏感学生</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>孩子今天在需要观察数学规律的题目上有一定优势，能够从样例和操作过程中发现答案变化的规律，而不是盲目模拟每一步。这样的思考方式很适合处理复赛中的性质题。后续建议多练习把规律说明清楚，并用小数据验证结论，避免因为证明不完整或特殊情况遗漏而失分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>排序二分应用较好学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在统计类题目中表现较好，能意识到暴力枚举会超时，并尝试通过排序、二分或双指针来缩小查找范围。说明孩子已经具备一定的优化意识。后续建议继续加强边界处理，比如左右端点、是否重复计数、答案范围是否需要 long long 等细节，这些往往决定最终得分是否稳定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>树上问题理解较好学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天在树上问题中的理解比较好，能顺着路径、距离和覆盖过程去分析，而不是只把题目当成普通模拟。对于这类题，能先找出关键路径和最终需要覆盖的范围非常重要。后续建议继续练习树上DFS、距离计算和最远点等基础能力，把思路转化成更熟练的代码实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>位运算题有亮点学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天在位运算相关题目中有一些亮点，能够尝试从二进制位的角度分析大小关系，说明孩子对这类抽象问题有一定敏感度。不过位运算题通常对推导和代码统计都要求较高，容易在下标、前缀统计或贡献计算上出错。后续建议多用小样例手推每一位的变化，再逐步写成代码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>特殊性质能看出但落码不稳学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天能看出部分题目的关键性质，说明理解并不差，但在把性质落到代码时还不够稳，容易因为变量含义、边界范围或多组数据处理出现问题。这类失分比较可惜。后续建议在写代码前先把核心变量写清楚：它表示什么、什么时候更新、答案从哪里来。这样能减少思路正确但代码失分的情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>暴力到正解过渡不足学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天能够先写出一些直观做法，说明读题后可以开始动手，但在从暴力做法继续优化时会有些困难。Day4 的重点正是通过特殊性质减少计算量，因此补题时不能只看最终代码，更要复盘“为什么这个性质能让题目变简单”。后续建议每道题都先写下暴力复杂度，再思考哪里可以被合并、排序或转化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>部分分与特殊数据意识较好学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天在部分题目中能够根据特殊数据或简单情况先拿到一部分分数，这是一个很好的考试习惯。复赛题常常有分层数据，先解决能解决的部分，再逐步优化，是很实际的策略。后续建议在补题时把部分分做法和正解联系起来，理解正解是在部分分基础上多利用了哪些性质。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day4 主要进行CSP-S复赛真题选讲与算法测试：课程围绕“从特殊性质出发”展开，训练学生从题目条件、数据范围、特殊情况和关键性质中寻找突破口。课堂中结合典型真题讲解如何利用特殊性质简化问题、从部分分过渡到完整做法；下午完成补题和6道算法测试，晚上进行测试题讲解、补题与总结。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>性质题适应待加强学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天面对性质较强的综合题时适应还需要加强，容易停留在表面模拟，或者看到题面复杂就不知道从哪里下手。这个阶段建议先建立固定分析流程：看样例、看数据范围、找特殊情况、想暴力做法，再判断能不能优化。只要能把第一步分析做扎实，后续面对真题会更有方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试表现选择对应反馈，不需要发给家长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>学生画像</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>典型特征</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>反馈侧重点</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>特殊性质把握优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>能快速抓住题目关键性质，并将其转化为简洁做法。</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>关键转化能力较强学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>能把题目条件转成数学式、可达状态或区间统计问题。</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>数学规律敏感学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>对总和变化、奇偶/大小关系、最高位等规律比较敏感。</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>排序二分应用较好学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>能想到排序、二分、双指针等优化方式处理统计类问题。</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>树上问题理解较好学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>对树上距离、追赶、路径覆盖等题有思路。</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>位运算题有亮点学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>异或、二进制最高位等题目有想法，但实现复杂度较高。</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>特殊性质能看出但落码不稳学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>能发现部分性质，但代码实现和边界处理影响得分。</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>暴力到正解过渡不足学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>能写暴力或部分分，难以继续利用特殊性质优化。</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>部分分与特殊数据意识较好学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>能根据特殊性质、小数据或简化情况争取部分分。</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>性质题适应待加强学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>题目条件较复杂时，不太会主动寻找关键性质。</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A31:F37"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F2 C9:F20 D3:F8 D25:F27 C21:F24">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
+      <formula1>'名单'!$A:$A</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Day5 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -8464,524 +8464,677 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.375" customWidth="1"/>
-    <col min="6" max="11" width="13" customWidth="1"/>
-    <col min="15" max="15" width="27.75" customWidth="1"/>
-    <col min="16" max="16" width="31.5" customWidth="1"/>
-    <col min="17" max="17" width="52.25" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:17">
-      <c r="A1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="K1" s="55" t="s">
-        <v>458</v>
-      </c>
-      <c r="L1" s="55" t="s">
-        <v>459</v>
-      </c>
-      <c r="M1" s="55" t="s">
-        <v>460</v>
-      </c>
-      <c r="N1" s="55" t="s">
-        <v>461</v>
-      </c>
-      <c r="O1" s="55" t="s">
-        <v>462</v>
-      </c>
-      <c r="P1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q1" s="55" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="2" ht="41.25" customHeight="1" spans="1:17">
-      <c r="A2" s="120" t="s">
-        <v>464</v>
-      </c>
-      <c r="B2" s="134" t="s">
-        <v>465</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="M2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="O2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="P2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q2" s="55" t="str">
-        <f>A2&amp;P8&amp;O8&amp;K8&amp;L8&amp;M8&amp;N8</f>
-        <v>今天的课程主要进行了对于博弈论的学习、以及一道 CSP-S 的压轴题贪吃蛇。</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:17">
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-    </row>
-    <row r="5" customHeight="1" spans="1:17">
-      <c r="B5" s="180" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="F5" s="193"/>
-      <c r="G5" s="193"/>
-      <c r="H5" s="194"/>
-      <c r="I5" s="194"/>
-      <c r="J5" s="194"/>
-      <c r="K5" s="182"/>
-      <c r="L5" s="182"/>
-      <c r="M5" s="182"/>
-      <c r="N5" s="182"/>
-      <c r="O5" s="182"/>
-      <c r="P5" s="182"/>
-    </row>
-    <row r="6" customHeight="1" spans="1:17">
-      <c r="B6" s="180" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D6" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="F6" s="193"/>
-      <c r="G6" s="194"/>
-      <c r="H6" s="194"/>
-      <c r="I6" s="194"/>
-      <c r="J6" s="194"/>
-      <c r="K6" s="182"/>
-      <c r="L6" s="182"/>
-      <c r="M6" s="182"/>
-      <c r="N6" s="182"/>
-      <c r="O6" s="182"/>
-      <c r="P6" s="182"/>
-    </row>
-    <row r="7" customHeight="1" spans="1:17">
-      <c r="B7" s="180" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="193"/>
-      <c r="G7" s="194"/>
-      <c r="H7" s="194"/>
-      <c r="I7" s="194"/>
-      <c r="J7" s="194"/>
-      <c r="K7" s="182"/>
-      <c r="L7" s="182"/>
-      <c r="M7" s="182"/>
-      <c r="N7" s="182"/>
-      <c r="O7" s="182"/>
-      <c r="P7" s="182"/>
-    </row>
-    <row r="8" customHeight="1" spans="1:17">
-      <c r="B8" s="180" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="193"/>
-      <c r="G8" s="180"/>
-      <c r="H8" s="194"/>
-      <c r="I8" s="194"/>
-      <c r="J8" s="194"/>
-      <c r="K8" s="182"/>
-      <c r="L8" s="182"/>
-      <c r="M8" s="182"/>
-      <c r="N8" s="182"/>
-      <c r="O8" s="182"/>
-      <c r="P8" s="182"/>
-    </row>
-    <row r="9" customHeight="1" spans="1:17">
-      <c r="B9" s="180" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="194"/>
-      <c r="G9" s="195"/>
-      <c r="H9" s="194"/>
-      <c r="I9" s="194"/>
-      <c r="J9" s="194"/>
-      <c r="K9" s="182"/>
-      <c r="L9" s="182"/>
-      <c r="M9" s="182"/>
-      <c r="N9" s="182"/>
-      <c r="O9" s="182"/>
-      <c r="P9" s="182"/>
-    </row>
-    <row r="10" customHeight="1" spans="1:17">
-      <c r="B10" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="194"/>
-      <c r="G10" s="193"/>
-      <c r="H10" s="194"/>
-      <c r="I10" s="194"/>
-      <c r="J10" s="194"/>
-      <c r="K10" s="182"/>
-      <c r="L10" s="182"/>
-      <c r="M10" s="182"/>
-      <c r="N10" s="182"/>
-      <c r="O10" s="182"/>
-      <c r="P10" s="182"/>
-    </row>
-    <row r="11" customHeight="1" spans="1:17">
-      <c r="B11" s="180" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="193"/>
-      <c r="G11" s="194"/>
-      <c r="H11" s="194"/>
-      <c r="I11" s="194"/>
-      <c r="J11" s="194"/>
-      <c r="K11" s="182"/>
-      <c r="L11" s="182"/>
-      <c r="M11" s="182"/>
-      <c r="N11" s="182"/>
-      <c r="O11" s="182"/>
-      <c r="P11" s="182"/>
-    </row>
-    <row r="12" customHeight="1" spans="1:17">
-      <c r="B12" s="180" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="194"/>
-      <c r="G12" s="194"/>
-      <c r="H12" s="194"/>
-      <c r="I12" s="194"/>
-      <c r="J12" s="194"/>
-      <c r="K12" s="182"/>
-      <c r="L12" s="182"/>
-      <c r="M12" s="182"/>
-      <c r="N12" s="182"/>
-      <c r="O12" s="182"/>
-      <c r="P12" s="182"/>
-    </row>
-    <row r="13" customHeight="1" spans="1:17">
-      <c r="B13" s="180" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="193"/>
-      <c r="G13" s="194"/>
-      <c r="H13" s="194"/>
-      <c r="I13" s="194"/>
-      <c r="J13" s="194"/>
-      <c r="K13" s="182"/>
-      <c r="L13" s="182"/>
-      <c r="M13" s="182"/>
-      <c r="N13" s="182"/>
-      <c r="O13" s="182"/>
-      <c r="P13" s="182"/>
-    </row>
-    <row r="14" customHeight="1" spans="1:17">
-      <c r="B14" s="180" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="194"/>
-      <c r="G14" s="193"/>
-      <c r="H14" s="194"/>
-      <c r="I14" s="194"/>
-      <c r="J14" s="194"/>
-      <c r="K14" s="182"/>
-      <c r="L14" s="182"/>
-      <c r="M14" s="182"/>
-      <c r="N14" s="182"/>
-      <c r="O14" s="182"/>
-      <c r="P14" s="182"/>
-    </row>
-    <row r="15" customHeight="1" spans="1:17">
-      <c r="B15" s="180" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="135" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="194"/>
-      <c r="G15" s="194"/>
-      <c r="H15" s="194"/>
-      <c r="I15" s="194"/>
-      <c r="J15" s="194"/>
-      <c r="K15" s="182"/>
-      <c r="L15" s="182"/>
-      <c r="M15" s="182"/>
-      <c r="N15" s="182"/>
-      <c r="O15" s="182"/>
-      <c r="P15" s="182"/>
-    </row>
-    <row r="16" customHeight="1" spans="1:17">
-      <c r="B16" s="180" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="135" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="194"/>
-      <c r="G16" s="194"/>
-      <c r="H16" s="194"/>
-      <c r="I16" s="194"/>
-      <c r="J16" s="194"/>
-      <c r="K16" s="182"/>
-      <c r="L16" s="182"/>
-      <c r="M16" s="182"/>
-      <c r="N16" s="182"/>
-      <c r="O16" s="182"/>
-      <c r="P16" s="182"/>
-    </row>
-    <row r="17" customHeight="1" spans="1:16">
-      <c r="B17" s="180" t="s">
-        <v>110</v>
-      </c>
-      <c r="C17" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D17" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E17" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="F17" s="194"/>
-      <c r="G17" s="194"/>
-      <c r="H17" s="194"/>
-      <c r="I17" s="194"/>
-      <c r="J17" s="194"/>
-      <c r="K17" s="182"/>
-      <c r="L17" s="182"/>
-      <c r="M17" s="182"/>
-      <c r="N17" s="182"/>
-      <c r="O17" s="182"/>
-      <c r="P17" s="182"/>
-    </row>
-    <row r="18" customHeight="1" spans="1:16">
-      <c r="B18" s="180" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="194"/>
-      <c r="G18" s="194"/>
-      <c r="H18" s="194"/>
-      <c r="I18" s="194"/>
-      <c r="J18" s="194"/>
-      <c r="K18" s="182"/>
-      <c r="L18" s="182"/>
-      <c r="M18" s="182"/>
-      <c r="N18" s="182"/>
-      <c r="O18" s="182"/>
-      <c r="P18" s="182"/>
-    </row>
-    <row r="19" customHeight="1" spans="1:16">
-      <c r="B19" s="180" t="s">
-        <v>100</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="194"/>
-      <c r="G19" s="194"/>
-      <c r="H19" s="194"/>
-      <c r="I19" s="194"/>
-      <c r="J19" s="194"/>
-      <c r="K19" s="182"/>
-      <c r="L19" s="182"/>
-      <c r="M19" s="182"/>
-      <c r="N19" s="182"/>
-      <c r="O19" s="182"/>
-      <c r="P19" s="182"/>
-    </row>
-    <row r="20" customHeight="1" spans="1:16">
-      <c r="B20" s="180" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="135" t="s">
-        <v>293</v>
-      </c>
-      <c r="F20" s="194"/>
-      <c r="G20" s="194"/>
-      <c r="H20" s="194"/>
-      <c r="I20" s="194"/>
-      <c r="J20" s="194"/>
-      <c r="K20" s="182"/>
-      <c r="L20" s="182"/>
-      <c r="M20" s="182"/>
-      <c r="N20" s="182"/>
-      <c r="O20" s="182"/>
-      <c r="P20" s="182"/>
-    </row>
-    <row r="32" customHeight="1" spans="1:16">
-      <c r="A32" s="56" t="s">
-        <v>172</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>课程内容</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>反思</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>反馈结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>综合模拟能力优秀学生</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>孩子今天在模拟测试中的综合表现非常突出，四道题都能找到有效切入点。T1这类维护题能抓住“总和与偏移”的核心，T2能进一步处理环形路线和窗口优化，T3、T4也能拿到较有含金量的分数，说明孩子面对综合题时分析比较全面。后续建议继续保持这种稳定性，同时在长题面和大数据限制下多留时间检查细节，争取把优势转化成更稳的高分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>模拟维护稳定学生</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>孩子今天在T1循环与重构上表现较稳，能看出题目真正需要维护的是数组总和和当前位置关系，而不是盲目模拟整个序列。这说明孩子对基础维护类问题理解比较扎实。相对来说，T2以后对优化和建模要求更高，得分空间还可以继续提升。后续建议保持基础题稳拿分的优势，再训练从简单维护过渡到复杂模型的能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="92" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>环形问题优化较好学生</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>孩子今天在T2跃迁回路这类环形路线题上有亮点，能够意识到逐个起点暴力模拟不够，需要把环形问题转成线性区间来处理。这类转化能力很重要，也说明孩子具备一定的优化意识。后续建议继续巩固滑动窗口、单调队列和下标变换，尤其注意编号、取模和长整型细节，避免思路正确但实现扣分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>资源调度DP有想法学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在T3选举这类资源调度题中有一定想法，能尝试理解“先获得协作者，再提高后续效率”的过程，也能意识到不同选择顺序会影响总时间。这道题建模难度较高，能拿到部分分已经说明孩子在认真分析。后续建议把复杂题拆成几个小问题：先处理没有协作者的情况，再考虑协作者数量和顺序，逐步建立完整模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>哈希匹配有亮点学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天在T4最大回文匹配和中有一些亮点，能够围绕“相同长度子数组”和“回文条件”展开思考，说明孩子对结构匹配问题有一定敏感度。这道题难点在于把回文条件转化成可以比较的形式，并用哈希快速判断。后续建议继续练习字符串和数组哈希类题目，重点关注等价转化、边界和哈希比较的稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>基础部分分策略较好学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天的部分分意识比较好，能先完成自己确定会做的部分，再尝试从小数据或特殊情况入手推进后面的题。模拟赛中这种策略很实用，因为不一定每题都能完整攻克。后续建议在补题时把自己的部分分做法和标准做法对照起来，看看每一步优化解决了什么问题，这样下次遇到类似题会更有方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>思路推进强于代码学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天在一些综合题中能提出方向，但代码实现阶段还不够稳，导致最终分数没有完全体现出思考水平。尤其是环形下标、DP数组、哈希比较这类实现细节，一旦处理不严谨就容易失分。后续建议写复杂题前先明确变量含义和更新顺序，再用小样例手动验证，减少“想到了但写不出来”的情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>长题面拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天面对长题面综合题时会有些吃力，容易被背景描述和条件数量影响，没能迅速抓住真正需要维护或优化的核心。T1相对直接，能完成一部分；但T2-T4需要先拆解模型，再选择算法。后续建议做题时先用自己的话写下“输入是什么、操作是什么、要求最大或最小什么”，再从小数据开始推。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>复杂优化题突破不足学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天基础题和直接模拟题表现还可以，但遇到需要进一步优化的题目时，容易停在暴力想法上。模拟赛后半部分题目通常需要把暴力中的重复计算找出来，再转成数据结构、DP或哈希。后续补题时建议不要只看代码，而要重点问自己：暴力哪里慢，正解是怎样减少重复计算的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day5 上午围绕S组复赛模拟训练展开，重点补充贪吃蛇与博弈相关内容，帮助学生理解Nim、Bash以及必胜态、必败态等基本概念。下午进行CSP-S模拟测试，题目覆盖模拟维护、环形路线优化、资源调度与动态规划、哈希匹配等综合能力；晚上进行测试讲解，复盘题目中的建模方法、优化思路和代码实现细节。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天在模拟测试中暴露出基础和综合读题两方面都需要加强。T1这类相对基础的维护题如果还不稳定，说明数组位置、循环移动、变量更新等基础实现需要先补牢；T2-T4则可以先从题解中的小数据做法开始理解。后续建议优先完成T1订正，再选择每道题的部分分做法练习，逐步建立信心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>学生画像</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>典型分数特征</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>反馈侧重点</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>综合模拟能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>总分约260分以上；T1约80-100，T2约60分以上，T3/T4至少各有30分以上或其中一题突破明显。</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>强调四题综合能力、长题面处理和高分稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>模拟维护稳定学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T1约80-100；T2-T4多为基础部分分，如每题0-30或只有一题略高。</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>肯定T1维护稳定，提醒从基础维护过渡到综合优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>环形问题优化较好学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T2约60-100；能超过暴力分，T1通常较稳，T3/T4不一定高。</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>突出环形展开、滑动窗口、单调队列和下标细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>资源调度DP有想法学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>T3约30-70；能拿到N较小、K=N或协作者相关部分分，T1/T2可能有基础分。</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>强调复杂建模意识，建议分层理解协作者、选票和时间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>哈希匹配有亮点学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T4约20-60；能拿n,m&lt;=300、B全相等或n较小等部分分，其他题分数不一定均衡。</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>突出回文条件转化、数组/字符串哈希和边界检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>基础部分分策略较好学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>总分约120-200；T1能拿40分以上，T2-T4能通过暴力、小数据或特殊性质累计部分分。</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>肯定考试策略，建议对比部分分做法和满分做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>思路推进强于代码学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>讲解或草稿能说出T2/T3/T4方向，但实际得分偏低；常见为T2/T3/T4各只有10-30分。</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>反馈重心放在变量含义、边界、小样例验证和落码稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>长题面拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T1有一定分数；T2-T4因题意拆解慢，多停留在样例或低分部分分。</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>建议训练先复述题意、圈限制、写暴力，再考虑优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>复杂优化题突破不足学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>T1约40-80；T2-T4基本能理解题意但主要停在暴力，优化部分得分较少。</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>强调从暴力瓶颈出发，寻找数据结构、DP或哈希优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>总分约0-100；T1低于40或不稳定，T2-T4多数为空题、样例级尝试或低分。</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>优先补T1和每题最基础部分分，先建立读题和实现信心。</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A32:M38"/>
-  </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:P2">
-      <formula1>"A,B,C"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
+      <formula1>'名单'!$A:$A</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C5:E16 C17:E20">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15909,7 +16062,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -16611,6 +16764,176 @@
       <c r="C41" t="inlineStr">
         <is>
           <t>题目条件较复杂时，不太会主动寻找关键性质。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>综合模拟能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>T1-T4整体得分较高；T1维护、T2环形优化、T3资源调度、T4哈希匹配均有稳定表现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>模拟维护稳定学生</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>T1基本满分或高分；T2-T4能拿部分分，但复杂优化题得分一般。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>环形问题优化较好学生</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>T2跃迁回路有较好分数；能理解环形展开、滑动窗口或单调队列思想。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>资源调度DP有想法学生</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>T3选举能拿部分分或中高分；能理解协作者、选票和时间分摊的关系。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>哈希匹配有亮点学生</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>T4最大回文匹配和有部分分或较好分；能想到回文、子数组匹配或哈希方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>基础部分分策略较好学生</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>T1能做出；T2-T4能通过暴力、小数据或特殊性质拿部分分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>思路推进强于代码学生</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>T2-T4有思路或草稿推导，但代码实现复杂，实际得分低于理解水平。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>长题面拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>T1可得分；T2-T4题面较长时抓不住核心条件，得分偏低。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>复杂优化题突破不足学生</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>T1较稳，T2-T4能理解题意但主要停留在暴力，优化分较少。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>T1也不稳定；T2-T4多数为空题、低分或只有样例级尝试。</t>
         </is>
       </c>
     </row>
@@ -26520,7 +26843,7 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试表现选择对应反馈，不需要发给家长。</t>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
         </is>
       </c>
     </row>
@@ -26532,7 +26855,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>典型特征</t>
+          <t>典型分数特征</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -26541,7 +26864,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>模板综合双优学生</t>
@@ -26549,16 +26872,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>模板题完成稳定，非模板综合题也能主动观察性质并推进优化。</t>
+          <t>T1-T7模板题基本满分；T8、T9能做出，T10有较高分，T11至少能拿部分分。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>强调综合能力强，同时提醒继续检查边界和细节。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
+          <t>反馈强调模板稳定、综合题分析能力强，提醒继续检查细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>基础扎实迁移待提升学生</t>
@@ -26566,16 +26889,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>模板题较稳，但遇到综合题时从基础做法迁移到优化做法会变慢。</t>
+          <t>T1-T7模板题大多满分；T8、T9有分，T10/T11低分或只有少量部分分。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>肯定基础，建议补题时复盘优化过程。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
+          <t>肯定基础，建议训练从模板迁移到综合题的优化思路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>模板稳定难题突破不足学生</t>
@@ -26583,16 +26906,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>基础题完成较好，但难题容易等待完整正解，部分分意识不足。</t>
+          <t>T1-T7模板题较稳；T8能拿分，T9以后明显下降，T10/T11多为空或低分。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>引导先拿可拿分，再冲击高分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
+          <t>强调先拿部分分，不要等完整正解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>思维突出模板待稳学生</t>
@@ -26600,16 +26923,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>非模板题有想法，能观察规律，但基础模板和代码稳定性影响得分。</t>
+          <t>T8-T10综合题有亮点或部分分较高；但T1-T7模板题中有1-2题因模板/实现失分。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>突出思维优势，提醒补稳模板与实现。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
+          <t>突出思维优势，提醒基础模板和代码实现要补稳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>思路正确细节失分学生</t>
@@ -26617,16 +26940,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>大方向判断正确，但边界、数组、初始化、输出等细节容易失分。</t>
+          <t>多题有提交和正确方向；T1-T7或T8/T9因边界、数组、初始化等细节丢较多分。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>强调检查习惯和代码稳定性。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
+          <t>反馈重点放在检查习惯、代码稳定性和赛后订正。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>观察题表现较好学生</t>
@@ -26634,16 +26957,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>规律观察类题目表现不错，能从样例和条件中找到突破口。</t>
+          <t>T8《一和二》、T9《快来数一数》得分较好；T10坐标统计和T11树上性质题得分一般。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>鼓励继续归纳规律，同时补复杂实现。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
+          <t>肯定观察规律能力，建议补复杂统计和树上题实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>部分分意识较好学生</t>
@@ -26651,16 +26974,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>不会完整做法时能尝试简单情况或特殊数据，愿意争取部分分。</t>
+          <t>T1-T7能拿一部分；T8-T11即使不会正解，也能通过暴力/特殊性质拿部分分。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>肯定考试策略，建议对比部分分与满分做法。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
+          <t>强调部分分策略好，建议对比部分分与满分做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>模板掌握不均学生</t>
@@ -26668,7 +26991,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>部分模板能完成，但树上、图论、DP等模块存在断点。</t>
+          <t>T1-T7模板题得分波动明显，例如并查集/树状数组会，LCA/最短路/DP模板失分。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -26677,7 +27000,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="36" customHeight="1">
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>综合题畏难学生</t>
@@ -26685,16 +27008,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>基础题能做一部分，题面较长或条件较多时容易停顿。</t>
+          <t>T1-T7基础题有一定得分；T8-T11大多空题、低分或只过样例。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>引导拆题、复述题意、先写简单做法。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="36" customHeight="1">
+          <t>反馈强调拆题和先写简单做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>基础待夯实学生</t>
@@ -26702,12 +27025,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>基础模板和代码实现都不够稳定，综合题独立推进困难。</t>
+          <t>T1-T7模板题整体得分偏低；T8-T11基本无有效得分。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>建议优先订正基础题和默写常见模板。</t>
+          <t>建议优先订正基础模板题，先建立代码信心。</t>
         </is>
       </c>
     </row>
@@ -28325,7 +28648,7 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试表现选择对应反馈，不需要发给家长。</t>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
         </is>
       </c>
     </row>
@@ -28337,7 +28660,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>典型特征</t>
+          <t>典型分数特征</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -28346,7 +28669,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>DP综合掌握优秀学生</t>
@@ -28354,16 +28677,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>基础模板和DP综合题都表现稳定，状态设计与转移推导较清晰。</t>
+          <t>T1-T6基础模板/工具题稳定；T7-T11 DP综合题中至少3题较高分。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>强调DP理解到位，提醒复杂题中检查细节。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
+          <t>强调DP状态设计和综合建模能力强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>模板扎实DP迁移待提升学生</t>
@@ -28371,16 +28694,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>模板题较稳，但从普通题迁移到综合DP建模时不够顺。</t>
+          <t>T1-T6基础题较稳；T7括号、T8货币等基础DP有分，T9-T11综合DP低分。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>建议复盘状态含义、转移来源和优化原因。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
+          <t>建议复盘状态含义和转移来源。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>状态设计清晰转移待稳学生</t>
@@ -28388,16 +28711,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>能找到状态方向，但转移细节、初始化和边界还需打磨。</t>
+          <t>T7-T10能写出状态方向并拿部分分；但初始化、边界或转移顺序导致未满分。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>突出理解能力，提醒把思路写稳。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
+          <t>突出理解能力，提醒把转移细节写稳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>DP思维较强代码细节失分学生</t>
@@ -28405,16 +28728,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>能分析子问题和状态关系，但循环、取模、数组等实现细节失分。</t>
+          <t>T7-T11有多题思路接近，但因数组范围、取模、循环顺序等实现问题丢分。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>强调调试和小样例手推。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
+          <t>强调小样例手推和代码检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>背包计数类题目表现较好学生</t>
@@ -28422,16 +28745,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>对选择/不选择、方案数累加等模型比较敏感。</t>
+          <t>T7括号计数、T8货币系统得分较好；T9 Emiya、T11状态压缩类得分一般。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>建议从优势模型过渡到多维和综合DP。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
+          <t>建议从优势模型过渡到更复杂计数DP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>路径DP理解较好学生</t>
@@ -28439,16 +28762,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>对路径规划、同步转移等过程型DP接受较好。</t>
+          <t>T10传纸条得分较好，路径/同步转移理解较顺；T7/T9/T11抽象计数题得分偏低。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>建议继续巩固路径DP，再过渡到抽象计数题。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
+          <t>建议以路径DP为基础，逐步练抽象建模。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>状态压缩有亮点学生</t>
@@ -28456,16 +28779,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>能意识到用状态记录选择情况，但状态编号和转移实现复杂。</t>
+          <t>T11 Bill的挑战有部分分或思路；但T7-T10基础DP可能不够稳定。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>建议拆步骤写清状态、转移和边界。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
+          <t>强调思维亮点，提醒先补稳常规DP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>工具模板不稳影响DP学生</t>
@@ -28473,16 +28796,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DP思路能跟上部分内容，但基础工具和代码框架影响发挥。</t>
+          <t>T1-T6中exgcd、单调队列、MST等前置模板有失分，影响后续DP题时间。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>建议先补稳数组、循环、常见模板。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="36" customHeight="1">
+          <t>建议先补基础工具，减少考试消耗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>会做基础DP难题突破不足学生</t>
@@ -28490,16 +28813,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>基础DP能完成，难题容易停在第一层思路，优化不足。</t>
+          <t>T3 LIS、T5 LCS、T6状压入门能得分；T7-T11综合题多为部分分或低分。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>引导从暴力状态逐步优化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="36" customHeight="1">
+          <t>建议从暴力状态逐步优化，不要停在基础模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>DP基础待夯实学生</t>
@@ -28507,7 +28830,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>状态、转移、初始值理解还不稳定，代码推进慢。</t>
+          <t>T3/T5等基础DP模板仍不稳定；T7-T11基本低分。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -29771,7 +30094,7 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试表现选择对应反馈，不需要发给家长。</t>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
         </is>
       </c>
     </row>
@@ -29783,7 +30106,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>典型特征</t>
+          <t>典型分数特征</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -29792,7 +30115,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>暴力优化思路优秀学生</t>
@@ -29800,16 +30123,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>能先写出基础思路，再主动减少重复计算、寻找优化方向。</t>
+          <t>T1-T4基本能做出或较高分；T5/T6也能从暴力推进到部分优化。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>强调复赛思维成熟，提醒稳定落码。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
+          <t>强调从暴力到优化的复赛思维。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>性质观察敏锐学生</t>
@@ -29817,16 +30140,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>能抓住奇偶性、数据范围、特殊条件等关键性质。</t>
+          <t>T1奇偶性、T2判别式、T3可行区间等性质题得分较好。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>建议把观察到的规律写成完整证明和代码。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
+          <t>建议把观察到的性质写成稳定代码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>数学判定表现较好学生</t>
@@ -29834,16 +30157,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>数学条件转化能力较好，能把题目变成可判断的问题。</t>
+          <t>T2最佳拍照地点得分较高，T1/T3也较稳；T5/T6复杂题得分一般。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>提醒注意数据类型、查找位置和边界情况。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
+          <t>提醒数据类型、二分位置和边界判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>区间维护稳定学生</t>
@@ -29851,16 +30174,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>过程变化类题目较稳，能维护当前可行范围。</t>
+          <t>T3温度得分较高；能维护可行范围，但T4-T6综合策略题得分一般。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>建议迁移到更多状态维护题。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
+          <t>建议迁移区间维护思路到更多题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>策略题理解较好学生</t>
@@ -29868,16 +30191,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>游戏、胜负、选择策略类题有思路，但证明和实现需加强。</t>
+          <t>T4射箭比赛有较好得分或能判断偶数出现性质；T5/T6仍偏难。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>引导先说清策略结论，再写代码。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
+          <t>引导先证明策略结论，再写代码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>构造字符串有想法学生</t>
@@ -29885,16 +30208,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>构造和模拟变化题有想法，能从目标形态反推。</t>
+          <t>T6修复二进制串有部分分或特殊情况分；其他中档题得分不一定稳定。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>提醒多用小样例检查所有情况。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
+          <t>提醒用小样例覆盖所有构造情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>暴力能写优化不足学生</t>
@@ -29902,16 +30225,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>能写基础做法，但数据变大时不知如何优化。</t>
+          <t>T1-T3能写暴力或基础做法；T4-T6因复杂度或性质不足低分。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>建议复盘暴力超时点和可利用性质。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
+          <t>建议复盘暴力为什么超时，寻找优化点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>部分分策略较好学生</t>
@@ -29919,16 +30242,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>能从简单情况或特殊数据入手争取分数。</t>
+          <t>每题都有尝试，T1-T6多题能拿特殊性质/暴力部分分，但满分题不多。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>建议对比部分分做法与标准做法。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="36" customHeight="1">
+          <t>肯定考试策略，建议对比部分分和正解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>读题拆解待提升学生</t>
@@ -29936,16 +30259,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>题面较长时容易抓不住核心条件，动手过早。</t>
+          <t>题面较长的T4-T6得分低；T1-T3也常因题意理解不完整失分。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>建议先复述题意、圈关键限制再写代码。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="36" customHeight="1">
+          <t>建议先复述题意、圈关键限制再写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>真实真题适应待加强学生</t>
@@ -29953,12 +30276,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>面对真题综合性压力较大，拆解和推进不稳定。</t>
+          <t>T1-T6整体低分，主要停留在样例理解或少量暴力。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>建议优先订正讲过题，建立固定做题流程。</t>
+          <t>建议订正课堂讲过题，建立固定做题流程。</t>
         </is>
       </c>
     </row>
@@ -31511,7 +31834,7 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试表现选择对应反馈，不需要发给家长。</t>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
         </is>
       </c>
     </row>
@@ -31523,7 +31846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>典型特征</t>
+          <t>典型分数特征</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -31532,7 +31855,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>特殊性质把握优秀学生</t>
@@ -31540,16 +31863,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>能快速抓住题目关键性质，并将其转化为简洁做法。</t>
+          <t>T1-T4能较高分或满分；T5/T6至少能利用特殊性质拿部分分。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
+          <t>强调抓关键性质能力强，提醒稳定实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>关键转化能力较强学生</t>
@@ -31557,16 +31880,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>能把题目条件转成数学式、可达状态或区间统计问题。</t>
+          <t>T1总和规律、T2可达长度、T3数对统计中至少两题较高分。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
+          <t>反馈重点放在条件转化和代码落地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>数学规律敏感学生</t>
@@ -31574,16 +31897,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>对总和变化、奇偶/大小关系、最高位等规律比较敏感。</t>
+          <t>T1第三条边、T6异或最高位等规律题有得分亮点。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
+          <t>提醒验证特殊情况和证明完整性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>排序二分应用较好学生</t>
@@ -31591,16 +31914,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>能想到排序、二分、双指针等优化方式处理统计类问题。</t>
+          <t>T3对数得分较高，能用排序二分/双指针；其他性质题表现一般。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
+          <t>建议扩展到更多统计优化题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>树上问题理解较好学生</t>
@@ -31608,16 +31931,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>对树上距离、追赶、路径覆盖等题有思路。</t>
+          <t>T5涂树有较好得分或能写出路径/距离相关部分；T6位运算偏弱。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
+          <t>建议继续练树上距离、DFS和路径覆盖。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>位运算题有亮点学生</t>
@@ -31625,16 +31948,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>异或、二进制最高位等题目有想法，但实现复杂度较高。</t>
+          <t>T6异或题有部分分或较高分；T1-T4基础性质题不一定全稳。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
+          <t>强调二进制分析能力，提醒统计实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>特殊性质能看出但落码不稳学生</t>
@@ -31642,16 +31965,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>能发现部分性质，但代码实现和边界处理影响得分。</t>
+          <t>T1-T4有正确方向，但因long long、边界、set/二分使用等细节失分。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
+          <t>重点反馈思路不错但实现需稳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>暴力到正解过渡不足学生</t>
@@ -31659,16 +31982,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>能写暴力或部分分，难以继续利用特殊性质优化。</t>
+          <t>T1/T3能写暴力或基础做法；T2/T4/T5/T6优化不足，得分偏低。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="36" customHeight="1">
+          <t>建议复盘从暴力到正解的关键转化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>部分分与特殊数据意识较好学生</t>
@@ -31676,16 +31999,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>能根据特殊性质、小数据或简化情况争取部分分。</t>
+          <t>T1-T6多题能拿小数据/特殊性质分，但满分题较少。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="36" customHeight="1">
+          <t>肯定部分分意识，建议整理每题升级路线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>性质题适应待加强学生</t>
@@ -31693,12 +32016,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>题目条件较复杂时，不太会主动寻找关键性质。</t>
+          <t>T1-T6整体低分，主要问题是不知道从条件中找关键性质。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>按该特征选择反馈，重点突出当天题目中的表现与后续改进方向。</t>
+          <t>建议按“样例-特殊情况-暴力-优化”流程训练。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Day6 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -11393,700 +11393,677 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.875" customWidth="1"/>
-    <col min="14" max="14" width="54.5" customWidth="1"/>
-    <col min="16" max="16" width="36.5" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:16">
-      <c r="A1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="55" t="s">
-        <v>458</v>
-      </c>
-      <c r="G1" s="55" t="s">
-        <v>459</v>
-      </c>
-      <c r="H1" s="55" t="s">
-        <v>460</v>
-      </c>
-      <c r="I1" s="55" t="s">
-        <v>461</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>462</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="55" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="2" ht="68.25" customHeight="1" spans="1:16">
-      <c r="A2" s="120" t="s">
-        <v>555</v>
-      </c>
-      <c r="B2" s="134" t="s">
-        <v>465</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="H2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="J2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="55" t="str">
-        <f>A2&amp;N8&amp;J8&amp;F8&amp;G8&amp;H8&amp;I8</f>
-        <v>今天的课回顾了之前几天做过的题目，【xx】积极的参与补题，有问题能够积极的向老师提问，不过需要注意补题不光要补正解，也需要补一下部分分代码。震轩在本次测试中考的非常好。在第一道题中震轩获取了部分分，震轩能够发现题目的性质，通过贪心去实现代码，但是没有考虑到时间复杂度的问题导致超时，非常可惜。在第二道题中，震轩实现了暴力代码，但是由于实现过于复杂，导致部分分拿的没有很全，需要了解下拆环的方法。震轩在第三道题中获取了部分分，震轩能够考虑到一些最基本的情况</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:16">
-      <c r="A4" s="120"/>
-      <c r="F4" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>557</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" customHeight="1" spans="1:16">
-      <c r="F5" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" customHeight="1" spans="1:16">
-      <c r="F6" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="8" customHeight="1" spans="1:16">
-      <c r="F8" s="2" t="str">
-        <f>SUBSTITUTE(IF(F2="A",F4,IF(F2="B",F5,IF(F2="C",F6,""))),"【xx】",B2)</f>
-        <v>在第一道题中震轩获取了部分分，震轩能够发现题目的性质，通过贪心去实现代码，但是没有考虑到时间复杂度的问题导致超时，非常可惜。</v>
-      </c>
-      <c r="G8" s="2" t="str">
-        <f>SUBSTITUTE(IF(G2="A",G4,IF(G2="B",G5,IF(G2="C",G6,""))),"【xx】",B2)</f>
-        <v>在第二道题中，震轩实现了暴力代码，但是由于实现过于复杂，导致部分分拿的没有很全，需要了解下拆环的方法。</v>
-      </c>
-      <c r="H8" s="2" t="str">
-        <f>SUBSTITUTE(IF(H2="A",H4,IF(H2="B",H5,IF(H2="C",H6,""))),"【xx】",B2)</f>
-        <v>震轩在第三道题中获取了部分分，震轩能够考虑到一些最基本的情况</v>
-      </c>
-      <c r="I8" s="2" t="str">
-        <f>SUBSTITUTE(IF(I2="A",I4,IF(I2="B",I5,IF(I2="C",I6,""))),"【xx】",B2)</f>
-        <v/>
-      </c>
-      <c r="J8" s="2" t="str">
-        <f>SUBSTITUTE(IF(J2="A",J4,IF(J2="B",J5,IF(J2="C",J6,""))),"【xx】",B2)</f>
-        <v>震轩在本次测试中考的非常好。</v>
-      </c>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="11" ht="115.5" customHeight="1" spans="1:16">
-      <c r="A11" s="134"/>
-      <c r="B11" s="134" t="s">
-        <v>162</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="E11" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G11" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="H11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="I11" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="K11" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L11" s="135"/>
-      <c r="M11" s="131"/>
-      <c r="N11" s="132" t="s">
-        <v>571</v>
-      </c>
-      <c r="O11" s="131"/>
-      <c r="P11" s="118"/>
-    </row>
-    <row r="12" ht="90" customHeight="1" spans="1:16">
-      <c r="B12" s="134" t="s">
-        <v>125</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="H12" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="J12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="K12" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L12" s="135"/>
-      <c r="M12" s="131"/>
-      <c r="N12" s="132" t="s">
-        <v>572</v>
-      </c>
-      <c r="O12" s="131"/>
-      <c r="P12" s="118"/>
-    </row>
-    <row r="13" ht="102.75" customHeight="1" spans="1:16">
-      <c r="B13" s="134" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="H13" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="J13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="K13" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L13" s="135"/>
-      <c r="M13" s="131"/>
-      <c r="N13" s="132" t="s">
-        <v>573</v>
-      </c>
-      <c r="O13" s="131"/>
-      <c r="P13" s="118"/>
-    </row>
-    <row r="14" ht="102.75" customHeight="1" spans="1:16">
-      <c r="B14" s="134" t="s">
-        <v>574</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I14" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="J14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K14" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L14" s="135"/>
-      <c r="M14" s="131"/>
-      <c r="N14" s="132" t="s">
-        <v>575</v>
-      </c>
-      <c r="O14" s="131"/>
-      <c r="P14" s="118"/>
-    </row>
-    <row r="15" ht="90" customHeight="1" spans="1:16">
-      <c r="B15" s="134" t="s">
-        <v>576</v>
-      </c>
-      <c r="C15" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G15" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I15" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L15" s="135"/>
-      <c r="M15" s="131"/>
-      <c r="N15" s="132" t="s">
-        <v>577</v>
-      </c>
-      <c r="O15" s="131"/>
-      <c r="P15" s="118"/>
-    </row>
-    <row r="16" ht="102.75" customHeight="1" spans="1:16">
-      <c r="B16" s="134" t="s">
-        <v>148</v>
-      </c>
-      <c r="C16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="H16" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="I16" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K16" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L16" s="135"/>
-      <c r="M16" s="131"/>
-      <c r="N16" s="132" t="s">
-        <v>578</v>
-      </c>
-      <c r="O16" s="131"/>
-      <c r="P16" s="118"/>
-    </row>
-    <row r="17" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B17" s="134" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="H17" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I17" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="K17" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L17" s="135"/>
-      <c r="M17" s="131"/>
-      <c r="N17" s="132" t="s">
-        <v>579</v>
-      </c>
-      <c r="O17" s="131"/>
-      <c r="P17" s="118" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="18" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B18" s="134" t="s">
-        <v>135</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="G18" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="H18" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="I18" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K18" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L18" s="135"/>
-      <c r="M18" s="131"/>
-      <c r="N18" s="132" t="s">
-        <v>581</v>
-      </c>
-      <c r="O18" s="131"/>
-      <c r="P18" s="118"/>
-    </row>
-    <row r="19" ht="102.75" customHeight="1" spans="1:16">
-      <c r="B19" s="134" t="s">
-        <v>152</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I19" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K19" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L19" s="135"/>
-      <c r="M19" s="131"/>
-      <c r="N19" s="132" t="s">
-        <v>582</v>
-      </c>
-      <c r="O19" s="131"/>
-      <c r="P19" s="118"/>
-    </row>
-    <row r="20" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B20" s="134" t="s">
-        <v>157</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I20" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K20" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L20" s="135"/>
-      <c r="M20" s="131"/>
-      <c r="N20" s="132" t="s">
-        <v>583</v>
-      </c>
-      <c r="O20" s="131"/>
-      <c r="P20" s="118" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="21" ht="102.75" customHeight="1" spans="1:16">
-      <c r="B21" s="139" t="s">
-        <v>140</v>
-      </c>
-      <c r="C21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K21" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L21" s="135"/>
-      <c r="M21" s="131"/>
-      <c r="N21" s="132" t="s">
-        <v>585</v>
-      </c>
-      <c r="O21" s="131"/>
-      <c r="P21" s="118"/>
-    </row>
-    <row r="22" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B22" s="134" t="s">
-        <v>145</v>
-      </c>
-      <c r="C22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="E22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F22" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="G22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I22" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K22" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L22" s="135"/>
-      <c r="M22" s="131"/>
-      <c r="N22" s="132" t="s">
-        <v>586</v>
-      </c>
-      <c r="O22" s="131"/>
-      <c r="P22" s="118"/>
-    </row>
-    <row r="23" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B23" s="139" t="s">
-        <v>167</v>
-      </c>
-      <c r="C23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="D23" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="E23" s="107" t="s">
-        <v>201</v>
-      </c>
-      <c r="F23" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="G23" s="107" t="s">
-        <v>293</v>
-      </c>
-      <c r="H23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I23" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="J23" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="K23" s="60" t="s">
-        <v>570</v>
-      </c>
-      <c r="L23" s="135"/>
-      <c r="M23" s="131"/>
-      <c r="N23" s="132" t="s">
-        <v>587</v>
-      </c>
-      <c r="O23" s="131"/>
-      <c r="P23" s="118"/>
-    </row>
-    <row r="31" customHeight="1" spans="1:16">
-      <c r="A31" s="56" t="s">
-        <v>172</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>课程内容</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>反思</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>反馈结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>综合建模能力优秀学生</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>孩子今天在综合模拟测试中的整体表现比较突出，面对四道风格差异较大的题目都能找到有效切入点。T1能看出购买策略的关键，T2能处理环形顺序问题，T3、T4也能在分类讨论或树上问题中拿到有含金量的分数，说明孩子的综合分析能力和考试节奏都比较好。后续建议继续保持全面性，同时在复杂题上多留一点时间检查边界和实现细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>糖果贪心稳定学生</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>孩子今天在T1糖果游戏上表现较稳，能够抓住“当前能买什么、买哪一种更划算”的核心思路，而不是简单地一颗一颗模拟。能把题目里的价格和返还关系转成清晰的选择策略，说明孩子对贪心类问题有不错的理解。后续建议继续训练把直觉写成稳定代码，尤其注意排序、筛选和连续购买次数这类细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="92" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>环形顺序优化较好学生</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>孩子今天在T2勇者比太郎这类环形顺序题中有亮点，能够意识到不同起点会影响初始条件，并尝试把环形过程转成更容易处理的线性区间。这类题很考验建模和优化意识，能拿到较好分数说明孩子不是只停留在暴力枚举。后续建议继续巩固前缀和、区间最大值和滑动窗口思想，减少下标处理上的失误。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>分类讨论能力较强学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在T3古堡法阵这类分类讨论题中有一定优势，能够根据免费边数量、是否相交、建边代价大小等条件分情况分析。这样的题目不一定代码很长，但需要把情况想完整，能拿到分数说明孩子的条件拆解能力不错。后续建议继续训练把每一种情况列清楚，再用小样例验证，避免漏掉边界情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>树上DP有突破学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天在T4训猫这类树上综合题中有一些突破，能围绕猫的移动过程、树上连通关系和高度顺序展开思考。T4难度较高，涉及树上距离、连通块合并和动态规划，能拿到部分分已经说明孩子愿意挑战复杂模型。后续建议先从链和小树情况理解移动规律，再逐步过渡到完整的树上做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>部分分策略清晰学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天的部分分策略比较清晰，能够先处理自己确定能完成的情况，再尝试从小数据、特殊条件或简化模型入手拿分。模拟赛里这种策略很重要，因为综合题不一定每道都能完整解决。后续建议补题时把自己的部分分做法和标准做法放在一起比较，弄清楚每一步优化到底解决了什么问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>思路推进强于代码学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天在部分题目中能说出方向，但代码实现阶段还不够稳定，导致实际得分没有完全体现出思考水平。比如T2的环形下标、T3的分类边界、T4的树上距离与合并细节，都容易出现“想到了但写不稳”的情况。后续建议写复杂题前先明确变量含义和处理顺序，再用小样例手动走一遍，减少实现失分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>长题面建模待提升学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天面对长题面和背景信息较多的题目时会有些吃力，容易被故事描述影响，没能快速抓住真正要优化的量。T1相对容易切入，T2-T4则需要先把题意压缩成清晰模型，再选择对应方法。后续建议做题时先用自己的话写下“当前状态是什么、每步会改变什么、最终要求什么”，这样会更容易找到突破口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>综合优化突破不足学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天在基础题和直接模拟上有一定表现，但遇到需要进一步优化的题目时，容易停在暴力做法上。Day6的题目普遍需要从简单想法继续往前推，比如去掉无用选择、把环形转成区间、把情况分类完整。后续补题时建议不要只看最终代码，而要重点复盘：暴力为什么慢，正解是怎样减少重复计算或减少情况的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day6 上午进行S组复赛模拟训练（二）的补题与复盘，帮助学生整理前一天模拟赛中的问题和订正方法。下午进行综合模拟测试，题目覆盖贪心选择、环形顺序优化、分类讨论与树上连通块动态规划等内容；晚上进行测试讲解，重点复盘如何从暴力和特殊数据逐步推进到更完整的做法。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天在模拟测试中暴露出基础读题和代码实现两方面都需要加强。T1如果还不稳定，说明排序、贪心和变量更新需要先补牢；T2-T4可以先从题解里的小数据或特殊情况做法开始理解，不急着一步到位。后续建议优先完成T1订正，再选择每道题最基础的部分分做法练习，先建立做题信心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>学生画像</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>典型分数特征</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>反馈侧重点</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>综合建模能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>总分约260分以上；T1/T2较高，T3或T4至少一题有明显突破，四题都有有效得分。</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>强调综合建模、考试节奏和高分稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>糖果贪心稳定学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T1约70-100；能超过小数据暴力分，T2-T4多为部分分。</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>肯定贪心选择和连续购买处理，提醒代码细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>环形顺序优化较好学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T2约60-100；能用前缀和、区间最大值或滑动窗口思想，T1通常较稳。</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>突出环形转线性、起点枚举优化和下标稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>分类讨论能力较强学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>T3约50-100；能处理M=0/M=1，或两条免费边是否相交、Q大小等情况。</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>强调情况拆解完整性和边界验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>树上DP有突破学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T4约30-70；能拿链、小树、特殊结构或树上连通块相关部分分。</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>突出树上距离、连通块合并和高度顺序理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>部分分策略清晰学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>总分约120-200；T1能拿基础分，T2-T4能通过小数据、特殊性质或暴力累计部分分。</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>肯定考试策略，建议对比部分分与满分路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>思路推进强于代码学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>能讲出T2/T3/T4方向，但实际常因下标、分类、LCA/并查集实现得分偏低。</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>反馈重心放在变量定义、小样例验证和落码稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>长题面建模待提升学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T1有一定得分；T2-T4因题意拆解慢，多停留在样例级或低分部分分。</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>建议先压缩题意，再写暴力并寻找优化量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>综合优化突破不足学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>T1/T2有基础得分；T3/T4基本理解题意但主要停在暴力或分类不完整。</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>强调从暴力瓶颈出发，寻找贪心、区间、分类或树上优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>总分约0-100；T1低于50或不稳定，T2-T4多数为空题、样例级尝试或低分。</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>优先订正T1和每题基础部分分，建立读题与实现信心。</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A31:H37"/>
-  </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:E2 F2:J2">
-      <formula1>"A,B,C"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
+      <formula1>'名单'!$A:$A</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C11:E20 D21:E23">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16062,7 +16039,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -16934,6 +16911,110 @@
       <c r="C51" t="inlineStr">
         <is>
           <t>T1也不稳定；T2-T4多数为空题、低分或只有样例级尝试。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>综合建模能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B52"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>强调综合建模、考试节奏和高分稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>糖果贪心稳定学生</t>
+        </is>
+      </c>
+      <c r="B53"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>肯定贪心选择和连续购买处理，提醒代码细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>环形顺序优化较好学生</t>
+        </is>
+      </c>
+      <c r="B54"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>突出环形转线性、起点枚举优化和下标稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>分类讨论能力较强学生</t>
+        </is>
+      </c>
+      <c r="B55"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>强调情况拆解完整性和边界验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>树上DP有突破学生</t>
+        </is>
+      </c>
+      <c r="B56"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>突出树上距离、连通块合并和高度顺序理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>部分分策略清晰学生</t>
+        </is>
+      </c>
+      <c r="B57"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>肯定考试策略，建议对比部分分与满分路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>长题面建模待提升学生</t>
+        </is>
+      </c>
+      <c r="B58"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>建议先压缩题意，再写暴力并寻找优化量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>综合优化突破不足学生</t>
+        </is>
+      </c>
+      <c r="B59"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>强调从暴力瓶颈出发，寻找贪心、区间、分类或树上优化。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Day7 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -13977,757 +13977,677 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="35.125" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="21.375" customWidth="1"/>
-    <col min="7" max="7" width="23.625" customWidth="1"/>
-    <col min="8" max="8" width="19" customWidth="1"/>
-    <col min="9" max="10" width="21.125" customWidth="1"/>
-    <col min="14" max="14" width="54.875" customWidth="1"/>
-    <col min="15" max="15" width="20.875" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:16">
-      <c r="A1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="55" t="s">
-        <v>458</v>
-      </c>
-      <c r="G1" s="55" t="s">
-        <v>459</v>
-      </c>
-      <c r="H1" s="55" t="s">
-        <v>460</v>
-      </c>
-      <c r="I1" s="55" t="s">
-        <v>461</v>
-      </c>
-      <c r="J1" s="55" t="s">
-        <v>462</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="55" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="2" ht="68.25" customHeight="1" spans="1:16">
-      <c r="A2" s="120" t="s">
-        <v>640</v>
-      </c>
-      <c r="B2" s="134" t="s">
-        <v>157</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="H2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="55" t="str">
-        <f>A2&amp;N8&amp;J8&amp;F8&amp;G8&amp;H8&amp;I8</f>
-        <v>今天的课程讲解昨天的 cf 比赛，讲解了关于 gcd 和 lcm 的做题技巧，以及如何使用根号分治把问题拆解成大小两个问题，然后去处理。【xx】积极的参与听讲，并且在听完后能积极的参与补题。杨涵语在本次测试中考的非常好。杨涵语在第一道题中获取了满分，这是一道非常容易写错的题目，杨涵语能够观察到题目的关键性质，非常精细的实现模拟的代码。杨涵语在第二道题中获取了部分分，杨涵语有着不错的观察能力，观察到了性质，但是并不完全正确，需要多考虑下再实现。杨涵语在第三道题中获取较高的部分分，杨涵语对字符串较为熟悉，并且能够很好的对情况进行分类讨论，但是在实现的过程中遇到了困难。杨涵语在第四道题中较高的部分分，杨涵语有着不错的思维和代码实现能力，能完成多个内容的部分分。</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:16">
-      <c r="F4" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>642</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:16">
-      <c r="F5" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>647</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>648</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:16">
-      <c r="F6" s="2" t="s">
-        <v>649</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="8" customHeight="1" spans="1:16">
-      <c r="F8" s="2" t="str">
-        <f>SUBSTITUTE(IF(F2="A",F4,IF(F2="B",F5,IF(F2="C",F6,""))),"【xx】",B2)</f>
-        <v>杨涵语在第一道题中获取了满分，这是一道非常容易写错的题目，杨涵语能够观察到题目的关键性质，非常精细的实现模拟的代码。</v>
-      </c>
-      <c r="G8" s="2" t="str">
-        <f>SUBSTITUTE(IF(G2="A",G4,IF(G2="B",G5,IF(G2="C",G6,""))),"【xx】",B2)</f>
-        <v>杨涵语在第二道题中获取了部分分，杨涵语有着不错的观察能力，观察到了性质，但是并不完全正确，需要多考虑下再实现。</v>
-      </c>
-      <c r="H8" s="2" t="str">
-        <f>SUBSTITUTE(IF(H2="A",H4,IF(H2="B",H5,IF(H2="C",H6,""))),"【xx】",B2)</f>
-        <v>杨涵语在第三道题中获取较高的部分分，杨涵语对字符串较为熟悉，并且能够很好的对情况进行分类讨论，但是在实现的过程中遇到了困难。</v>
-      </c>
-      <c r="I8" s="2" t="str">
-        <f>SUBSTITUTE(IF(I2="A",I4,IF(I2="B",I5,IF(I2="C",I6,""))),"【xx】",B2)</f>
-        <v>杨涵语在第四道题中较高的部分分，杨涵语有着不错的思维和代码实现能力，能完成多个内容的部分分。</v>
-      </c>
-      <c r="J8" s="2" t="str">
-        <f>SUBSTITUTE(IF(J2="A",J4,IF(J2="B",J5,IF(J2="C",J6,""))),"【xx】",B2)</f>
-        <v>杨涵语在本次测试中考的非常好。</v>
-      </c>
-    </row>
-    <row r="9" customHeight="1" spans="1:16">
-      <c r="F9" s="2" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="10" customHeight="1" spans="1:16">
-      <c r="F10" s="2" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="11" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B11" s="134" t="s">
-        <v>125</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="E11" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G11" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J11" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="K11" s="136" t="s">
-        <v>653</v>
-      </c>
-      <c r="L11" s="136" t="s">
-        <v>654</v>
-      </c>
-      <c r="M11" s="136" t="s">
-        <v>655</v>
-      </c>
-      <c r="N11" s="132" t="s">
-        <v>656</v>
-      </c>
-      <c r="O11" s="131"/>
-      <c r="P11" s="118"/>
-    </row>
-    <row r="12" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B12" s="134" t="s">
-        <v>576</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H12" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J12" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="K12" s="137" t="s">
-        <v>657</v>
-      </c>
-      <c r="L12" s="137" t="s">
-        <v>658</v>
-      </c>
-      <c r="M12" s="136" t="s">
-        <v>659</v>
-      </c>
-      <c r="N12" s="132" t="s">
-        <v>660</v>
-      </c>
-      <c r="O12" s="131"/>
-      <c r="P12" s="118"/>
-    </row>
-    <row r="13" ht="128.25" customHeight="1" spans="1:16">
-      <c r="B13" s="134" t="s">
-        <v>162</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G13" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="H13" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I13" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J13" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="K13" s="137" t="s">
-        <v>661</v>
-      </c>
-      <c r="L13" s="137" t="s">
-        <v>662</v>
-      </c>
-      <c r="M13" s="136" t="s">
-        <v>525</v>
-      </c>
-      <c r="N13" s="132" t="s">
-        <v>663</v>
-      </c>
-      <c r="O13" s="131"/>
-      <c r="P13" s="118"/>
-    </row>
-    <row r="14" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B14" s="134" t="s">
-        <v>574</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="138" t="s">
-        <v>24</v>
-      </c>
-      <c r="G14" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I14" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J14" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="K14" s="136" t="s">
-        <v>664</v>
-      </c>
-      <c r="L14" s="136" t="s">
-        <v>665</v>
-      </c>
-      <c r="M14" s="136" t="s">
-        <v>666</v>
-      </c>
-      <c r="N14" s="132" t="s">
-        <v>667</v>
-      </c>
-      <c r="O14" s="131"/>
-      <c r="P14" s="118"/>
-    </row>
-    <row r="15" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B15" s="134" t="s">
-        <v>148</v>
-      </c>
-      <c r="C15" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J15" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" s="137" t="s">
-        <v>668</v>
-      </c>
-      <c r="L15" s="137" t="s">
-        <v>669</v>
-      </c>
-      <c r="M15" s="136" t="s">
-        <v>670</v>
-      </c>
-      <c r="N15" s="132" t="s">
-        <v>671</v>
-      </c>
-      <c r="O15" s="131"/>
-      <c r="P15" s="118"/>
-    </row>
-    <row r="16" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B16" s="139" t="s">
-        <v>140</v>
-      </c>
-      <c r="C16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="85" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I16" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="135" t="s">
-        <v>23</v>
-      </c>
-      <c r="K16" s="137" t="s">
-        <v>672</v>
-      </c>
-      <c r="L16" s="137" t="s">
-        <v>673</v>
-      </c>
-      <c r="M16" s="136" t="s">
-        <v>674</v>
-      </c>
-      <c r="N16" s="132" t="s">
-        <v>675</v>
-      </c>
-      <c r="O16" s="131"/>
-      <c r="P16" s="118"/>
-    </row>
-    <row r="17" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B17" s="134" t="s">
-        <v>145</v>
-      </c>
-      <c r="C17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="H17" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I17" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="J17" s="135" t="s">
-        <v>33</v>
-      </c>
-      <c r="K17" s="137" t="s">
-        <v>676</v>
-      </c>
-      <c r="L17" s="137" t="s">
-        <v>677</v>
-      </c>
-      <c r="M17" s="137" t="s">
-        <v>678</v>
-      </c>
-      <c r="N17" s="132" t="s">
-        <v>679</v>
-      </c>
-      <c r="O17" s="131"/>
-      <c r="P17" s="118" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="18" ht="128.25" customHeight="1" spans="1:16">
-      <c r="B18" s="139" t="s">
-        <v>167</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E18" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J18" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K18" s="136" t="s">
-        <v>680</v>
-      </c>
-      <c r="L18" s="136" t="s">
-        <v>681</v>
-      </c>
-      <c r="M18" s="136" t="s">
-        <v>682</v>
-      </c>
-      <c r="N18" s="132" t="s">
-        <v>683</v>
-      </c>
-      <c r="O18" s="131"/>
-      <c r="P18" s="118"/>
-    </row>
-    <row r="19" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B19" s="134" t="s">
-        <v>152</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J19" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K19" s="137" t="s">
-        <v>684</v>
-      </c>
-      <c r="L19" s="137" t="s">
-        <v>685</v>
-      </c>
-      <c r="M19" s="136" t="s">
-        <v>686</v>
-      </c>
-      <c r="N19" s="132" t="s">
-        <v>687</v>
-      </c>
-      <c r="O19" s="131"/>
-      <c r="P19" s="118"/>
-    </row>
-    <row r="20" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B20" s="134" t="s">
-        <v>157</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I20" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="J20" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K20" s="137" t="s">
-        <v>688</v>
-      </c>
-      <c r="L20" s="136" t="s">
-        <v>689</v>
-      </c>
-      <c r="M20" s="136" t="s">
-        <v>690</v>
-      </c>
-      <c r="N20" s="132" t="s">
-        <v>691</v>
-      </c>
-      <c r="O20" s="131"/>
-      <c r="P20" s="118" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="21" ht="315" customHeight="1" spans="1:16">
-      <c r="B21" s="134" t="s">
-        <v>135</v>
-      </c>
-      <c r="C21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="J21" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K21" s="137" t="s">
-        <v>692</v>
-      </c>
-      <c r="L21" s="137" t="s">
-        <v>693</v>
-      </c>
-      <c r="M21" s="136" t="s">
-        <v>694</v>
-      </c>
-      <c r="N21" s="132" t="s">
-        <v>695</v>
-      </c>
-      <c r="O21" s="131"/>
-      <c r="P21" s="118"/>
-    </row>
-    <row r="22" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B22" s="134" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="E22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I22" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="J22" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K22" s="137" t="s">
-        <v>696</v>
-      </c>
-      <c r="L22" s="136" t="s">
-        <v>697</v>
-      </c>
-      <c r="M22" s="136" t="s">
-        <v>698</v>
-      </c>
-      <c r="N22" s="132" t="s">
-        <v>699</v>
-      </c>
-      <c r="O22" s="131"/>
-      <c r="P22" s="118"/>
-    </row>
-    <row r="23" ht="115.5" customHeight="1" spans="1:16">
-      <c r="B23" s="134" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="J23" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="K23" s="137" t="s">
-        <v>700</v>
-      </c>
-      <c r="L23" s="136" t="s">
-        <v>701</v>
-      </c>
-      <c r="M23" s="136" t="s">
-        <v>702</v>
-      </c>
-      <c r="N23" s="132" t="s">
-        <v>703</v>
-      </c>
-      <c r="O23" s="131"/>
-      <c r="P23" s="118"/>
-    </row>
-    <row r="31" customHeight="1" spans="1:16">
-      <c r="A31" s="56" t="s">
-        <v>172</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>课程内容</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>反思</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>反馈结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>综合推理能力优秀学生</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>孩子今天在综合模拟测试中的表现比较全面，四道题都能找到有效切入点。T1能快速抓住数字末位性质，T2能从数据出现次数中还原规律，T3、T4也能在递归优化和计数问题中拿到有含金量的分数。整体来看，孩子对题目条件的提炼能力较强，后续建议继续保持这种全面性，并在复杂题上多留时间检查边界和特殊情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>末位性质掌握稳定学生</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>孩子今天在T1这类数字性质题上表现较稳，能够抓住“是否能变成4的倍数主要看最后两位”这一关键点，再去分析交换次数。能把看似复杂的操作压缩成一个小范围判断，说明孩子的性质观察能力不错。后续建议继续训练这类题的完整分类，尤其是0次、1次、2次操作以及无解情况，避免漏掉边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="92" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>频次还原能力较好学生</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>孩子今天在T2数据缺失这类还原题中有亮点，能够从一堆无序数据里观察出现次数的规律，而不是盲目枚举原序列。这类题很考验从结果反推原结构的能力，能拿到较好分数说明孩子的逻辑整理比较清楚。后续建议继续练习排序、分组和计数类题目，把“规律想到了”进一步转化成稳定实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>递归优化有想法学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在T3整数这类代价优化题中有一定想法，能围绕“减一、加大、除二”三种操作分析不同路径的优劣。题目数据范围很大，不能只靠直接模拟，能拿到部分分说明孩子已经开始从状态和转移角度思考。后续建议继续训练递归、记忆化和分类讨论，特别注意某个操作不可用时该如何处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>字符串计数有突破学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天在T4字符串计数题中有一些突破，能意识到直接数合法方案比较困难，需要从不能划分的特殊结构入手。这样的计数题对抽象能力要求较高，能拿到部分分已经说明孩子愿意挑战复杂模型。后续建议先把小长度样例和特殊情况想清楚，再逐步整理出完整的计数公式，避免一上来就被大范围数据吓住。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>特殊数据利用较好学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天的特殊数据意识比较好，能先处理自己确定能做的情况，例如T1的小范围判断、T2的小n或少量取值、T3的小数据或某些操作不可用、T4的固定字符串或小字符集。模拟赛中这种策略很实用，因为不一定每道题都能完整攻克。后续建议补题时把特殊情况和满分做法对照起来，理解每一步优化解决了什么问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>思路正确实现待稳学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天在部分题目中能提出正确方向，但代码实现阶段还不够稳定，导致最终分数没有完全体现出思考水平。比如T2的分组边界、T3的递归状态、T4的计数容斥，一旦细节处理不严谨就容易失分。后续建议写复杂题前先把状态含义和分支情况列清楚，再用小样例逐步验证，减少“想到了但写不稳”的情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>性质题迁移待提升学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天面对需要找规律和做转化的题目时还有些吃力，容易停留在样例层面，没有及时抽出题目真正考察的性质。T1相对容易切入，但T2-T4都需要进一步观察频次、操作代价或字符串结构。后续建议做题时先问自己：哪些信息真正影响答案，哪些操作可以被简化，先从小数据手推几组再写代码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>综合题畏难需引导学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天在基础部分有一定尝试，但遇到T3、T4这种综合度较高的题目时，容易产生畏难情绪，推进不够深入。其实这类题并不是一开始就要求完整正解，先写出暴力、小数据或特殊情况也能帮助建立思路。后续建议考试中先保证T1和自己能做的部分分，再选择一题深入推进，不要因为后两题题面难就完全放弃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day7 上午进行S组复赛模拟训练（三）的补题与复盘，帮助学生整理前面模拟赛中暴露出的读题、建模和实现问题。下午进行综合模拟测试，题目覆盖数字性质判断、数据频次还原、递归代价优化和字符串计数等内容；晚上进行测试讲解，重点复盘如何从性质观察、频次规律和补集计数中找到突破口。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天在模拟测试中暴露出基础读题和代码实现两方面都需要加强。T1如果还不稳定，说明数字性质、枚举分类和字符串处理需要先补牢；T2-T4可以先从题解中的小数据做法和特殊情况开始理解。后续建议优先完成T1订正，再选择每道题最基础的部分分做法练习，先把读题和实现信心建立起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>学生画像</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>典型分数特征</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>反馈侧重点</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>综合推理能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>总分约260分以上；T1/T2较高，T3或T4至少一题有明显突破，四题都有有效得分。</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>强调综合推理、性质提炼和复杂题稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>末位性质掌握稳定学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T1约80-100；能完整判断0/1/2次交换和无解情况，T2-T4多为部分分。</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>肯定数字性质观察，提醒分类完整和边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>频次还原能力较好学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T2约60-100；能通过排序分组、出现次数规律判断缺失值或Infinite。</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>突出频次还原、分组检查和反推能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>递归优化有想法学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>T3约30-70；能处理小数据、单一操作限制或部分递归/记忆化转移。</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>强调状态设计、操作可用性和大数据优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>字符串计数有突破学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T4约20-60；能处理m=1、无-1、小n，或能想到从坏串/特殊结构计数。</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>突出补集思路、特殊结构和计数边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>特殊数据利用较好学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>总分约120-200；T1较稳，T2-T4能通过小数据、特殊性质或简化情况累计部分分。</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>肯定部分分策略，建议对比特殊数据与满分做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>思路正确实现待稳学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>能讲出T2/T3/T4方向，但实际常因分组边界、递归状态、容斥细节导致得分偏低。</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>反馈重心放在状态定义、小样例验证和实现稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>性质题迁移待提升学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T1有一定分数；T2-T4因规律提炼慢，多停留在样例级或低分部分分。</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>建议从小数据手推，训练把样例规律转成通用性质。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>综合题畏难需引导学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>T1/T2有基础尝试；T3/T4基本理解题意但推进不足，空题或低分较多。</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>强调先拿可做部分分，再选择一题深入推进。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>模拟赛基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>总分约0-100；T1低于50或不稳定，T2-T4多数为空题、样例级尝试或低分。</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>优先订正T1和每题基础部分分，建立读题与实现信心。</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A31:H37"/>
-  </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:E2 F2:J2">
-      <formula1>"A,B,C"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
+      <formula1>'名单'!$A:$A</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F15 C23:E23 C11:E20 H11:I12 D21:E22">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16039,7 +15959,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -17015,6 +16935,123 @@
       <c r="C59" t="inlineStr">
         <is>
           <t>强调从暴力瓶颈出发，寻找贪心、区间、分类或树上优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>综合推理能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B60"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>强调综合推理、性质提炼和复杂题稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>末位性质掌握稳定学生</t>
+        </is>
+      </c>
+      <c r="B61"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>肯定数字性质观察，提醒分类完整和边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>频次还原能力较好学生</t>
+        </is>
+      </c>
+      <c r="B62"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>突出频次还原、分组检查和反推能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>递归优化有想法学生</t>
+        </is>
+      </c>
+      <c r="B63"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>强调状态设计、操作可用性和大数据优化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>字符串计数有突破学生</t>
+        </is>
+      </c>
+      <c r="B64"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>突出补集思路、特殊结构和计数边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>特殊数据利用较好学生</t>
+        </is>
+      </c>
+      <c r="B65"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>肯定部分分策略，建议对比特殊数据与满分做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>思路正确实现待稳学生</t>
+        </is>
+      </c>
+      <c r="B66"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>反馈重心放在状态定义、小样例验证和实现稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>性质题迁移待提升学生</t>
+        </is>
+      </c>
+      <c r="B67"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>建议从小数据手推，训练把样例规律转成通用性质。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>综合题畏难需引导学生</t>
+        </is>
+      </c>
+      <c r="B68"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>强调先拿可做部分分，再选择一题深入推进。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Day9 feedback profiles
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -15959,7 +15959,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -17052,6 +17052,136 @@
       <c r="C68" t="inlineStr">
         <is>
           <t>强调先拿可做部分分，再选择一题深入推进。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>综合冲刺能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B69"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>强调冲刺阶段综合能力、赛场取舍和高分稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>性质观察稳定学生</t>
+        </is>
+      </c>
+      <c r="B70"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>肯定性质观察和简单题稳拿分能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>最短路统计较好学生</t>
+        </is>
+      </c>
+      <c r="B71"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>突出图论建模、路径拆分和统计去重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>配对DP有想法学生</t>
+        </is>
+      </c>
+      <c r="B72"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>强调过程抽象、区间交叉关系和DP状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>网格计数有突破学生</t>
+        </is>
+      </c>
+      <c r="B73"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>突出结构转化、矩形统计和计数边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>部分分规划清晰学生</t>
+        </is>
+      </c>
+      <c r="B74"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>肯定考试策略，建议对比部分分与满分升级路线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>思路推进强于实现学生</t>
+        </is>
+      </c>
+      <c r="B75"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>反馈重心放在变量定义、统计范围和小样例验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>复杂题拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="B76"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>建议先拆模型、写暴力，再寻找优化工具。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>后半场突破不足学生</t>
+        </is>
+      </c>
+      <c r="B77"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>强调稳住前两题，再选择一题深入突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>冲刺阶段基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B78"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>优先订正T1和每题基础部分分，稳定可拿分。</t>
         </is>
       </c>
     </row>
@@ -21059,726 +21189,677 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="44.25" customWidth="1"/>
-    <col min="6" max="6" width="28.5" customWidth="1"/>
-    <col min="7" max="7" width="20.5" customWidth="1"/>
-    <col min="8" max="8" width="24.5" customWidth="1"/>
-    <col min="9" max="10" width="22.625" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:15">
-      <c r="A1" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="55" t="s">
-        <v>903</v>
-      </c>
-      <c r="F1" s="55" t="s">
-        <v>458</v>
-      </c>
-      <c r="G1" s="55" t="s">
-        <v>459</v>
-      </c>
-      <c r="H1" s="55" t="s">
-        <v>460</v>
-      </c>
-      <c r="I1" s="55" t="s">
-        <v>461</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>462</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="55" t="s">
-        <v>20</v>
-      </c>
-      <c r="O1" s="55" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="2" ht="68.25" customHeight="1" spans="1:15">
-      <c r="A2" s="120" t="s">
-        <v>904</v>
-      </c>
-      <c r="B2" s="134" t="s">
-        <v>905</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="55" t="s">
-        <v>202</v>
-      </c>
-      <c r="H2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" s="55" t="s">
-        <v>80</v>
-      </c>
-      <c r="O2" s="55" t="str">
-        <f>A8&amp;J8&amp;F8&amp;G8&amp;H8</f>
-        <v>今天课程主要讲解了昨天的 cf 比赛，先给大家讲解了做思维题的技巧，以及会从什么角度去思考题目，最后从分析 csp 的原题旅游巴士，在此基础上推导出 cf D题的做法。涵语能够积极的参与课堂，并在讲解后能把 B 题和 C题全部完成。涵语在本次测试中考的不错。在第一道题中涵语获取了部分分，涵语有着较强的代码实现能力，写出了 dfs 枚举的代码，但是没有观察到题目的关键性质，导致失分，需要多观察题目性质。在第二道题中涵语想到了是最短路算法，但是在实现模版的时候写错了，非常可惜，可以再把模版在练习下总体来说，涵语发挥不错，能很好的实施自己的比赛策略，在难度较低的模拟赛中，能够认真思考 T1 的正解并实现，对于较难的题目 T2,T3,T4,涵语也能够尽可能的获取部分分，在后续的练习中，涵语最需要做的是：提升自己做绿题的能力，争取在比赛中能够做出 T2 的正解，加油。</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:15">
-      <c r="F4" s="2" t="s">
-        <v>906</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>907</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>908</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>909</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:15">
-      <c r="F5" s="55" t="s">
-        <v>910</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>911</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>912</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>913</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:15">
-      <c r="F6" s="2" t="s">
-        <v>914</v>
-      </c>
-      <c r="G6" s="55" t="s">
-        <v>915</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="8" customHeight="1" spans="1:15">
-      <c r="A8" s="2" t="str">
-        <f>SUBSTITUTE(A2,"【xx】",B2)</f>
-        <v>今天课程主要讲解了昨天的 cf 比赛，先给大家讲解了做思维题的技巧，以及会从什么角度去思考题目，最后从分析 csp 的原题旅游巴士，在此基础上推导出 cf D题的做法。涵语能够积极的参与课堂，并在讲解后能把 B 题和 C题全部完成。</v>
-      </c>
-      <c r="F8" s="2" t="str">
-        <f>SUBSTITUTE(IF(F2="A",F4,IF(F2="B",F5,IF(F2="C",F6,""))),"【xx】",B2)</f>
-        <v>在第一道题中涵语获取了部分分，涵语有着较强的代码实现能力，写出了 dfs 枚举的代码，但是没有观察到题目的关键性质，导致失分，需要多观察题目性质。</v>
-      </c>
-      <c r="G8" s="2" t="str">
-        <f>SUBSTITUTE(IF(G2="A",G4,IF(G2="B",G5,IF(G2="C",G6,""))),"【xx】",B2)</f>
-        <v>在第二道题中涵语想到了是最短路算法，但是在实现模版的时候写错了，非常可惜，可以再把模版在练习下</v>
-      </c>
-      <c r="H8" s="2" t="str">
-        <f>SUBSTITUTE(IF(H2="A",H4,IF(H2="B",H5,IF(H2="C",H6,""))),"【xx】",B2)</f>
-        <v>总体来说，涵语发挥不错，能很好的实施自己的比赛策略，在难度较低的模拟赛中，能够认真思考 T1 的正解并实现，对于较难的题目 T2,T3,T4,涵语也能够尽可能的获取部分分，在后续的练习中，涵语最需要做的是：提升自己做绿题的能力，争取在比赛中能够做出 T2 的正解，加油。</v>
-      </c>
-      <c r="I8" s="2" t="str">
-        <f>SUBSTITUTE(IF(I2="A",I4,IF(I2="B",I5,IF(I2="C",I6,""))),"【xx】",B2)</f>
-        <v>涵语第四道题中较高的部分分，涵语能够熟练的使用 st 对代码进行优化。</v>
-      </c>
-      <c r="J8" s="2" t="str">
-        <f>SUBSTITUTE(IF(J2="A",J4,IF(J2="B",J5,IF(J2="C",J6,""))),"【xx】",B2)</f>
-        <v>涵语在本次测试中考的不错。</v>
-      </c>
-    </row>
-    <row r="10" customHeight="1" spans="1:15">
-      <c r="J10" s="55" t="s">
-        <v>916</v>
-      </c>
-    </row>
-    <row r="11" customHeight="1" spans="1:15">
-      <c r="B11" s="134" t="s">
-        <v>125</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="E11" s="107" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="H11" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="J11" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="K11" s="136" t="s">
-        <v>917</v>
-      </c>
-      <c r="L11" s="136" t="s">
-        <v>918</v>
-      </c>
-      <c r="M11" s="136" t="s">
-        <v>919</v>
-      </c>
-      <c r="N11" s="60" t="s">
-        <v>920</v>
-      </c>
-    </row>
-    <row r="12" ht="39" customHeight="1" spans="1:15">
-      <c r="B12" s="134" t="s">
-        <v>162</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G12" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="H12" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I12" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="K12" s="137" t="s">
-        <v>921</v>
-      </c>
-      <c r="L12" s="137" t="s">
-        <v>922</v>
-      </c>
-      <c r="M12" s="136" t="s">
-        <v>509</v>
-      </c>
-      <c r="N12" s="60" t="s">
-        <v>923</v>
-      </c>
-    </row>
-    <row r="13" ht="39" customHeight="1" spans="1:15">
-      <c r="B13" s="134" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="H13" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J13" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="K13" s="137" t="s">
-        <v>924</v>
-      </c>
-      <c r="L13" s="136" t="s">
-        <v>925</v>
-      </c>
-      <c r="M13" s="136" t="s">
-        <v>926</v>
-      </c>
-      <c r="N13" s="60" t="s">
-        <v>927</v>
-      </c>
-    </row>
-    <row r="14" ht="77.25" customHeight="1" spans="1:15">
-      <c r="B14" s="134" t="s">
-        <v>576</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="138" t="s">
-        <v>116</v>
-      </c>
-      <c r="G14" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="135" t="s">
-        <v>24</v>
-      </c>
-      <c r="J14" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K14" s="137" t="s">
-        <v>928</v>
-      </c>
-      <c r="L14" s="137" t="s">
-        <v>929</v>
-      </c>
-      <c r="M14" s="136" t="s">
-        <v>930</v>
-      </c>
-      <c r="N14" s="60" t="s">
-        <v>931</v>
-      </c>
-    </row>
-    <row r="15" ht="77.25" customHeight="1" spans="1:15">
-      <c r="B15" s="139" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="G15" s="60" t="s">
-        <v>201</v>
-      </c>
-      <c r="H15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="J15" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" s="137" t="s">
-        <v>932</v>
-      </c>
-      <c r="L15" s="137" t="s">
-        <v>933</v>
-      </c>
-      <c r="M15" s="136" t="s">
-        <v>934</v>
-      </c>
-      <c r="N15" s="60" t="s">
-        <v>935</v>
-      </c>
-    </row>
-    <row r="16" ht="39" customHeight="1" spans="1:15">
-      <c r="B16" s="134" t="s">
-        <v>148</v>
-      </c>
-      <c r="C16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="K16" s="137" t="s">
-        <v>936</v>
-      </c>
-      <c r="L16" s="136" t="s">
-        <v>937</v>
-      </c>
-      <c r="M16" s="136" t="s">
-        <v>938</v>
-      </c>
-      <c r="N16" s="60" t="s">
-        <v>939</v>
-      </c>
-    </row>
-    <row r="17" customHeight="1" spans="1:14">
-      <c r="B17" s="134" t="s">
-        <v>574</v>
-      </c>
-      <c r="C17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="H17" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="I17" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="K17" s="136" t="s">
-        <v>940</v>
-      </c>
-      <c r="L17" s="136" t="s">
-        <v>941</v>
-      </c>
-      <c r="M17" s="136" t="s">
-        <v>942</v>
-      </c>
-      <c r="N17" s="60" t="s">
-        <v>943</v>
-      </c>
-    </row>
-    <row r="18" ht="141" customHeight="1" spans="1:14">
-      <c r="B18" s="134" t="s">
-        <v>152</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J18" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K18" s="137" t="s">
-        <v>944</v>
-      </c>
-      <c r="L18" s="137" t="s">
-        <v>945</v>
-      </c>
-      <c r="M18" s="136" t="s">
-        <v>946</v>
-      </c>
-      <c r="N18" s="60" t="s">
-        <v>947</v>
-      </c>
-    </row>
-    <row r="19" customHeight="1" spans="1:14">
-      <c r="B19" s="134" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I19" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J19" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K19" s="136" t="s">
-        <v>948</v>
-      </c>
-      <c r="L19" s="136" t="s">
-        <v>949</v>
-      </c>
-      <c r="M19" s="136" t="s">
-        <v>950</v>
-      </c>
-      <c r="N19" s="60" t="s">
-        <v>951</v>
-      </c>
-    </row>
-    <row r="20" customHeight="1" spans="1:14">
-      <c r="B20" s="139" t="s">
-        <v>167</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="107" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="G20" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I20" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J20" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K20" s="136" t="s">
-        <v>952</v>
-      </c>
-      <c r="L20" s="136" t="s">
-        <v>953</v>
-      </c>
-      <c r="M20" s="136" t="s">
-        <v>954</v>
-      </c>
-      <c r="N20" s="60" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="21" ht="39" customHeight="1" spans="1:14">
-      <c r="B21" s="134" t="s">
-        <v>135</v>
-      </c>
-      <c r="C21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J21" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K21" s="137" t="s">
-        <v>956</v>
-      </c>
-      <c r="L21" s="137" t="s">
-        <v>957</v>
-      </c>
-      <c r="M21" s="137" t="s">
-        <v>958</v>
-      </c>
-      <c r="N21" s="60" t="s">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="22" ht="128.25" customHeight="1" spans="1:14">
-      <c r="B22" s="134" t="s">
-        <v>145</v>
-      </c>
-      <c r="C22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="E22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="F22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G22" s="107" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="I22" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J22" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K22" s="137" t="s">
-        <v>960</v>
-      </c>
-      <c r="L22" s="137" t="s">
-        <v>961</v>
-      </c>
-      <c r="M22" s="137" t="s">
-        <v>962</v>
-      </c>
-      <c r="N22" s="60" t="s">
-        <v>963</v>
-      </c>
-    </row>
-    <row r="23" ht="26.25" customHeight="1" spans="1:14">
-      <c r="B23" s="134" t="s">
-        <v>157</v>
-      </c>
-      <c r="C23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="D23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="E23" s="107" t="s">
-        <v>201</v>
-      </c>
-      <c r="F23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="G23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="H23" s="60" t="s">
-        <v>293</v>
-      </c>
-      <c r="I23" s="135" t="s">
-        <v>80</v>
-      </c>
-      <c r="J23" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="K23" s="136" t="s">
-        <v>964</v>
-      </c>
-      <c r="L23" s="137" t="s">
-        <v>965</v>
-      </c>
-      <c r="M23" s="136" t="s">
-        <v>966</v>
-      </c>
-      <c r="N23" s="60" t="s">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="31" customHeight="1" spans="1:14">
-      <c r="A31" s="56" t="s">
-        <v>172</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>课程内容</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>总结</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>反思</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>反馈结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>综合冲刺能力优秀学生</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>孩子今天在最后阶段的综合模拟中表现比较突出，四道题都能找到有效切入点。T1能快速抓住集合最大值的性质，T2能理解新建道路对最短路的影响，T3、T4也能在动态规划和计数题中拿到有含金量的分数。整体来看，孩子已经具备较好的综合分析和赛场取舍能力，后续建议继续保持稳定节奏，把主要精力放在减少细节失误和提升难题表达完整度上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>性质观察稳定学生</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>孩子今天在T1众最大数上表现较稳，能够从子集最大值出现次数的规律中快速发现关键结论，而不是陷入枚举所有子集。这说明孩子对题目性质的提炼能力不错，也能在简单题中把分数拿稳。后续建议继续保持这种先观察、再证明、最后实现的习惯，遇到看似复杂的题目时先寻找真正影响答案的核心量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="92" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>最短路统计较好学生</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>孩子今天在T2建设工程这类图论统计题中有亮点，能意识到新建道路只会以两种方向影响从S到T的路径，并尝试用从起点和终点出发的距离来判断方案。这类题不仅考最短路，还考统计和去重，能拿到较好分数说明孩子建模能力不错。后续建议继续巩固Dijkstra、排序二分和边界判断，提升图论题的稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>配对DP有想法学生</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>孩子今天在T3两只手的24老师这类配对决策题中有一定想法，能尝试把拿牌过程转化成区间关系和得分选择。题目状态变化比较绕，能拿到部分分说明孩子愿意从过程模拟中抽象出更清晰的结构。后续建议先从小数据DP理解“哪些配对可以同时成立”，再逐步过渡到更高效的优化做法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="92" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>网格计数有突破学生</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>孩子今天在T4聚餐这类网格计数题中有一些突破，能够注意到座位不能相邻和数量超过一半会强烈限制矩形形态。这道题难点在于把条件转化成棋盘格结构，再统计合法矩形。能拿到部分分已经说明孩子对结构化计数有一定敏感度。后续建议继续练习从限制条件推出形态，再用前缀、单调栈等工具完成统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>部分分规划清晰学生</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>孩子今天的部分分规划比较清晰，能先保证T1这类可拿分题，再从T2-T4的小数据、特殊情况或暴力做法中争取分数。综合模拟中这种策略很重要，因为后面题目难度高，不一定每题都能完整解决。后续建议补题时把自己的部分分做法和标准做法对照起来，重点理解每一步优化为什么能减少枚举。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>思路推进强于实现学生</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>孩子今天在部分题目中能说出方向，但代码实现阶段还不够稳定，导致最终分数没有完全体现出思考水平。比如T2的距离数组和二分统计，T3的状态转移，T4的矩形边界与计数，都需要非常细致的实现。后续建议写复杂题前先把变量含义、统计范围和边界条件列清楚，再用小样例逐步验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>复杂题拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>孩子今天面对综合度较高的题目时，拆解速度还需要提升。T1相对容易切入，但T2-T4都需要先把题意压缩成更明确的模型，再选择图论、DP或计数工具。后续建议做题时先写出“题目真正要求统计什么、一次选择会改变什么、暴力为什么慢”，再从特殊数据开始推进。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>后半场突破不足学生</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>孩子今天在基础题和前半部分有一定尝试，但到T3、T4这类后半场难题时推进不足，容易停在题意理解或简单模拟上。其实模拟赛后半题也可以先从小范围、特殊结构或部分分入手，不一定一开始就追求完整正解。后续建议先稳住T1和T2可拿分部分，再选择一题深入思考，逐步提升难题耐心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="92" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day9 上午进行S组复赛模拟训练（四）的补题与复盘，帮助学生梳理前面模拟赛中的知识漏洞和答题策略。下午进行综合模拟测试，题目覆盖集合性质观察、最短路统计、区间配对动态规划和棋盘格矩形计数等内容；晚上进行测试讲解，重点复盘如何从关键性质、路径拆分、状态转移和结构计数中寻找突破。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>冲刺阶段基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C+</t>
+        </is>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>孩子今天在模拟测试中暴露出基础读题和代码实现两方面都需要继续加强。T1如果还不稳定，说明性质观察和简化题意需要先补牢；T2-T4可以先从题解中的小数据做法和特殊情况开始理解。后续建议优先完成T1订正，再选择每道题最基础的部分分做法练习，先把能拿到的分数稳定下来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>学生画像说明：以下内容用于帮助老师根据学生当天考试分数选择对应反馈，不需要发给家长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>学生画像</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>典型分数特征</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>反馈侧重点</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>综合冲刺能力优秀学生</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>总分约260分以上；T1/T2较高，T3或T4至少一题有明显突破，四题都有有效得分。</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>强调冲刺阶段综合能力、赛场取舍和高分稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>性质观察稳定学生</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T1约90-100；能发现答案就是原集合最大值，T2-T4多为部分分。</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>肯定性质观察和简单题稳拿分能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>最短路统计较好学生</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>T2约50-100；能跑S/T两次最短路，并用排序二分或类似方式统计可行点对。</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>突出图论建模、路径拆分和统计去重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>配对DP有想法学生</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>T3约30-70；能拿小N DP、区间配对关系或树状数组优化相关部分分。</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>强调过程抽象、区间交叉关系和DP状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>网格计数有突破学生</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>T4约20-60；能处理小网格、棋盘格特殊数据，或能推出合法矩形的棋盘格性质。</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>突出结构转化、矩形统计和计数边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>部分分规划清晰学生</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>总分约120-200；T1基本稳定，T2-T4能通过小数据、特殊性质或暴力累计部分分。</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>肯定考试策略，建议对比部分分与满分升级路线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>思路推进强于实现学生</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>能讲出T2/T3/T4方向，但实际常因二分统计、DP转移、矩形边界等实现细节得分偏低。</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>反馈重心放在变量定义、统计范围和小样例验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>复杂题拆解待提升学生</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T1有一定分数；T2-T4因题意压缩和模型建立慢，多停留在样例级或低分部分分。</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>建议先拆模型、写暴力，再寻找优化工具。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>后半场突破不足学生</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>T1/T2有基础尝试；T3/T4基本理解题意但推进不足，空题或低分较多。</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>强调稳住前两题，再选择一题深入突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>冲刺阶段基础待夯实学生</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>总分约0-100；T1低于60或不稳定，T2-T4多数为空题、样例级尝试或低分。</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>优先订正T1和每题基础部分分，稳定可拿分。</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A31:H37"/>
-  </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:D2 E2 F2:I2 J2">
-      <formula1>"A,B,C"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
+      <formula1>'名单'!$A:$A</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C23 F15:F20 H11:H17 I11:I12 I14:I16 C11:E20 D21:E23">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:F11">
       <formula1>"A+,A,A-,B+,B,B-,C+,C"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Link daily feedback sheets to templates
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -1,40 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <ns0:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <ns0:workbookPr/>
-  <ns0:bookViews>
-    <ns0:workbookView windowWidth="29400" windowHeight="12420" activeTab="2"/>
-  </ns0:bookViews>
-  <ns0:sheets>
-    <ns0:sheet name="座位表" sheetId="1" r:id="rId1"/>
-    <ns0:sheet name="名单" sheetId="2" r:id="rId2"/>
-    <ns0:sheet name="day1" sheetId="3" r:id="rId3"/>
-    <ns0:sheet name="Day1反馈表" sheetId="4" r:id="rId4"/>
-    <ns0:sheet name="day2" sheetId="5" r:id="rId5"/>
-    <ns0:sheet name="Day2反馈表" sheetId="6" r:id="rId6"/>
-    <ns0:sheet name="day3" sheetId="7" r:id="rId7"/>
-    <ns0:sheet name="Day3反馈表" sheetId="8" r:id="rId8"/>
-    <ns0:sheet name="day4" sheetId="9" r:id="rId9"/>
-    <ns0:sheet name="Day4反馈表" sheetId="10" r:id="rId10"/>
-    <ns0:sheet name="day5" sheetId="11" r:id="rId11"/>
-    <ns0:sheet name="陈一实" sheetId="13" r:id="rId13"/>
-    <ns0:sheet name="Day5反馈表" sheetId="14" r:id="rId14"/>
-    <ns0:sheet name="day6" sheetId="15" r:id="rId15"/>
-    <ns0:sheet name="Day6反馈表" sheetId="17" r:id="rId17"/>
-    <ns0:sheet name="day7" sheetId="18" r:id="rId18"/>
-    <ns0:sheet name="Day7反馈表" sheetId="20" r:id="rId20"/>
-    <ns0:sheet name="day8" sheetId="21" r:id="rId21"/>
-    <ns0:sheet name="Day8反馈表" sheetId="22" r:id="rId22"/>
-    <ns0:sheet name="Sheet26" sheetId="23" r:id="rId23"/>
-    <ns0:sheet name="day9" sheetId="24" r:id="rId24"/>
-    <ns0:sheet name="Day9反馈表" sheetId="26" r:id="rId26"/>
-    <ns0:sheet name="大反馈" sheetId="27" r:id="rId27"/>
-    <ns0:sheet name="集训营综合反馈卡" sheetId="28" r:id="rId28"/>
-  </ns0:sheets>
-  <ns0:calcPr calcId="191029"/>
-  <ns0:extLst>
-    <ns0:ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="29400" windowHeight="12420" activeTab="2"/>
+  </bookViews>
+  <sheets>
+    <sheet name="座位表" sheetId="1" ns1:id="rId1"/>
+    <sheet name="名单" sheetId="2" ns1:id="rId2"/>
+    <sheet name="day1" sheetId="3" ns1:id="rId3"/>
+    <sheet name="Day1反馈表" sheetId="4" ns1:id="rId4"/>
+    <sheet name="day2" sheetId="5" ns1:id="rId5"/>
+    <sheet name="Day2反馈表" sheetId="6" ns1:id="rId6"/>
+    <sheet name="day3" sheetId="7" ns1:id="rId7"/>
+    <sheet name="Day3反馈表" sheetId="8" ns1:id="rId8"/>
+    <sheet name="day4" sheetId="9" ns1:id="rId9"/>
+    <sheet name="Day4反馈表" sheetId="10" ns1:id="rId10"/>
+    <sheet name="day5" sheetId="11" ns1:id="rId11"/>
+    <sheet name="陈一实" sheetId="13" ns1:id="rId13"/>
+    <sheet name="Day5反馈表" sheetId="14" ns1:id="rId14"/>
+    <sheet name="day6" sheetId="15" ns1:id="rId15"/>
+    <sheet name="Day6反馈表" sheetId="17" ns1:id="rId17"/>
+    <sheet name="day7" sheetId="18" ns1:id="rId18"/>
+    <sheet name="Day7反馈表" sheetId="20" ns1:id="rId20"/>
+    <sheet name="day8" sheetId="21" ns1:id="rId21"/>
+    <sheet name="Day8反馈表" sheetId="22" ns1:id="rId22"/>
+    <sheet name="Sheet26" sheetId="23" ns1:id="rId23"/>
+    <sheet name="day9" sheetId="24" ns1:id="rId24"/>
+    <sheet name="Day9反馈表" sheetId="26" ns1:id="rId26"/>
+    <sheet name="大反馈" sheetId="27" ns1:id="rId27"/>
+    <sheet name="集训营综合反馈卡" sheetId="28" ns1:id="rId28"/>
+  </sheets>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <extLst>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <ns2:calcFeatures>
         <ns2:feature name="microsoft.com:RD"/>
         <ns2:feature name="microsoft.com:Single"/>
@@ -44,9 +44,9 @@
         <ns2:feature name="microsoft.com:LAMBDA_WF"/>
         <ns2:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </ns2:calcFeatures>
-    </ns0:ext>
-  </ns0:extLst>
-</ns0:workbook>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7338,7 +7338,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -7426,9 +7426,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="83"/>
-      <c r="D4" s="180" t="s">
-        <v>110</v>
-      </c>
+      <c r="D4" s="180"/>
       <c r="E4" s="196"/>
       <c r="F4" s="196"/>
       <c r="G4" s="196"/>
@@ -7525,24 +7523,20 @@
     </row>
     <row r="8" customHeight="1" spans="1:23">
       <c r="A8" s="73"/>
-      <c r="B8" s="198" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$G$100,2,FALSE)</f>
-        <v>A-</v>
+      <c r="B8" s="198">
+        <f>IFERROR(INDEX('day4'!$C:$C,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="C8" s="158"/>
-      <c r="D8" s="198" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$G$100,3,FALSE)</f>
-        <v>B+</v>
+      <c r="D8" s="198">
+        <f>IFERROR(INDEX('day4'!$E:$E,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="E8" s="158"/>
-      <c r="F8" s="198" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$G$100,4,FALSE)</f>
-        <v>B+</v>
+      <c r="F8" s="198">
+        <f>IFERROR(INDEX('day4'!$D:$D,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="G8" s="158"/>
-      <c r="H8" s="198" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$G$100,5,FALSE)</f>
-        <v>B</v>
+      <c r="H8" s="198">
+        <f>IFERROR(INDEX('day4'!$F:$F,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="158"/>
       <c r="J8" s="73"/>
@@ -7638,9 +7632,8 @@
         <v>181</v>
       </c>
       <c r="D12" s="81"/>
-      <c r="E12" s="118" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$G$100,6,FALSE)</f>
-        <v>异或哈希&amp;&amp;和哈希，两者通过随机数&amp;&amp;哈希来实现，前者可以运算维护物品出现次数是不是偶数次，后者维护每样物品是不是只出现几次；在做一些给予数学/其他公式时，实在不会可以把公式进行转换再去尝试。异或运算的前缀和异或。</v>
+      <c r="E12" s="118">
+        <f>IFERROR(INDEX('day4'!$G:$G,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="F12" s="120"/>
       <c r="G12" s="120"/>
@@ -7691,9 +7684,8 @@
         <v>182</v>
       </c>
       <c r="D14" s="81"/>
-      <c r="E14" s="118" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$Z$100,7,FALSE)</f>
-        <v>没有合理分配时间，在一道题上花费了太多时间；没有仔细审题导致数据范围开小。</v>
+      <c r="E14" s="118">
+        <f>IFERROR(INDEX('day4'!$H:$H,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="F14" s="118"/>
       <c r="G14" s="118"/>
@@ -7744,9 +7736,8 @@
         <v>184</v>
       </c>
       <c r="D16" s="81"/>
-      <c r="E16" s="118" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$Z$100,8,FALSE)</f>
-        <v>哈希使用方法，多联系dp题目来帮助更好的设计状态(转移方程)，考试时先从我擅长的题目做起，再去做难的题目，不要被卡太久，太久就换题：）；多做题来锻炼思维能力，可以在做题时更快想出方法</v>
+      <c r="E16" s="118">
+        <f>IFERROR(INDEX('day4'!$I:$I,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="F16" s="118"/>
       <c r="G16" s="118"/>
@@ -7795,9 +7786,8 @@
       <c r="B18" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="120" t="str">
-        <f>VLOOKUP(D4,'day4'!$B$7:$Z$100,9,FALSE)</f>
-        <v>今天选讲了提高组的真题，重点讲解了在面对冗长代码时如何通过模块化拆分、封装函数来保持逻辑清晰，并介绍了哈希这一高效优化技巧，帮助同学们在解决字符串及模拟问题时更加得心应手。智宸同学课堂积极度良好。能够参与互动，跟上课堂节奏，表现出学习热情。智宸在本次测试中表现不错，智宸能够解决基础的问题，在做其他题目时能够去获取部分分数，在面对中等题的时候，也能能够分析出问题的类型，但是孩子对于普及组二分 or 双指针的使用不是很熟练，实现代码的时候遇到了困难，需要加强基础算法的熟练度，继续加油。后续会通过不断练习来提高算法优化技巧的熟练度。</v>
+      <c r="C18" s="120">
+        <f>IFERROR(INDEX('day4'!$A:$A,MATCH($D$4,'day4'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day4'!$J:$J,MATCH($D$4,'day4'!$B:$B,0)),"")</f>
       </c>
       <c r="D18" s="120"/>
       <c r="E18" s="120"/>
@@ -8446,12 +8436,15 @@
     <mergeCell ref="B4:C5"/>
     <mergeCell ref="C18:I19"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:G9 S9:T9 F11:G11 G13:H13 G76:H76 G97:H97" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C73:J75 C94:J96">
       <formula1>"A,A+,A-,B,B+,B-,C,C+,S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4">
+      <formula1>'day4'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9561,7 +9554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9721,9 +9714,7 @@
         <v>553</v>
       </c>
       <c r="D5" s="76"/>
-      <c r="E5" s="180" t="s">
-        <v>54</v>
-      </c>
+      <c r="E5" s="180"/>
       <c r="F5" s="107"/>
       <c r="G5" s="107"/>
       <c r="H5" s="107"/>
@@ -9839,25 +9830,22 @@
     <row r="8" ht="21.75" customHeight="1" spans="1:35">
       <c r="A8" s="73"/>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,4,FALSE)</f>
-        <v>B+</v>
+      <c r="C8" s="87">
+        <f>IFERROR(INDEX('day5'!$D:$D,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="D8" s="80"/>
       <c r="E8" s="80"/>
       <c r="F8" s="80"/>
       <c r="G8" s="80"/>
-      <c r="H8" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,5,FALSE)</f>
-        <v>B+</v>
+      <c r="H8" s="87">
+        <f>IFERROR(INDEX('day5'!$E:$E,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="80"/>
       <c r="J8" s="80"/>
       <c r="K8" s="80"/>
       <c r="L8" s="80"/>
-      <c r="M8" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,6,FALSE)</f>
-        <v>B</v>
+      <c r="M8" s="87">
+        <f>IFERROR(INDEX('day5'!$F:$F,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="N8" s="80"/>
       <c r="O8" s="80"/>
@@ -10023,34 +10011,19 @@
     <row r="13" ht="27" customHeight="1" spans="1:35">
       <c r="A13" s="73"/>
       <c r="B13" s="78"/>
-      <c r="C13" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,11,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="C13" s="87"/>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
-      <c r="F13" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,12,FALSE)</f>
-        <v>B+</v>
-      </c>
+      <c r="F13" s="87"/>
       <c r="G13" s="80"/>
       <c r="H13" s="81"/>
-      <c r="I13" s="94" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,13,FALSE)</f>
-        <v>A</v>
-      </c>
+      <c r="I13" s="94"/>
       <c r="J13" s="80"/>
       <c r="K13" s="81"/>
-      <c r="L13" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,14,FALSE)</f>
-        <v>A-</v>
-      </c>
+      <c r="L13" s="87"/>
       <c r="M13" s="80"/>
       <c r="N13" s="81"/>
-      <c r="O13" s="87" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,15,FALSE)</f>
-        <v>B</v>
-      </c>
+      <c r="O13" s="87"/>
       <c r="P13" s="80"/>
       <c r="Q13" s="80"/>
       <c r="R13" s="80"/>
@@ -10173,9 +10146,8 @@
       <c r="C17" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="D17" s="109" t="str">
-        <f>VLOOKUP(E5,'day51'!$B$1:$AB$100,16,FALSE)</f>
-        <v>今天的课程主要进行了对于博弈论的学习、以及一道 CSP-S 的压轴题贪吃蛇。岳琳能够听懂的博弈的逻辑，以及能够理解贪吃蛇的做法。岳琳在本次CSP模拟中考的不错。岳琳在第一道题中，能够想到通过模拟去实现代码，但是因为没有测试样例导致爆 0 了。在剩下的题目中，岳琳能正确的读取题意并且有着较强的代码实现能力，获取了大部分的分数，非常不错，继续保持。后续可以增强对于 dp 以及哈希的练习，以及在实现代码后需要对代码进行测试，继续加油。</v>
+      <c r="D17" s="109">
+        <f>IFERROR(INDEX('day5'!$A:$A,MATCH($E$5,'day5'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day5'!$J:$J,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="E17" s="109"/>
       <c r="F17" s="109"/>
@@ -10289,9 +10261,12 @@
     <mergeCell ref="L13:N15"/>
     <mergeCell ref="O13:S15"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AE10:AF11" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5">
+      <formula1>'day5'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10980,7 +10955,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -11080,9 +11055,7 @@
         <v>553</v>
       </c>
       <c r="D5" s="76"/>
-      <c r="E5" s="186" t="s">
-        <v>79</v>
-      </c>
+      <c r="E5" s="186"/>
       <c r="F5" s="77"/>
       <c r="G5" s="77"/>
       <c r="H5" s="77"/>
@@ -11152,25 +11125,22 @@
     <row r="8" ht="30.75" customHeight="1" spans="1:20">
       <c r="A8" s="73"/>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,3,FALSE)</f>
-        <v>B+</v>
+      <c r="C8" s="87">
+        <f>IFERROR(INDEX('day6'!$D:$D,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="D8" s="80"/>
       <c r="E8" s="80"/>
       <c r="F8" s="80"/>
       <c r="G8" s="80"/>
-      <c r="H8" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,4,FALSE)</f>
-        <v>B+</v>
+      <c r="H8" s="87">
+        <f>IFERROR(INDEX('day6'!$E:$E,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="80"/>
       <c r="J8" s="80"/>
       <c r="K8" s="80"/>
       <c r="L8" s="80"/>
-      <c r="M8" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,5,FALSE)</f>
-        <v>B+</v>
+      <c r="M8" s="87">
+        <f>IFERROR(INDEX('day6'!$F:$F,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="N8" s="80"/>
       <c r="O8" s="80"/>
@@ -11261,34 +11231,19 @@
     <row r="13" ht="66.75" customHeight="1" spans="1:20">
       <c r="A13" s="73"/>
       <c r="B13" s="78"/>
-      <c r="C13" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,11,FALSE)</f>
-        <v>B+</v>
-      </c>
+      <c r="C13" s="87"/>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
-      <c r="F13" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,12,FALSE)</f>
-        <v>A-</v>
-      </c>
+      <c r="F13" s="87"/>
       <c r="G13" s="80"/>
       <c r="H13" s="81"/>
-      <c r="I13" s="94" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,13,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="I13" s="94"/>
       <c r="J13" s="80"/>
       <c r="K13" s="81"/>
-      <c r="L13" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,14,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="L13" s="87"/>
       <c r="M13" s="80"/>
       <c r="N13" s="81"/>
-      <c r="O13" s="87" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,15,FALSE)</f>
-        <v>B+</v>
-      </c>
+      <c r="O13" s="87"/>
       <c r="P13" s="80"/>
       <c r="Q13" s="80"/>
       <c r="R13" s="80"/>
@@ -11362,12 +11317,8 @@
       <c r="F17" s="101"/>
       <c r="G17" s="101"/>
       <c r="H17" s="101"/>
-      <c r="I17" s="102" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,18,FALSE)</f>
-        <v>今天学习了在OI赛制中使用对拍检测自己代码是否正确，并且补充了昨晚讲剩下的 “ 博弈论 ” 。
-在 “ 跃迁回路 ” 和 “ 勇者比太郎 ” 中学习了破环成链的思想。
-“ 古堡法阵 ” 中运用了分类讨论的思想并学习了通过看数据范围推测做法的技巧
-“ 训猫 ” 中学习了如何从链上特性推导出树上特性</v>
+      <c r="I17" s="102">
+        <f>IFERROR(INDEX('day6'!$G:$G,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="J17" s="80"/>
       <c r="K17" s="80"/>
@@ -11404,12 +11355,8 @@
       <c r="F19" s="101"/>
       <c r="G19" s="101"/>
       <c r="H19" s="101"/>
-      <c r="I19" s="102" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,19,FALSE)</f>
-        <v>在题目 “ 糖果游戏 ” 中不会优化代码的时间复杂度 ， 导致TLE错误；
-且没有推理出 “ 古堡法阵 ” 中的多种情况与公式导致错误答案
-未意识到 “ 跃迁回路 ” 和 “ 勇者比太郎 ” 是同类问题 ， 导致第二题只拿了部分分
-//未意识到 “ 训猫 ” 是个树上问题</v>
+      <c r="I19" s="102">
+        <f>IFERROR(INDEX('day6'!$H:$H,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="J19" s="80"/>
       <c r="K19" s="80"/>
@@ -11446,9 +11393,8 @@
       <c r="F21" s="107"/>
       <c r="G21" s="107"/>
       <c r="H21" s="108"/>
-      <c r="I21" s="102" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,20,FALSE)</f>
-        <v>多练习题目，活跃思维，做题时多联想，找到与其相似的的模板或者相似的题，更有利于完成题目，注意不要在一道题上耗费太多时间，不然会导致有些题目没时间做</v>
+      <c r="I21" s="102">
+        <f>IFERROR(INDEX('day6'!$I:$I,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="J21" s="80"/>
       <c r="K21" s="80"/>
@@ -11468,9 +11414,8 @@
       <c r="C22" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="D22" s="109" t="str">
-        <f>VLOOKUP(E5,'day61'!$B$1:$Z$99,16,FALSE)</f>
-        <v>今天课堂主要解析了昨日测试中的第3题与第4题，第3题帮助大家梳理了动态规划的思路与优化技巧，第4题则再次应用了哈希方法解决字符串相关问题。今日测试采用OI赛制，贴近CSP-S复赛的实际氛围，邓宇然在本次测试中的评级为B+。测试成绩分析：在第1题中，未能对金币使用与获取步骤进行数学上的运算优化。在第2题中，未能运用昨天所学的知识建立正确的模型。在第3题中，对分类讨论思想应用不充分。在第4题中，考虑了当数据较小时的得分方案，但对深度优先搜索的代码熟练度较低，代码出现了错误，导致严重失分。整体表现良好，掌握了大部分知识点，并能完成多数任务。但在分析题目时的深度和解题的完整性方面还有待加强。学习态度积极，后续应更加注重系统训练，多积累与归纳解题方法，从而提升稳定性和效率。</v>
+      <c r="D22" s="109">
+        <f>IFERROR(INDEX('day6'!$A:$A,MATCH($E$5,'day6'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day6'!$J:$J,MATCH($E$5,'day6'!$B:$B,0)),"")</f>
       </c>
       <c r="E22" s="109"/>
       <c r="F22" s="109"/>
@@ -11534,6 +11479,11 @@
       <c r="T24" s="110"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5">
+      <formula1>'day6'!$B:$B</formula1>
+    </dataValidation>
+  </dataValidations>
   <mergeCells count="34">
     <mergeCell ref="B4:S4"/>
     <mergeCell ref="C5:D5"/>
@@ -13493,7 +13443,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -13593,9 +13543,7 @@
         <v>553</v>
       </c>
       <c r="D5" s="76"/>
-      <c r="E5" s="180" t="s">
-        <v>110</v>
-      </c>
+      <c r="E5" s="180"/>
       <c r="F5" s="77"/>
       <c r="G5" s="77"/>
       <c r="H5" s="77"/>
@@ -13665,25 +13613,22 @@
     <row r="8" ht="30.75" customHeight="1" spans="1:20">
       <c r="A8" s="73"/>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,3,FALSE)</f>
-        <v>B</v>
+      <c r="C8" s="87">
+        <f>IFERROR(INDEX('day7'!$D:$D,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="D8" s="80"/>
       <c r="E8" s="80"/>
       <c r="F8" s="80"/>
       <c r="G8" s="80"/>
-      <c r="H8" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,4,FALSE)</f>
-        <v>B</v>
+      <c r="H8" s="87">
+        <f>IFERROR(INDEX('day7'!$E:$E,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="80"/>
       <c r="J8" s="80"/>
       <c r="K8" s="80"/>
       <c r="L8" s="80"/>
-      <c r="M8" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,5,FALSE)</f>
-        <v>B-</v>
+      <c r="M8" s="87">
+        <f>IFERROR(INDEX('day7'!$F:$F,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="N8" s="80"/>
       <c r="O8" s="80"/>
@@ -13774,34 +13719,19 @@
     <row r="13" ht="66.75" customHeight="1" spans="1:20">
       <c r="A13" s="73"/>
       <c r="B13" s="78"/>
-      <c r="C13" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,11,FALSE)</f>
-        <v>B+</v>
-      </c>
+      <c r="C13" s="87"/>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
-      <c r="F13" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,12,FALSE)</f>
-        <v>B+</v>
-      </c>
+      <c r="F13" s="87"/>
       <c r="G13" s="80"/>
       <c r="H13" s="81"/>
-      <c r="I13" s="94" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,13,FALSE)</f>
-        <v>B</v>
-      </c>
+      <c r="I13" s="94"/>
       <c r="J13" s="80"/>
       <c r="K13" s="81"/>
-      <c r="L13" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,14,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="L13" s="87"/>
       <c r="M13" s="80"/>
       <c r="N13" s="81"/>
-      <c r="O13" s="87" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,15,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="O13" s="87"/>
       <c r="P13" s="80"/>
       <c r="Q13" s="80"/>
       <c r="R13" s="80"/>
@@ -13875,9 +13805,8 @@
       <c r="F17" s="101"/>
       <c r="G17" s="101"/>
       <c r="H17" s="101"/>
-      <c r="I17" s="102" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,18,FALSE)</f>
-        <v>csp-s复赛模拟卷；上午讲的染色 &amp;&amp; 消消乐(两道)十分(very)神秘的dp题，让我更加熟悉了(神秘)dp的设计状态&amp;&amp;状态转移方程式是怎么出来的。晚上的两道题—four告诉我在某些时候可以用一点(神奇)的特判,数据缺失告诉我要更好的去观察题目本身的意思不要看题目那么长又看不懂就跳过(有可能后面的更加难看懂:) )，之后做题(maybe)会更加easy，复习&amp;&amp;巩固了dp，括号匹配，栈，前缀和等知识，学会了怎么快速找到某一个数字上一次出现的位置，来帮助进行dp的状态转移：）</v>
+      <c r="I17" s="102">
+        <f>IFERROR(INDEX('day7'!$G:$G,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="J17" s="80"/>
       <c r="K17" s="80"/>
@@ -13914,9 +13843,8 @@
       <c r="F19" s="101"/>
       <c r="G19" s="101"/>
       <c r="H19" s="101"/>
-      <c r="I19" s="102" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,19,FALSE)</f>
-        <v>没有仔细观察题目中的数据范围导致数组开小了；有些题目中的神秘性质没有观察到导致扣分；没有分配好做题顺序，应该先做自己擅长的在去做不会的，这样更顺手；有些讲过类似的题没有做出来:(</v>
+      <c r="I19" s="102">
+        <f>IFERROR(INDEX('day7'!$H:$H,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="J19" s="80"/>
       <c r="K19" s="80"/>
@@ -13953,9 +13881,8 @@
       <c r="F21" s="107"/>
       <c r="G21" s="107"/>
       <c r="H21" s="108"/>
-      <c r="I21" s="102" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,20,FALSE)</f>
-        <v>设计dp的(神秘)状态/转移方程是怎么出来的；如何更好的去理解题意,通过样例和解释更好的帮助自己理解题意；怎么想出来一些(神秘)的特判；还需要多练题来提高思维。</v>
+      <c r="I21" s="102">
+        <f>IFERROR(INDEX('day7'!$I:$I,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="J21" s="80"/>
       <c r="K21" s="80"/>
@@ -13975,9 +13902,8 @@
       <c r="C22" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="D22" s="109" t="str">
-        <f>VLOOKUP(E5,'day71'!$B$1:$Z$99,16,FALSE)</f>
-        <v>今天的课程讲解了两道近年的 csp 的动态规划的题目，老师带着大家从部分分入手，帮助大家感受了 dp 真题的难度，以及应该通过怎样的方式去思考。金智宸在本次测试中获得的等级为B-。成绩分析：在第1题中，考虑到了特殊情况，但对数据较大时，考虑有疏漏。在第2题中，想到了贪心算法，但对贪心的策略存在疏漏。在第3题中，考虑小数据时，细节上有一些疏忽。在第4题中，考虑范围过大，未能注意到特殊测试点。此次测验中存在明显不足，体现出在知识掌握和解题方法上的短板。在思考到正解的情况下，但是不能正确的实现代码，以及实现代码后智宸不能保证代码的正确性，后续需要针对弱点进行补强，从而实现持续改进，继续加油。</v>
+      <c r="D22" s="109">
+        <f>IFERROR(INDEX('day7'!$A:$A,MATCH($E$5,'day7'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day7'!$J:$J,MATCH($E$5,'day7'!$B:$B,0)),"")</f>
       </c>
       <c r="E22" s="109"/>
       <c r="F22" s="109"/>
@@ -14977,12 +14903,15 @@
     <mergeCell ref="L13:N15"/>
     <mergeCell ref="O13:S15"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G49:H49 X54:Y54 G69:H69" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C46:J48 C66:J68">
       <formula1>"A,A+,A-,B,B+,B-,C,C+,S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5">
+      <formula1>'day7'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16637,7 +16566,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -16694,9 +16623,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="83"/>
-      <c r="D4" s="151" t="s">
-        <v>54</v>
-      </c>
+      <c r="D4" s="151"/>
       <c r="E4" s="152"/>
       <c r="F4" s="152"/>
       <c r="G4" s="152"/>
@@ -16750,24 +16677,20 @@
     </row>
     <row r="8" customHeight="1" spans="1:10">
       <c r="A8" s="156"/>
-      <c r="B8" s="157" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$Z$100,2,FALSE)</f>
-        <v>A-</v>
+      <c r="B8" s="157">
+        <f>IFERROR(INDEX('day8'!$C:$C,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="C8" s="158"/>
-      <c r="D8" s="157" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$Z$100,3,FALSE)</f>
-        <v>B+</v>
+      <c r="D8" s="157">
+        <f>IFERROR(INDEX('day8'!$D:$D,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="E8" s="158"/>
-      <c r="F8" s="157" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$G$101,4,FALSE)</f>
-        <v>A-</v>
+      <c r="F8" s="157">
+        <f>IFERROR(INDEX('day8'!$C:$C,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="G8" s="158"/>
-      <c r="H8" s="157" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$G$101,5,FALSE)</f>
-        <v>B+</v>
+      <c r="H8" s="157">
+        <f>IFERROR(INDEX('day8'!$D:$D,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="158"/>
       <c r="J8" s="156"/>
@@ -16815,15 +16738,8 @@
         <v>900</v>
       </c>
       <c r="D12" s="164"/>
-      <c r="E12" s="165" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$G$101,6,FALSE)</f>
-        <v>今天主要是补题，只讲了两题，学到了：
-模拟题第3题思路：
-特殊性质：当a=0时，只能对数字进行加或除，此时可选择使用一次加法使n变为距离它最近的2的次幂，再使用(n/2)*c的代价将数字归为1；当b=0时，只能对数字进行减或除，此时可选择将n减到最近的2的次幂后再进行除2操作。但做除时还要考虑当前是直接进行n-1次-1更优还是进行n/2次/2更优；当a=b=c时，对于n只要是偶数就能除就除。当n为2的次幂时，直接全部/2即可，否则寻找n在2进制下有多少个1，在取将n进行一次加后进行除法的代价和进行1的数量的加法后进行除法的最小值。
-正解：对于n要进行2进制下1的个数次-1的操作。但对于0b101111来说，最优解是将低位连续的1变为高位连续的1，以此优化减法次数就是最优算法。
-以后考试若出现+1，-1，/2的操作就忘二进制想
-模拟题第4题思路：
-合法方案=总方案数（m的-1的个数次幂）-不合法方案数（1、只有一种字符，如aaaaaaaa 2、长度为奇数的只有2种字符的回文串，如abababa 3、只有两种字符且其中一个字符只有1个的回文串，例如aaaaabaaaaa）</v>
+      <c r="E12" s="165">
+        <f>IFERROR(INDEX('day8'!$N:$N,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="F12" s="166"/>
       <c r="G12" s="166"/>
@@ -16850,12 +16766,7 @@
         <v>901</v>
       </c>
       <c r="D14" s="164"/>
-      <c r="E14" s="165" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$Z$101,7,FALSE)</f>
-        <v>第一题忘开long long导致样例差点没过
-第三题没考虑异或的优先级，没加括号导致没过
-第七题开太多long long导致内存爆掉</v>
-      </c>
+      <c r="E14" s="165"/>
       <c r="F14" s="165"/>
       <c r="G14" s="165"/>
       <c r="H14" s="165"/>
@@ -16881,10 +16792,7 @@
         <v>902</v>
       </c>
       <c r="D16" s="164"/>
-      <c r="E16" s="170" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$Z$101,8,FALSE)</f>
-        <v>写符合时先考虑优先级，多复习模板代码，能不开开long long就不开，防止在思路正确下内存爆炸导致大部分样例不过</v>
-      </c>
+      <c r="E16" s="170"/>
       <c r="F16" s="170"/>
       <c r="G16" s="170"/>
       <c r="H16" s="170"/>
@@ -16908,10 +16816,8 @@
       <c r="B18" s="162" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="166" t="str">
-        <f>VLOOKUP(D4,'day8'!$B$7:$Z$100,9,FALSE)</f>
-        <v>本节课的核心内容是对昨日测试第三题的思路复盘，并结合多种类型的字符串问题进行了拓展训练。课堂重点放在“分类讨论”这一方法的应用上，老师通过多角度拆分问题，让同学们理解到在算法竞赛中灵活分情况分析的重要性。岳琳课堂参与积极，能跟上讲解并利用课余时间补题；理解力良好，已经会把涉及加/减/乘/除 2 的操作放到二进制角度思考，也掌握用“总情况减去不合法情况”简化计数题的方法。补题较勤，但实现细节上有几次失误：忘记用 long long 导致样例差点不过、算式优先级漏加括号出错、以及因过多使用 long long 导致内存问题，这些都是容易通过赛前检查避免的小失误。
-小结与建议：把模板当成必备工具，每天抽 15–20 分钟默写并跑一跑；提交前先用几个小样例检查输出，注意运算优先级与括号、变量类型别乱用 long long，遇到问题别慌，缩小样例一步步找错；每周做几道综合题并写两三句复盘，久了这些低级错误就会少很多。</v>
+      <c r="C18" s="166">
+        <f>IFERROR(INDEX('day8'!$A:$A,MATCH($D$4,'day8'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day8'!$O:$O,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
       </c>
       <c r="D18" s="166"/>
       <c r="E18" s="166"/>
@@ -16974,9 +16880,12 @@
     <mergeCell ref="B4:C5"/>
     <mergeCell ref="C18:I19"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:G9 F11:G11 G13:H13" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4">
+      <formula1>'day8'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18170,7 +18079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -18272,9 +18181,7 @@
         <v>553</v>
       </c>
       <c r="D5" s="76"/>
-      <c r="E5" s="50" t="s">
-        <v>54</v>
-      </c>
+      <c r="E5" s="50"/>
       <c r="F5" s="77"/>
       <c r="G5" s="77"/>
       <c r="H5" s="77"/>
@@ -18344,25 +18251,22 @@
     <row r="8" ht="30.75" customHeight="1" spans="1:20">
       <c r="A8" s="73"/>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,3,FALSE)</f>
-        <v>B</v>
+      <c r="C8" s="87">
+        <f>IFERROR(INDEX('day9'!$D:$D,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="D8" s="80"/>
       <c r="E8" s="80"/>
       <c r="F8" s="80"/>
       <c r="G8" s="80"/>
-      <c r="H8" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,3,FALSE)</f>
-        <v>B</v>
+      <c r="H8" s="87">
+        <f>IFERROR(INDEX('day9'!$E:$E,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="80"/>
       <c r="J8" s="80"/>
       <c r="K8" s="80"/>
       <c r="L8" s="80"/>
-      <c r="M8" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,4,FALSE)</f>
-        <v>B</v>
+      <c r="M8" s="87">
+        <f>IFERROR(INDEX('day9'!$F:$F,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="N8" s="80"/>
       <c r="O8" s="80"/>
@@ -18453,34 +18357,19 @@
     <row r="13" ht="66.75" customHeight="1" spans="1:20">
       <c r="A13" s="73"/>
       <c r="B13" s="78"/>
-      <c r="C13" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,15,FALSE)</f>
-        <v>B</v>
-      </c>
+      <c r="C13" s="87"/>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
-      <c r="F13" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,16,FALSE)</f>
-        <v>B</v>
-      </c>
+      <c r="F13" s="87"/>
       <c r="G13" s="80"/>
       <c r="H13" s="81"/>
-      <c r="I13" s="94" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,17,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="I13" s="94"/>
       <c r="J13" s="80"/>
       <c r="K13" s="81"/>
-      <c r="L13" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,18,FALSE)</f>
-        <v>C</v>
-      </c>
+      <c r="L13" s="87"/>
       <c r="M13" s="80"/>
       <c r="N13" s="81"/>
-      <c r="O13" s="87" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,19,FALSE)</f>
-        <v>B</v>
-      </c>
+      <c r="O13" s="87"/>
       <c r="P13" s="80"/>
       <c r="Q13" s="80"/>
       <c r="R13" s="80"/>
@@ -18554,16 +18443,8 @@
       <c r="F17" s="101"/>
       <c r="G17" s="101"/>
       <c r="H17" s="101"/>
-      <c r="I17" s="102" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,12,FALSE)</f>
-        <v>今天学到了：
-·2021-3回文思路：由于b时一个回文串，所以我们选择了第一个数，最后一个数也确定了。令l1=1，r1=2n，第一个数可以在a[l]与a[r]间选择，假设选择了a[l]作为第一个数，则最后一个数也确定了。令x为与选择的数相同的另一个数的下标-1，y为下标+1，令l+1，则第2个数同第1个数的操作，倒数第2个数在a[x]与a[y]间选择。如果两侧的都可以选，优先选左侧的，直到x=l,y=r结束。
-·模拟题第3题思路：只考虑aa，abab的选择情况最有价值，abba不满足
-·模拟题第4题思路：遍历每一行上方1010..形式的长度，再对于每一列用单调栈寻找最大矩形（同玉蟾宫）
-这20天总共学到了：
-1、模板代码：并查集、st表、树状数组、树上差分、LCA、最短路问题、最小生成树、树的直径、树的重心、归并排序、逆序对、快速排序与选择
-2、初赛知识：图论、树、Linux操作系统、组合数学、逆元
-3、往年真题</v>
+      <c r="I17" s="102">
+        <f>IFERROR(INDEX('day9'!$G:$G,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="J17" s="80"/>
       <c r="K17" s="80"/>
@@ -18600,11 +18481,8 @@
       <c r="F19" s="101"/>
       <c r="G19" s="101"/>
       <c r="H19" s="101"/>
-      <c r="I19" s="102" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,13,FALSE)</f>
-        <v>做模拟题第1题时想得太难了导致浪费时间
-做模拟题第2题时优化思路正确但写代码时不清导致代码写错
-做模拟题第3题时没读懂题就做导致做不出来</v>
+      <c r="I19" s="102">
+        <f>IFERROR(INDEX('day9'!$H:$H,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="J19" s="80"/>
       <c r="K19" s="80"/>
@@ -18641,11 +18519,8 @@
       <c r="F21" s="107"/>
       <c r="G21" s="107"/>
       <c r="H21" s="108"/>
-      <c r="I21" s="102" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,14,FALSE)</f>
-        <v>出现思路时提前写出来免得忘了，题目多读几遍，不放过任何一个关键词。
-之后多复习模板代码，多背初赛常见知识点，多复习之前做过的题，温习思路和技巧。
-考试时先读清题，注意关键词、数据范围、样例、特殊性质。先写暴力代码，全部暴力完后再思考优化，思考到后先写下来再改代码。</v>
+      <c r="I21" s="102">
+        <f>IFERROR(INDEX('day9'!$I:$I,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="J21" s="80"/>
       <c r="K21" s="80"/>
@@ -18665,11 +18540,8 @@
       <c r="C22" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="D22" s="109" t="str">
-        <f>VLOOKUP(E5,'day91'!$B$1:$AD$100,20,FALSE)</f>
-        <v>今天的课程讲解了两道近年的 CSP 动态规划真题，老师带着大家从部分分入手，帮助大家感受了 DP 真题的难度，以及应该通过怎样的方式去思考。岳琳在本次测试中的整体评级为 B。
-在考试中，他未能正确解决 T2 的最短路问题，T3 和 T4 也未能写出完整的暴力代码，导致总分较低。主要问题在于 动态规划掌握不够牢固、题目理解不够深入，以及考试策略欠缺。他在比赛中没有很好地保证基础分数，也没有利用暴力代码来对拍和验证思路，从而影响了整体发挥。
-总体来看，岳琳已经积累了一些算法和模板，但在实际比赛中的应用还不够熟练。后续训练中，需要重点加强 最短路（Dijkstra）、动态规划的状态设计与转移、单调栈 等常见算法的练习，并在模拟赛中训练 考试节奏和策略，学会先确保部分分，再逐步优化。只要在细节和实现上更加严谨，他的成绩会逐步提升。</v>
+      <c r="D22" s="109">
+        <f>IFERROR(INDEX('day9'!$A:$A,MATCH($E$5,'day9'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day9'!$J:$J,MATCH($E$5,'day9'!$B:$B,0)),"")</f>
       </c>
       <c r="E22" s="109"/>
       <c r="F22" s="109"/>
@@ -19669,12 +19541,15 @@
     <mergeCell ref="L13:N15"/>
     <mergeCell ref="O13:S15"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G78:H78 U78:V78 G98:H98" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C75:J77 C95:J97">
       <formula1>"A,A+,A-,B,B+,B-,C,C+,S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5">
+      <formula1>'day9'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22287,7 +22162,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -22386,9 +22261,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="83"/>
-      <c r="D4" s="127" t="s">
-        <v>69</v>
-      </c>
+      <c r="D4" s="127"/>
       <c r="E4" s="196"/>
       <c r="F4" s="196"/>
       <c r="G4" s="196"/>
@@ -22489,24 +22362,20 @@
     </row>
     <row r="8" customHeight="1" spans="1:25">
       <c r="A8" s="73"/>
-      <c r="B8" s="198" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$G$85,2,FALSE)</f>
-        <v>A-</v>
+      <c r="B8" s="198">
+        <f>IFERROR(INDEX('day1'!$C:$C,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="C8" s="158"/>
-      <c r="D8" s="198" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$G$85,3,FALSE)</f>
-        <v>A</v>
+      <c r="D8" s="198">
+        <f>IFERROR(INDEX('day1'!$E:$E,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="E8" s="158"/>
-      <c r="F8" s="198" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$G$85,4,FALSE)</f>
-        <v>A-</v>
+      <c r="F8" s="198">
+        <f>IFERROR(INDEX('day1'!$D:$D,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="G8" s="158"/>
-      <c r="H8" s="198" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$G$85,5,FALSE)</f>
-        <v>A-</v>
+      <c r="H8" s="198">
+        <f>IFERROR(INDEX('day1'!$F:$F,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="158"/>
       <c r="J8" s="73"/>
@@ -22621,13 +22490,8 @@
         <v>181</v>
       </c>
       <c r="D12" s="81"/>
-      <c r="E12" s="118" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$G$85,6,FALSE)</f>
-        <v>复习提高组算法：如前缀和，st表，树状数组，
-最优解问题：二分，贪心，枚举，最短路
-找父母问题：树状数组，并查集，最小生成树
-图上问题的算法：弗洛伊德；dij，spfa
-树上问题：换根dp，树上前缀和与差分</v>
+      <c r="E12" s="118">
+        <f>IFERROR(INDEX('day1'!$G:$G,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="F12" s="120"/>
       <c r="G12" s="120"/>
@@ -22678,9 +22542,8 @@
         <v>182</v>
       </c>
       <c r="D14" s="81"/>
-      <c r="E14" s="118" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$J$85,7,FALSE)</f>
-        <v>lca题目中for循环边界值写错了，考试时时一些能通过暴力或特殊样例骗分的没拿到</v>
+      <c r="E14" s="118">
+        <f>IFERROR(INDEX('day1'!$H:$H,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="F14" s="118"/>
       <c r="G14" s="118"/>
@@ -22737,9 +22600,8 @@
         <v>184</v>
       </c>
       <c r="D16" s="81"/>
-      <c r="E16" s="118" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$J$85,8,FALSE)</f>
-        <v>动态规划问题的状态转移方程，多做一些dp题目，练习更加熟练推导状态转移方程</v>
+      <c r="E16" s="118">
+        <f>IFERROR(INDEX('day1'!$I:$I,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="F16" s="118"/>
       <c r="G16" s="118"/>
@@ -22792,10 +22654,8 @@
       <c r="B18" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="120" t="str">
-        <f>VLOOKUP(D4,'day1'!$B$1:$Z$85,9,FALSE)</f>
-        <v>今天主要复习了提高组的算法模板，先讲解了各类模板的基础功能，再结合实例分析了它们在实际问题中的运用技巧。熊子轩同学对模板的理解比较到位，在课堂中能灵活选用与组合，思路清晰，条理分明，能够针对不同题型提出恰当的算法方案。在测试中，他能迅速将常用模板应用到具体题目中，代码编写稳健，整体表现积极。
-不过在模板题部分，有一道题因细节处理不够严谨而失分较多；而在思维题部分，他采用了多道题的暴力解法，虽然没有完全解出最优解，但也凭借这种策略拿到了可观的分数。若能在细节检查上更加严谨，并在思维题中多尝试优化思路，成绩还有进一步提升的空间。</v>
+      <c r="C18" s="120">
+        <f>IFERROR(INDEX('day1'!$A:$A,MATCH($D$4,'day1'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day1'!$J:$J,MATCH($D$4,'day1'!$B:$B,0)),"")</f>
       </c>
       <c r="D18" s="121"/>
       <c r="E18" s="121"/>
@@ -23278,12 +23138,15 @@
     <mergeCell ref="D4:I5"/>
     <mergeCell ref="B4:C5"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F11:G11 G13:H13 U13:V13 G35:H35" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C32:J34">
       <formula1>"A,A+,A-,B,B+,B-,C,C+,S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4">
+      <formula1>'day1'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24092,7 +23955,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -24186,9 +24049,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="83"/>
-      <c r="D4" s="134" t="s">
-        <v>95</v>
-      </c>
+      <c r="D4" s="134"/>
       <c r="E4" s="196"/>
       <c r="F4" s="196"/>
       <c r="G4" s="196"/>
@@ -24297,24 +24158,20 @@
     </row>
     <row r="8" ht="30.75" customHeight="1" spans="1:25">
       <c r="A8" s="73"/>
-      <c r="B8" s="198" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$G$100,2,FALSE)</f>
-        <v>A-</v>
+      <c r="B8" s="198">
+        <f>IFERROR(INDEX('day2'!$C:$C,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="C8" s="158"/>
-      <c r="D8" s="198" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$G$100,3,FALSE)</f>
-        <v>B+</v>
+      <c r="D8" s="198">
+        <f>IFERROR(INDEX('day2'!$E:$E,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="E8" s="158"/>
-      <c r="F8" s="198" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$G$100,4,FALSE)</f>
-        <v>B+</v>
+      <c r="F8" s="198">
+        <f>IFERROR(INDEX('day2'!$D:$D,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="G8" s="158"/>
-      <c r="H8" s="198" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$G$100,5,FALSE)</f>
-        <v>B+</v>
+      <c r="H8" s="198">
+        <f>IFERROR(INDEX('day2'!$F:$F,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="158"/>
       <c r="J8" s="73"/>
@@ -24421,9 +24278,8 @@
         <v>181</v>
       </c>
       <c r="D12" s="81"/>
-      <c r="E12" s="118" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$G$100,6,FALSE)</f>
-        <v>记忆化搜索，背包 DP，区间 DP，树形 DP，状压 DP，单调队列/单调栈优化DP</v>
+      <c r="E12" s="118">
+        <f>IFERROR(INDEX('day2'!$G:$G,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="F12" s="120"/>
       <c r="G12" s="120"/>
@@ -24480,15 +24336,8 @@
         <v>182</v>
       </c>
       <c r="D14" s="81"/>
-      <c r="E14" s="118" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$Z$100,7,FALSE)</f>
-        <v>关于DP设计与exgcd算法掌握的现状反思
-最近在算法练习中遇到了明显的瓶颈。动态规划(DP)部分始终难以突破设计关，面对新问题时常常陷入状态定义的迷茫。具体表现为：
-无法准确识别子问题结构
-状态转移方程推导耗时过长
-边界条件处理经常遗漏
-而在数论算法的exgcd（扩展欧几里得算法）实现中
-对递归终止条件的理解不够直观</v>
+      <c r="E14" s="118">
+        <f>IFERROR(INDEX('day2'!$H:$H,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="F14" s="118"/>
       <c r="G14" s="118"/>
@@ -24543,9 +24392,8 @@
         <v>184</v>
       </c>
       <c r="D16" s="81"/>
-      <c r="E16" s="60" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$Z$100,8,FALSE)</f>
-        <v>多练习一些DP题目，多写几次exgcd</v>
+      <c r="E16" s="60">
+        <f>IFERROR(INDEX('day2'!$I:$I,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="F16" s="118"/>
       <c r="G16" s="118"/>
@@ -24598,9 +24446,8 @@
       <c r="B18" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="120" t="str">
-        <f>VLOOKUP(D4,'day2'!$B$7:$Z$100,9,FALSE)</f>
-        <v>今天重点讲解了种常见的数据结构在动态规划状态转移中的加速技巧。对于较难的题目也有很好的探究精神，对于早上讲解的动态规划问题，维皓也能及时想到朴素的转移方程，在老师讲解后能够理解优化转移的技巧。在模版测试中，维皓在今天的模版练习中，涵语对于 dp 的模版掌握的不错，基本都能写对，但是对于其他的一些模版维皓 掌握的还是有些欠缺。在代码方面，维皓在在面对高难度或综合性问题时思路拓展和细节优化仍需加强，在做题目时还是需要多考虑一些特殊的情况，去设计状态，我们会在后续加强孩子对于基础动态规划的练习，在实战中真正运用动态规划的思想，继续加油。</v>
+      <c r="C18" s="120">
+        <f>IFERROR(INDEX('day2'!$A:$A,MATCH($D$4,'day2'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day2'!$J:$J,MATCH($D$4,'day2'!$B:$B,0)),"")</f>
       </c>
       <c r="D18" s="120"/>
       <c r="E18" s="120"/>
@@ -24727,9 +24574,12 @@
     <mergeCell ref="B4:C5"/>
     <mergeCell ref="C18:I19"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F11:G11 U11:V11 G13:H13" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4">
+      <formula1>'day2'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -25538,7 +25388,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -25632,9 +25482,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="83"/>
-      <c r="D4" s="139" t="s">
-        <v>110</v>
-      </c>
+      <c r="D4" s="139"/>
       <c r="E4" s="196"/>
       <c r="F4" s="196"/>
       <c r="G4" s="196"/>
@@ -25743,24 +25591,20 @@
     </row>
     <row r="8" ht="30.75" customHeight="1" spans="1:25">
       <c r="A8" s="73"/>
-      <c r="B8" s="198" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$G$100,2,FALSE)</f>
-        <v>A-</v>
+      <c r="B8" s="198">
+        <f>IFERROR(INDEX('day3'!$C:$C,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="C8" s="158"/>
-      <c r="D8" s="198" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$G$100,3,FALSE)</f>
-        <v>B</v>
+      <c r="D8" s="198">
+        <f>IFERROR(INDEX('day3'!$E:$E,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="E8" s="158"/>
-      <c r="F8" s="198" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$G$100,4,FALSE)</f>
-        <v>B</v>
+      <c r="F8" s="198">
+        <f>IFERROR(INDEX('day3'!$D:$D,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="G8" s="158"/>
-      <c r="H8" s="198" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$G$100,5,FALSE)</f>
-        <v>B-</v>
+      <c r="H8" s="198">
+        <f>IFERROR(INDEX('day3'!$F:$F,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="I8" s="158"/>
       <c r="J8" s="73"/>
@@ -25867,9 +25711,8 @@
         <v>181</v>
       </c>
       <c r="D12" s="81"/>
-      <c r="E12" s="118" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$G$100,6,FALSE)</f>
-        <v>折半搜索；遇到情况较少的博弈类题目，先分类讨论，在总结；数学中判断两个函数是否有交点，联立方程通过德尔塔(小三角 = b^2+4ac)看是否有解；把一些不是图论的题目经过(神秘)分析转换后变成图上的题目；在求符合某种特殊的方案数时，如果直接计算能不太行，就可以用：合法方案数 = 总数-不合法数，用于解决一些求方案数(计数)问题。把之前没有学好的东西，巩固的更好，对于难题就有更多的手段去解决。</v>
+      <c r="E12" s="118">
+        <f>IFERROR(INDEX('day3'!$G:$G,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="F12" s="120"/>
       <c r="G12" s="120"/>
@@ -25926,9 +25769,8 @@
         <v>182</v>
       </c>
       <c r="D14" s="81"/>
-      <c r="E14" s="118" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$Z$100,7,FALSE)</f>
-        <v>没有把控好时间，只顾着做一道题；没有仔细的观察题目导致扣分，数组开小导致越界。</v>
+      <c r="E14" s="118">
+        <f>IFERROR(INDEX('day3'!$H:$H,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="F14" s="118"/>
       <c r="G14" s="118"/>
@@ -25983,9 +25825,8 @@
         <v>184</v>
       </c>
       <c r="D16" s="81"/>
-      <c r="E16" s="118" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$Z$100,8,FALSE)</f>
-        <v>如何把一些不是图论的题目经过(神秘)分析转换后变成图上的题目的(神秘)方法；博弈类题目的分类讨论；折半搜索；练习dp的题目来多加练习设计状态（转移方程）的能力</v>
+      <c r="E16" s="118">
+        <f>IFERROR(INDEX('day3'!$I:$I,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="F16" s="118"/>
       <c r="G16" s="118"/>
@@ -26038,9 +25879,8 @@
       <c r="B18" s="101" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="120" t="str">
-        <f>VLOOKUP(D4,'day3'!$B$7:$Z$100,9,FALSE)</f>
-        <v>今天主要选讲了提高组的真题，聚焦在如何从题目中捕捉特殊性质与关键特点，并结合一些“小技巧”来将原本 O(n²) 或更高复杂度的算法调优到 O(n log n) 或 O(n) 级别。智宸在课堂上能够专心听讲并在必要时做出回应。在代码方面，智宸已能意识到从题目中提取关键信息对于算法的重要性，并尝试使用基础的小技巧来缩减常数或降低复杂度。在测试中，智宸能够在题目中抓住关键性质，成功写出了一些题目的部分分代码，还是不错的。但是在一道用二分优化的题目中，孩子没想到优化方法，后续需要通过不断练习来提高算法优化技巧的熟练度。后续会通过不断练习来提高算法优化技巧的熟练度。</v>
+      <c r="C18" s="120">
+        <f>IFERROR(INDEX('day3'!$A:$A,MATCH($D$4,'day3'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day3'!$J:$J,MATCH($D$4,'day3'!$B:$B,0)),"")</f>
       </c>
       <c r="D18" s="120"/>
       <c r="E18" s="120"/>
@@ -26464,12 +26304,15 @@
     <mergeCell ref="G47:H48"/>
     <mergeCell ref="I47:J48"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:G9 F11:G11 U11:V11 G13:H13 G52:H52" errorStyle="information">
       <formula1>"A,B,C,暂无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C49:J51">
       <formula1>"A,A+,A-,B,B+,B-,C,C+,S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4">
+      <formula1>'day3'!$B:$B</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix feedback sheet link checks
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -7896,10 +7896,7 @@
         <v>190</v>
       </c>
       <c r="D70" s="76"/>
-      <c r="E70" s="124" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="E70" s="124"/>
       <c r="F70" s="125"/>
       <c r="G70" s="125"/>
       <c r="H70" s="125"/>
@@ -16817,7 +16814,7 @@
         <v>186</v>
       </c>
       <c r="C18" s="166">
-        <f>IFERROR(INDEX('day8'!$A:$A,MATCH($D$4,'day8'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day8'!$O:$O,MATCH($D$4,'day8'!$B:$B,0)),"")</f>
+        <f>IFERROR(IF(INDEX('day8'!$O:$O,MATCH($D$4,'day8'!$B:$B,0))&lt;&gt;"",INDEX('day8'!$A:$A,MATCH($D$4,'day8'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day8'!$O:$O,MATCH($D$4,'day8'!$B:$B,0)),INDEX('day8'!$N:$N,MATCH($D$4,'day8'!$B:$B,0))),"")</f>
       </c>
       <c r="D18" s="166"/>
       <c r="E18" s="166"/>

</xml_diff>

<commit_message>
Fix Day5 feedback sheet layout
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -9555,7 +9555,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AI19"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col min="3" max="3" width="9.125" customWidth="1"/>
@@ -9578,8 +9578,10 @@
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:35">
-      <c r="A1" s="62" t="s">
-        <v>173</v>
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>暑假集训学习反馈卡</t>
+        </is>
       </c>
       <c r="B1" s="63"/>
       <c r="C1" s="63"/>
@@ -9600,9 +9602,7 @@
       <c r="R1" s="63"/>
       <c r="S1" s="63"/>
       <c r="T1" s="64"/>
-      <c r="X1" s="62" t="s">
-        <v>174</v>
-      </c>
+      <c r="X1" s="62"/>
       <c r="Y1" s="63"/>
       <c r="Z1" s="63"/>
       <c r="AA1" s="63"/>
@@ -9699,16 +9699,16 @@
       <c r="AE4" s="113"/>
       <c r="AF4" s="113"/>
       <c r="AG4" s="113"/>
-      <c r="AH4" s="72" t="s">
-        <v>8</v>
-      </c>
+      <c r="AH4" s="72"/>
       <c r="AI4" s="73"/>
     </row>
     <row r="5" ht="21" customHeight="1" spans="1:35">
       <c r="A5" s="73"/>
       <c r="B5" s="74"/>
-      <c r="C5" s="75" t="s">
-        <v>553</v>
+      <c r="C5" s="75" t="inlineStr">
+        <is>
+          <t>学员姓名</t>
+        </is>
       </c>
       <c r="D5" s="76"/>
       <c r="E5" s="180"/>
@@ -9729,9 +9729,7 @@
       <c r="T5" s="73"/>
       <c r="X5" s="73"/>
       <c r="Y5" s="74"/>
-      <c r="Z5" s="114" t="s">
-        <v>175</v>
-      </c>
+      <c r="Z5" s="114"/>
       <c r="AA5" s="60"/>
       <c r="AB5" s="60"/>
       <c r="AC5" s="60"/>
@@ -9745,25 +9743,35 @@
     <row r="6" customHeight="1" spans="1:35">
       <c r="A6" s="73"/>
       <c r="B6" s="78"/>
-      <c r="C6" s="79" t="s">
-        <v>13</v>
+      <c r="C6" s="79" t="inlineStr">
+        <is>
+          <t>课堂积极性</t>
+        </is>
       </c>
       <c r="D6" s="80"/>
       <c r="E6" s="80"/>
       <c r="F6" s="80"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="82" t="s">
-        <v>14</v>
-      </c>
+      <c r="G6" s="81" t="inlineStr">
+        <is>
+          <t>代码能力</t>
+        </is>
+      </c>
+      <c r="H6" s="82"/>
       <c r="I6" s="82"/>
       <c r="J6" s="82"/>
-      <c r="K6" s="82"/>
+      <c r="K6" s="82" t="inlineStr">
+        <is>
+          <t>理解能力</t>
+        </is>
+      </c>
       <c r="L6" s="83"/>
-      <c r="M6" s="79" t="s">
-        <v>15</v>
-      </c>
+      <c r="M6" s="79"/>
       <c r="N6" s="79"/>
-      <c r="O6" s="79"/>
+      <c r="O6" s="79" t="inlineStr">
+        <is>
+          <t>综合评价</t>
+        </is>
+      </c>
       <c r="P6" s="79"/>
       <c r="Q6" s="80"/>
       <c r="R6" s="80"/>
@@ -9771,22 +9779,14 @@
       <c r="T6" s="73"/>
       <c r="X6" s="73"/>
       <c r="Y6" s="78"/>
-      <c r="Z6" s="116" t="s">
-        <v>176</v>
-      </c>
+      <c r="Z6" s="116"/>
       <c r="AA6" s="83"/>
-      <c r="AB6" s="116" t="s">
-        <v>177</v>
-      </c>
+      <c r="AB6" s="116"/>
       <c r="AC6" s="82"/>
       <c r="AD6" s="83"/>
-      <c r="AE6" s="116" t="s">
-        <v>178</v>
-      </c>
+      <c r="AE6" s="116"/>
       <c r="AF6" s="83"/>
-      <c r="AG6" s="116" t="s">
-        <v>179</v>
-      </c>
+      <c r="AG6" s="116"/>
       <c r="AH6" s="83"/>
       <c r="AI6" s="73"/>
     </row>
@@ -9828,24 +9828,26 @@
       <c r="A8" s="73"/>
       <c r="B8" s="78"/>
       <c r="C8" s="87">
-        <f>IFERROR(INDEX('day5'!$D:$D,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
+        <f>IFERROR(INDEX('day5'!$C:$C,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="D8" s="80"/>
       <c r="E8" s="80"/>
       <c r="F8" s="80"/>
-      <c r="G8" s="80"/>
-      <c r="H8" s="87">
-        <f>IFERROR(INDEX('day5'!$E:$E,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
-      </c>
+      <c r="G8" s="80">
+        <f>IFERROR(INDEX('day5'!$D:$D,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
+      </c>
+      <c r="H8" s="87"/>
       <c r="I8" s="80"/>
       <c r="J8" s="80"/>
-      <c r="K8" s="80"/>
+      <c r="K8" s="80">
+        <f>IFERROR(INDEX('day5'!$E:$E,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
+      </c>
       <c r="L8" s="80"/>
-      <c r="M8" s="87">
+      <c r="M8" s="87"/>
+      <c r="N8" s="80"/>
+      <c r="O8" s="80">
         <f>IFERROR(INDEX('day5'!$F:$F,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
-      <c r="N8" s="80"/>
-      <c r="O8" s="80"/>
       <c r="P8" s="80"/>
       <c r="Q8" s="80"/>
       <c r="R8" s="80"/>
@@ -9853,23 +9855,14 @@
       <c r="T8" s="73"/>
       <c r="X8" s="73"/>
       <c r="Y8" s="78"/>
-      <c r="Z8" s="94">
-        <v>30</v>
-      </c>
+      <c r="Z8" s="94"/>
       <c r="AA8" s="94"/>
-      <c r="AB8" s="94">
-        <v>28.5</v>
-      </c>
+      <c r="AB8" s="94"/>
       <c r="AC8" s="94"/>
       <c r="AD8" s="94"/>
-      <c r="AE8" s="94">
-        <v>30</v>
-      </c>
+      <c r="AE8" s="94"/>
       <c r="AF8" s="94"/>
-      <c r="AG8" s="94">
-        <f>SUM(Z8:AF10)</f>
-        <v>88.5</v>
-      </c>
+      <c r="AG8" s="94"/>
       <c r="AH8" s="94"/>
       <c r="AI8" s="73"/>
     </row>
@@ -9924,29 +9917,25 @@
     <row r="11" customHeight="1" spans="1:35">
       <c r="A11" s="73"/>
       <c r="B11" s="78"/>
-      <c r="C11" s="79" t="s">
-        <v>458</v>
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>学生总结</t>
+        </is>
       </c>
       <c r="D11" s="89"/>
       <c r="E11" s="90"/>
-      <c r="F11" s="79" t="s">
-        <v>459</v>
+      <c r="F11" s="79">
+        <f>IFERROR(INDEX('day5'!$G:$G,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
       </c>
       <c r="G11" s="89"/>
       <c r="H11" s="90"/>
-      <c r="I11" s="79" t="s">
-        <v>460</v>
-      </c>
+      <c r="I11" s="79"/>
       <c r="J11" s="89"/>
       <c r="K11" s="90"/>
-      <c r="L11" s="79" t="s">
-        <v>461</v>
-      </c>
+      <c r="L11" s="79"/>
       <c r="M11" s="89"/>
       <c r="N11" s="90"/>
-      <c r="O11" s="79" t="s">
-        <v>554</v>
-      </c>
+      <c r="O11" s="79"/>
       <c r="P11" s="89"/>
       <c r="Q11" s="89"/>
       <c r="R11" s="89"/>
@@ -9988,17 +9977,11 @@
       <c r="T12" s="73"/>
       <c r="X12" s="73"/>
       <c r="Y12" s="78"/>
-      <c r="Z12" s="101" t="s">
-        <v>180</v>
-      </c>
-      <c r="AA12" s="119" t="s">
-        <v>181</v>
-      </c>
+      <c r="Z12" s="101"/>
+      <c r="AA12" s="119"/>
       <c r="AB12" s="80"/>
       <c r="AC12" s="81"/>
-      <c r="AD12" s="118" t="s">
-        <v>183</v>
-      </c>
+      <c r="AD12" s="118"/>
       <c r="AE12" s="118"/>
       <c r="AF12" s="118"/>
       <c r="AG12" s="118"/>
@@ -10008,10 +9991,16 @@
     <row r="13" ht="27" customHeight="1" spans="1:35">
       <c r="A13" s="73"/>
       <c r="B13" s="78"/>
-      <c r="C13" s="87"/>
+      <c r="C13" s="87" t="inlineStr">
+        <is>
+          <t>学生自我反思</t>
+        </is>
+      </c>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
-      <c r="F13" s="87"/>
+      <c r="F13" s="87">
+        <f>IFERROR(INDEX('day5'!$H:$H,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
+      </c>
       <c r="G13" s="80"/>
       <c r="H13" s="81"/>
       <c r="I13" s="94"/>
@@ -10055,14 +10044,10 @@
       <c r="X14" s="73"/>
       <c r="Y14" s="78"/>
       <c r="Z14" s="101"/>
-      <c r="AA14" s="119" t="s">
-        <v>182</v>
-      </c>
+      <c r="AA14" s="119"/>
       <c r="AB14" s="80"/>
       <c r="AC14" s="81"/>
-      <c r="AD14" s="118" t="s">
-        <v>185</v>
-      </c>
+      <c r="AD14" s="118"/>
       <c r="AE14" s="118"/>
       <c r="AF14" s="118"/>
       <c r="AG14" s="118"/>
@@ -10072,10 +10057,16 @@
     <row r="15" ht="5.25" customHeight="1" spans="1:35">
       <c r="A15" s="73"/>
       <c r="B15" s="78"/>
-      <c r="C15" s="84"/>
+      <c r="C15" s="84" t="inlineStr">
+        <is>
+          <t>计划</t>
+        </is>
+      </c>
       <c r="D15" s="85"/>
       <c r="E15" s="86"/>
-      <c r="F15" s="84"/>
+      <c r="F15" s="84">
+        <f>IFERROR(INDEX('day5'!$I:$I,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
+      </c>
       <c r="G15" s="85"/>
       <c r="H15" s="86"/>
       <c r="I15" s="84"/>
@@ -10123,14 +10114,10 @@
       <c r="X16" s="73"/>
       <c r="Y16" s="78"/>
       <c r="Z16" s="101"/>
-      <c r="AA16" s="119" t="s">
-        <v>184</v>
-      </c>
+      <c r="AA16" s="119"/>
       <c r="AB16" s="80"/>
       <c r="AC16" s="81"/>
-      <c r="AD16" s="118" t="s">
-        <v>187</v>
-      </c>
+      <c r="AD16" s="118"/>
       <c r="AE16" s="118"/>
       <c r="AF16" s="118"/>
       <c r="AG16" s="118"/>
@@ -10140,8 +10127,10 @@
     <row r="17" customHeight="1" spans="1:20">
       <c r="A17" s="71"/>
       <c r="B17" s="74"/>
-      <c r="C17" s="101" t="s">
-        <v>186</v>
+      <c r="C17" s="101" t="inlineStr">
+        <is>
+          <t>教师寄语</t>
+        </is>
       </c>
       <c r="D17" s="109">
         <f>IFERROR(INDEX('day5'!$A:$A,MATCH($E$5,'day5'!$B:$B,0))&amp;CHAR(10)&amp;CHAR(10)&amp;INDEX('day5'!$J:$J,MATCH($E$5,'day5'!$B:$B,0)),"")</f>
@@ -10208,60 +10197,33 @@
       <c r="T19" s="110"/>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="24">
+    <mergeCell ref="A1:T3"/>
     <mergeCell ref="B4:S4"/>
-    <mergeCell ref="Y4:AG4"/>
+    <mergeCell ref="A4:A18"/>
+    <mergeCell ref="B5:B18"/>
+    <mergeCell ref="T4:T18"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:S5"/>
-    <mergeCell ref="Z5:AH5"/>
-    <mergeCell ref="C16:S16"/>
-    <mergeCell ref="AA16:AC16"/>
-    <mergeCell ref="AD16:AH16"/>
+    <mergeCell ref="C6:F7"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="K6:N7"/>
+    <mergeCell ref="O6:S7"/>
+    <mergeCell ref="C8:F10"/>
+    <mergeCell ref="G8:J10"/>
+    <mergeCell ref="K8:N10"/>
+    <mergeCell ref="O8:S10"/>
+    <mergeCell ref="C11:E12"/>
+    <mergeCell ref="F11:S12"/>
+    <mergeCell ref="C13:E14"/>
+    <mergeCell ref="F13:S14"/>
+    <mergeCell ref="C15:E16"/>
+    <mergeCell ref="F15:S16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:S18"/>
     <mergeCell ref="A19:T19"/>
-    <mergeCell ref="A4:A16"/>
-    <mergeCell ref="B5:B16"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="T4:T16"/>
-    <mergeCell ref="X4:X16"/>
-    <mergeCell ref="Y5:Y16"/>
-    <mergeCell ref="Z12:Z16"/>
-    <mergeCell ref="AI4:AI16"/>
-    <mergeCell ref="AD12:AH13"/>
-    <mergeCell ref="AD14:AH15"/>
-    <mergeCell ref="AB8:AD10"/>
-    <mergeCell ref="AE8:AF10"/>
-    <mergeCell ref="AG8:AH10"/>
-    <mergeCell ref="AA12:AC13"/>
-    <mergeCell ref="AE6:AF7"/>
-    <mergeCell ref="AG6:AH7"/>
-    <mergeCell ref="AA14:AC15"/>
-    <mergeCell ref="X1:AI3"/>
-    <mergeCell ref="Z6:AA7"/>
-    <mergeCell ref="AB6:AD7"/>
-    <mergeCell ref="Z8:AA10"/>
-    <mergeCell ref="A1:T3"/>
-    <mergeCell ref="C6:G7"/>
-    <mergeCell ref="H6:L7"/>
-    <mergeCell ref="M6:S7"/>
-    <mergeCell ref="D17:S18"/>
-    <mergeCell ref="C11:E12"/>
-    <mergeCell ref="F11:H12"/>
-    <mergeCell ref="I11:K12"/>
-    <mergeCell ref="L11:N12"/>
-    <mergeCell ref="C8:G10"/>
-    <mergeCell ref="H8:L10"/>
-    <mergeCell ref="O11:S12"/>
-    <mergeCell ref="M8:S10"/>
-    <mergeCell ref="C13:E15"/>
-    <mergeCell ref="F13:H15"/>
-    <mergeCell ref="I13:K15"/>
-    <mergeCell ref="L13:N15"/>
-    <mergeCell ref="O13:S15"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AE10:AF11" errorStyle="information">
-      <formula1>"A,B,C,暂无"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5">
       <formula1>'day5'!$B:$B</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Add second feedback card style preview
</commit_message>
<xml_diff>
--- a/XP05反馈表.xlsx
+++ b/XP05反馈表.xlsx
@@ -4,7 +4,7 @@
   <ns0:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <ns0:workbookPr/>
   <ns0:bookViews>
-    <ns0:workbookView windowWidth="29400" windowHeight="12420" activeTab="19"/>
+    <ns0:workbookView windowWidth="29400" windowHeight="12420" activeTab="11"/>
   </ns0:bookViews>
   <ns0:sheets>
     <ns0:sheet name="座位表" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <ns0:sheet name="day4" sheetId="9" r:id="rId9"/>
     <ns0:sheet name="Day4反馈表" sheetId="10" r:id="rId10"/>
     <ns0:sheet name="day5" sheetId="11" r:id="rId11"/>
-    <ns0:sheet name="陈一实" sheetId="13" r:id="rId13"/>
+    <ns0:sheet name="反馈卡样式预览2" sheetId="13" r:id="rId13"/>
     <ns0:sheet name="Day5反馈表" sheetId="14" r:id="rId14"/>
     <ns0:sheet name="day6" sheetId="15" r:id="rId15"/>
     <ns0:sheet name="Day6反馈表" sheetId="17" r:id="rId17"/>
@@ -4670,7 +4670,7 @@
     <ns0:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <ns0:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </ns0:numFmts>
-  <ns0:fonts count="93">
+  <ns0:fonts count="102">
     <ns0:font>
       <ns0:sz val="12"/>
       <ns0:color theme="1"/>
@@ -5290,8 +5290,67 @@
       <ns0:name val="Microsoft YaHei"/>
       <ns0:charset val="134"/>
     </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="22"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FFE8F6F3"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF21313C"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FF21313C"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color rgb="FF6B7B88"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="22"/>
+      <ns0:color rgb="FF0E5A63"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="20"/>
+      <ns0:color rgb="FF12343B"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="10"/>
+      <ns0:color rgb="FF52616B"/>
+      <ns0:name val="Microsoft YaHei"/>
+      <ns0:charset val="134"/>
+    </ns0:font>
   </ns0:fonts>
-  <ns0:fills count="56">
+  <ns0:fills count="65">
     <ns0:fill>
       <ns0:patternFill patternType="none"/>
     </ns0:fill>
@@ -5622,8 +5681,62 @@
         <ns0:bgColor indexed="64"/>
       </ns0:patternFill>
     </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFF4F7F8"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF0F4C5C"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF0B3C49"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFF1B8"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFFFFF"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFE6F0F2"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFFBF0"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFF8FAFB"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFEAF4F4"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
   </ns0:fills>
-  <ns0:borders count="47">
+  <ns0:borders count="49">
     <ns0:border>
       <ns0:left/>
       <ns0:right/>
@@ -6157,6 +6270,36 @@
       </ns0:bottom>
       <ns0:diagonal/>
     </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFF2F6F7"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFF2F6F7"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFF2F6F7"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFF2F6F7"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFD9E2E7"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFD9E2E7"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFD9E2E7"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFD9E2E7"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
   </ns0:borders>
   <ns0:cellStyleXfs count="49">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -6307,7 +6450,7 @@
       <ns0:alignment vertical="center"/>
     </ns0:xf>
   </ns0:cellStyleXfs>
-  <ns0:cellXfs count="230">
+  <ns0:cellXfs count="252">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <ns0:alignment vertical="center"/>
     </ns0:xf>
@@ -6994,6 +7137,72 @@
       <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
     </ns0:xf>
     <ns0:xf numFmtId="0" fontId="88" fillId="54" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="96" fillId="56" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="95" fillId="57" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="93" fillId="57" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="94" fillId="57" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="95" fillId="58" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="97" fillId="59" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="95" fillId="58" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="99" fillId="60" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="99" fillId="59" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="94" fillId="57" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="95" fillId="57" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="101" fillId="56" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="100" fillId="56" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="101" fillId="56" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="97" fillId="61" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="96" fillId="60" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="97" fillId="62" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="96" fillId="62" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="95" fillId="57" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="96" fillId="63" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="97" fillId="64" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="98" fillId="64" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
     </ns0:xf>
   </ns0:cellXfs>
@@ -9308,424 +9517,481 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
-  <sheetData>
-    <row r="1" customHeight="1" spans="1:16">
-      <c r="A1" s="180" t="s">
-        <v>483</v>
-      </c>
-      <c r="B1" s="180" t="s">
-        <v>484</v>
-      </c>
-      <c r="C1" s="180" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="180"/>
-      <c r="E1" s="180"/>
-      <c r="F1" s="180"/>
-      <c r="G1" s="180"/>
-      <c r="H1" s="180"/>
-      <c r="I1" s="180"/>
-      <c r="J1" s="180"/>
-      <c r="K1" s="180"/>
-      <c r="L1" s="180"/>
-      <c r="M1" s="180"/>
-      <c r="N1" s="180"/>
-      <c r="O1" s="180"/>
-      <c r="P1" s="180"/>
-    </row>
-    <row r="2" ht="29.25" customHeight="1" spans="1:16">
-      <c r="A2" s="180">
-        <v>1</v>
-      </c>
-      <c r="B2" s="180">
-        <v>4</v>
-      </c>
-      <c r="C2" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="180" t="s">
-        <v>485</v>
-      </c>
-      <c r="F2" s="180" t="s">
-        <v>486</v>
-      </c>
-      <c r="G2" s="180" t="s">
-        <v>487</v>
-      </c>
-      <c r="H2" s="180" t="s">
-        <v>488</v>
-      </c>
-      <c r="I2" s="180" t="s">
-        <v>489</v>
-      </c>
-      <c r="J2" s="180" t="s">
-        <v>490</v>
-      </c>
-      <c r="K2" s="180" t="s">
-        <v>491</v>
-      </c>
-      <c r="L2" s="180" t="s">
-        <v>492</v>
-      </c>
-      <c r="M2" s="180" t="s">
-        <v>493</v>
-      </c>
-      <c r="N2" s="180" t="s">
-        <v>492</v>
-      </c>
-      <c r="O2" s="180" t="s">
-        <v>494</v>
-      </c>
-      <c r="P2" s="180" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:16">
-      <c r="B3" s="55" t="s">
-        <v>496</v>
-      </c>
-      <c r="L3" s="55" t="s">
-        <v>497</v>
-      </c>
-      <c r="N3" s="55" t="s">
-        <v>498</v>
-      </c>
-      <c r="O3" s="55" t="s">
-        <v>499</v>
-      </c>
-      <c r="P3" s="55" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="5" ht="29.25" customHeight="1" spans="1:16">
-      <c r="A5" s="180">
-        <v>2</v>
-      </c>
-      <c r="B5" s="180">
-        <v>4</v>
-      </c>
-      <c r="C5" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="180" t="s">
-        <v>501</v>
-      </c>
-      <c r="F5" s="188"/>
-      <c r="G5" s="180" t="s">
-        <v>502</v>
-      </c>
-      <c r="H5" s="180" t="s">
-        <v>503</v>
-      </c>
-      <c r="I5" s="189" t="s">
-        <v>504</v>
-      </c>
-      <c r="J5" s="180" t="s">
-        <v>503</v>
-      </c>
-      <c r="K5" s="180" t="s">
-        <v>505</v>
-      </c>
-      <c r="L5" s="180" t="s">
-        <v>506</v>
-      </c>
-      <c r="M5" s="188"/>
-      <c r="N5" s="180" t="s">
-        <v>507</v>
-      </c>
-      <c r="O5" s="180" t="s">
-        <v>508</v>
-      </c>
-      <c r="P5" s="180" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:16">
-      <c r="B6" s="55" t="s">
-        <v>496</v>
-      </c>
-      <c r="L6" s="55" t="s">
-        <v>509</v>
-      </c>
-      <c r="M6" s="55" t="s">
-        <v>509</v>
-      </c>
-      <c r="N6" s="55" t="s">
-        <v>509</v>
-      </c>
-      <c r="O6" s="55" t="s">
-        <v>509</v>
-      </c>
-      <c r="P6" s="55" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="8" ht="29.25" customHeight="1" spans="1:16">
-      <c r="A8" s="180">
-        <v>3</v>
-      </c>
-      <c r="B8" s="180">
-        <v>2</v>
-      </c>
-      <c r="C8" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="180" t="s">
-        <v>510</v>
-      </c>
-      <c r="F8" s="180" t="s">
-        <v>511</v>
-      </c>
-      <c r="G8" s="188">
-        <v>0</v>
-      </c>
-      <c r="H8" s="189" t="s">
-        <v>512</v>
-      </c>
-      <c r="I8" s="189" t="s">
-        <v>513</v>
-      </c>
-      <c r="J8" s="180" t="s">
-        <v>514</v>
-      </c>
-      <c r="K8" s="180" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="9" customHeight="1" spans="1:16">
-      <c r="G9" s="55" t="s">
-        <v>515</v>
-      </c>
-      <c r="J9" s="55" t="s">
-        <v>516</v>
-      </c>
-      <c r="K9" s="55" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="11" ht="29.25" customHeight="1" spans="1:16">
-      <c r="A11" s="180">
-        <v>4</v>
-      </c>
-      <c r="B11" s="180">
-        <v>2</v>
-      </c>
-      <c r="C11" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="180" t="s">
-        <v>518</v>
-      </c>
-      <c r="F11" s="180" t="s">
-        <v>519</v>
-      </c>
-      <c r="G11" s="180" t="s">
-        <v>520</v>
-      </c>
-      <c r="H11" s="180" t="s">
-        <v>521</v>
-      </c>
-      <c r="I11" s="180" t="s">
-        <v>514</v>
-      </c>
-      <c r="J11" s="188">
-        <v>0</v>
-      </c>
-      <c r="K11" s="180" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="12" customHeight="1" spans="1:16">
-      <c r="G12" s="55" t="s">
-        <v>523</v>
-      </c>
-      <c r="I12" s="55" t="s">
-        <v>524</v>
-      </c>
-      <c r="J12" s="55" t="s">
-        <v>525</v>
-      </c>
-      <c r="K12" s="55" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="14" ht="29.25" customHeight="1" spans="1:16">
-      <c r="A14" s="180">
-        <v>5</v>
-      </c>
-      <c r="B14" s="180">
-        <v>6</v>
-      </c>
-      <c r="C14" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E14" s="180" t="s">
-        <v>527</v>
-      </c>
-      <c r="F14" s="180" t="s">
-        <v>528</v>
-      </c>
-      <c r="G14" s="180" t="s">
-        <v>529</v>
-      </c>
-      <c r="H14" s="180" t="s">
-        <v>530</v>
-      </c>
-      <c r="I14" s="180" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="15" customHeight="1" spans="1:16">
-      <c r="F15" s="55" t="s">
-        <v>532</v>
-      </c>
-      <c r="H15" s="55" t="s">
-        <v>509</v>
-      </c>
-      <c r="I15" s="55" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="17" ht="43.5" customHeight="1" spans="1:9">
-      <c r="A17" s="133">
-        <v>6</v>
-      </c>
-      <c r="B17" s="190">
-        <v>9</v>
-      </c>
-      <c r="C17" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="191" t="s">
-        <v>533</v>
-      </c>
-      <c r="F17" s="191" t="s">
-        <v>534</v>
-      </c>
-      <c r="G17" s="191" t="s">
-        <v>535</v>
-      </c>
-      <c r="H17" s="191" t="s">
-        <v>536</v>
-      </c>
-      <c r="I17" s="191" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="18" customHeight="1" spans="1:9">
-      <c r="G18" s="55" t="s">
-        <v>538</v>
-      </c>
-      <c r="H18" s="55" t="s">
-        <v>539</v>
-      </c>
-      <c r="I18" s="55" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="20" ht="43.5" customHeight="1" spans="1:9">
-      <c r="A20" s="133">
-        <v>7</v>
-      </c>
-      <c r="B20" s="133">
-        <v>1</v>
-      </c>
-      <c r="C20" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="191" t="s">
-        <v>541</v>
-      </c>
-      <c r="F20" s="191" t="s">
-        <v>542</v>
-      </c>
-      <c r="G20" s="191" t="s">
-        <v>543</v>
-      </c>
-      <c r="H20" s="191" t="s">
-        <v>544</v>
-      </c>
-      <c r="I20" s="191" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="21" customHeight="1" spans="1:9">
-      <c r="A21" s="133"/>
-      <c r="B21" s="133"/>
-      <c r="C21" s="133"/>
-      <c r="D21" s="133"/>
-      <c r="E21" s="133"/>
-      <c r="F21" s="133"/>
-      <c r="G21" s="133" t="s">
-        <v>546</v>
-      </c>
-      <c r="H21" s="133" t="s">
-        <v>547</v>
-      </c>
-      <c r="I21" s="133" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="23" ht="43.5" customHeight="1" spans="1:9">
-      <c r="A23" s="133">
-        <v>8</v>
-      </c>
-      <c r="B23" s="133">
-        <v>1</v>
-      </c>
-      <c r="C23" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="180" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="191" t="s">
-        <v>548</v>
-      </c>
-      <c r="F23" s="191" t="s">
-        <v>549</v>
-      </c>
-      <c r="G23" s="191" t="s">
-        <v>550</v>
-      </c>
-      <c r="H23" s="191" t="s">
-        <v>551</v>
-      </c>
-      <c r="I23" s="191" t="s">
-        <v>552</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:outlinePr summaryBelow="0" summaryRight="0"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:K25"/>
+  <ns0:sheetFormatPr defaultRowHeight="18"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="10" customWidth="1"/>
+    <ns0:col min="2" max="2" width="10" customWidth="1"/>
+    <ns0:col min="3" max="3" width="4" customWidth="1"/>
+    <ns0:col min="4" max="4" width="12" customWidth="1"/>
+    <ns0:col min="5" max="5" width="12" customWidth="1"/>
+    <ns0:col min="6" max="6" width="12" customWidth="1"/>
+    <ns0:col min="7" max="7" width="12" customWidth="1"/>
+    <ns0:col min="8" max="8" width="12" customWidth="1"/>
+    <ns0:col min="9" max="9" width="12" customWidth="1"/>
+    <ns0:col min="10" max="10" width="12" customWidth="1"/>
+    <ns0:col min="11" max="11" width="4" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:11" ht="22" customHeight="1">
+      <ns0:c r="A1" s="231"/>
+      <ns0:c r="B1" s="231"/>
+      <ns0:c r="C1" s="231"/>
+      <ns0:c r="D1" s="242" t="inlineStr">
+        <ns0:is>
+          <ns0:t>XP05 集训营学习反馈卡</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" s="241"/>
+      <ns0:c r="F1" s="241"/>
+      <ns0:c r="G1" s="241"/>
+      <ns0:c r="H1" s="241"/>
+      <ns0:c r="I1" s="241"/>
+      <ns0:c r="J1" s="241"/>
+      <ns0:c r="K1" s="241"/>
+    </ns0:row>
+    <ns0:row r="2" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A2" s="232" t="inlineStr">
+        <ns0:is>
+          <ns0:t>XP05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="231"/>
+      <ns0:c r="C2" s="231"/>
+      <ns0:c r="D2" s="241"/>
+      <ns0:c r="E2" s="241"/>
+      <ns0:c r="F2" s="241"/>
+      <ns0:c r="G2" s="241"/>
+      <ns0:c r="H2" s="241"/>
+      <ns0:c r="I2" s="241"/>
+      <ns0:c r="J2" s="241"/>
+      <ns0:c r="K2" s="241"/>
+    </ns0:row>
+    <ns0:row r="3" spans="1:11" ht="20" customHeight="1">
+      <ns0:c r="A3" s="233" t="inlineStr">
+        <ns0:is>
+          <ns0:t>每日学习反馈</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="231"/>
+      <ns0:c r="C3" s="231"/>
+      <ns0:c r="D3" s="243" t="inlineStr">
+        <ns0:is>
+          <ns0:t>为家长阅读整理：课程内容、学习状态与老师建议集中展示</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E3" s="241"/>
+      <ns0:c r="F3" s="241"/>
+      <ns0:c r="G3" s="241"/>
+      <ns0:c r="H3" s="241"/>
+      <ns0:c r="I3" s="241"/>
+      <ns0:c r="J3" s="241"/>
+      <ns0:c r="K3" s="241"/>
+    </ns0:row>
+    <ns0:row r="4" spans="1:11" ht="8" customHeight="1">
+      <ns0:c r="A4" s="231"/>
+      <ns0:c r="B4" s="231"/>
+      <ns0:c r="C4" s="231"/>
+      <ns0:c r="D4" s="230"/>
+      <ns0:c r="E4" s="230"/>
+      <ns0:c r="F4" s="230"/>
+      <ns0:c r="G4" s="230"/>
+      <ns0:c r="H4" s="230"/>
+      <ns0:c r="I4" s="230"/>
+      <ns0:c r="J4" s="230"/>
+      <ns0:c r="K4" s="230"/>
+    </ns0:row>
+    <ns0:row r="5" spans="1:11" ht="26" customHeight="1">
+      <ns0:c r="A5" s="234" t="inlineStr">
+        <ns0:is>
+          <ns0:t>学生 / 画像</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="231"/>
+      <ns0:c r="C5" s="231"/>
+      <ns0:c r="D5" s="244" t="inlineStr">
+        <ns0:is>
+          <ns0:t>今日课程内容</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" s="244"/>
+      <ns0:c r="F5" s="244"/>
+      <ns0:c r="G5" s="244"/>
+      <ns0:c r="H5" s="244"/>
+      <ns0:c r="I5" s="244"/>
+      <ns0:c r="J5" s="244"/>
+      <ns0:c r="K5" s="244"/>
+    </ns0:row>
+    <ns0:row r="6" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A6" s="235"/>
+      <ns0:c r="B6" s="231"/>
+      <ns0:c r="C6" s="231"/>
+      <ns0:c r="D6" s="245">
+        <ns0:f>IFERROR(INDEX('day5'!$A:$A,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="E6" s="245"/>
+      <ns0:c r="F6" s="245"/>
+      <ns0:c r="G6" s="245"/>
+      <ns0:c r="H6" s="245"/>
+      <ns0:c r="I6" s="245"/>
+      <ns0:c r="J6" s="245"/>
+      <ns0:c r="K6" s="245"/>
+    </ns0:row>
+    <ns0:row r="7" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A7" s="231"/>
+      <ns0:c r="B7" s="231"/>
+      <ns0:c r="C7" s="231"/>
+      <ns0:c r="D7" s="245"/>
+      <ns0:c r="E7" s="245"/>
+      <ns0:c r="F7" s="245"/>
+      <ns0:c r="G7" s="245"/>
+      <ns0:c r="H7" s="245"/>
+      <ns0:c r="I7" s="245"/>
+      <ns0:c r="J7" s="245"/>
+      <ns0:c r="K7" s="245"/>
+    </ns0:row>
+    <ns0:row r="8" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A8" s="236" t="inlineStr">
+        <ns0:is>
+          <ns0:t>课堂积极性</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="231"/>
+      <ns0:c r="C8" s="231"/>
+      <ns0:c r="D8" s="230"/>
+      <ns0:c r="E8" s="230"/>
+      <ns0:c r="F8" s="230"/>
+      <ns0:c r="G8" s="230"/>
+      <ns0:c r="H8" s="230"/>
+      <ns0:c r="I8" s="230"/>
+      <ns0:c r="J8" s="230"/>
+      <ns0:c r="K8" s="230"/>
+    </ns0:row>
+    <ns0:row r="9" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A9" s="237">
+        <ns0:f>IFERROR(INDEX('day5'!$C:$C,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="B9" s="231"/>
+      <ns0:c r="C9" s="231"/>
+      <ns0:c r="D9" s="246" t="inlineStr">
+        <ns0:is>
+          <ns0:t>教师寄语</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" s="246"/>
+      <ns0:c r="F9" s="246"/>
+      <ns0:c r="G9" s="246"/>
+      <ns0:c r="H9" s="246"/>
+      <ns0:c r="I9" s="246"/>
+      <ns0:c r="J9" s="246"/>
+      <ns0:c r="K9" s="246"/>
+    </ns0:row>
+    <ns0:row r="10" spans="1:11" ht="34" customHeight="1">
+      <ns0:c r="A10" s="231"/>
+      <ns0:c r="B10" s="231"/>
+      <ns0:c r="C10" s="231"/>
+      <ns0:c r="D10" s="247">
+        <ns0:f>IFERROR(INDEX('day5'!$J:$J,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="E10" s="247"/>
+      <ns0:c r="F10" s="247"/>
+      <ns0:c r="G10" s="247"/>
+      <ns0:c r="H10" s="247"/>
+      <ns0:c r="I10" s="247"/>
+      <ns0:c r="J10" s="247"/>
+      <ns0:c r="K10" s="247"/>
+    </ns0:row>
+    <ns0:row r="11" spans="1:11" ht="8" customHeight="1">
+      <ns0:c r="A11" s="236" t="inlineStr">
+        <ns0:is>
+          <ns0:t>代码能力</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="231"/>
+      <ns0:c r="C11" s="231"/>
+      <ns0:c r="D11" s="247"/>
+      <ns0:c r="E11" s="247"/>
+      <ns0:c r="F11" s="247"/>
+      <ns0:c r="G11" s="247"/>
+      <ns0:c r="H11" s="247"/>
+      <ns0:c r="I11" s="247"/>
+      <ns0:c r="J11" s="247"/>
+      <ns0:c r="K11" s="247"/>
+    </ns0:row>
+    <ns0:row r="12" spans="1:11" ht="26" customHeight="1">
+      <ns0:c r="A12" s="237">
+        <ns0:f>IFERROR(INDEX('day5'!$D:$D,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="B12" s="231"/>
+      <ns0:c r="C12" s="231"/>
+      <ns0:c r="D12" s="247"/>
+      <ns0:c r="E12" s="247"/>
+      <ns0:c r="F12" s="247"/>
+      <ns0:c r="G12" s="247"/>
+      <ns0:c r="H12" s="247"/>
+      <ns0:c r="I12" s="247"/>
+      <ns0:c r="J12" s="247"/>
+      <ns0:c r="K12" s="247"/>
+    </ns0:row>
+    <ns0:row r="13" spans="1:11" ht="62" customHeight="1">
+      <ns0:c r="A13" s="231"/>
+      <ns0:c r="B13" s="231"/>
+      <ns0:c r="C13" s="231"/>
+      <ns0:c r="D13" s="247"/>
+      <ns0:c r="E13" s="247"/>
+      <ns0:c r="F13" s="247"/>
+      <ns0:c r="G13" s="247"/>
+      <ns0:c r="H13" s="247"/>
+      <ns0:c r="I13" s="247"/>
+      <ns0:c r="J13" s="247"/>
+      <ns0:c r="K13" s="247"/>
+    </ns0:row>
+    <ns0:row r="14" spans="1:11" ht="62" customHeight="1">
+      <ns0:c r="A14" s="236" t="inlineStr">
+        <ns0:is>
+          <ns0:t>理解能力</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="231"/>
+      <ns0:c r="C14" s="231"/>
+      <ns0:c r="D14" s="247"/>
+      <ns0:c r="E14" s="247"/>
+      <ns0:c r="F14" s="247"/>
+      <ns0:c r="G14" s="247"/>
+      <ns0:c r="H14" s="247"/>
+      <ns0:c r="I14" s="247"/>
+      <ns0:c r="J14" s="247"/>
+      <ns0:c r="K14" s="247"/>
+    </ns0:row>
+    <ns0:row r="15" spans="1:11" ht="8" customHeight="1">
+      <ns0:c r="A15" s="237">
+        <ns0:f>IFERROR(INDEX('day5'!$E:$E,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="B15" s="231"/>
+      <ns0:c r="C15" s="231"/>
+      <ns0:c r="D15" s="230"/>
+      <ns0:c r="E15" s="230"/>
+      <ns0:c r="F15" s="230"/>
+      <ns0:c r="G15" s="230"/>
+      <ns0:c r="H15" s="230"/>
+      <ns0:c r="I15" s="230"/>
+      <ns0:c r="J15" s="230"/>
+      <ns0:c r="K15" s="230"/>
+    </ns0:row>
+    <ns0:row r="16" spans="1:11" ht="26" customHeight="1">
+      <ns0:c r="A16" s="231"/>
+      <ns0:c r="B16" s="231"/>
+      <ns0:c r="C16" s="231"/>
+      <ns0:c r="D16" s="248" t="inlineStr">
+        <ns0:is>
+          <ns0:t>学生总结</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E16" s="248"/>
+      <ns0:c r="F16" s="248"/>
+      <ns0:c r="G16" s="248" t="inlineStr">
+        <ns0:is>
+          <ns0:t>学生反思</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H16" s="248"/>
+      <ns0:c r="I16" s="248" t="inlineStr">
+        <ns0:is>
+          <ns0:t>后续计划</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J16" s="248"/>
+      <ns0:c r="K16" s="248"/>
+    </ns0:row>
+    <ns0:row r="17" spans="1:11" ht="52" customHeight="1">
+      <ns0:c r="A17" s="236" t="inlineStr">
+        <ns0:is>
+          <ns0:t>综合评价</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="231"/>
+      <ns0:c r="C17" s="231"/>
+      <ns0:c r="D17" s="249">
+        <ns0:f>IFERROR(INDEX('day5'!$G:$G,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="E17" s="249"/>
+      <ns0:c r="F17" s="249"/>
+      <ns0:c r="G17" s="249">
+        <ns0:f>IFERROR(INDEX('day5'!$H:$H,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="H17" s="249"/>
+      <ns0:c r="I17" s="249">
+        <ns0:f>IFERROR(INDEX('day5'!$I:$I,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="J17" s="249"/>
+      <ns0:c r="K17" s="249"/>
+    </ns0:row>
+    <ns0:row r="18" spans="1:11" ht="52" customHeight="1">
+      <ns0:c r="A18" s="238">
+        <ns0:f>IFERROR(INDEX('day5'!$F:$F,MATCH($A$6,'day5'!$B:$B,0)),"")</ns0:f>
+      </ns0:c>
+      <ns0:c r="B18" s="231"/>
+      <ns0:c r="C18" s="231"/>
+      <ns0:c r="D18" s="249"/>
+      <ns0:c r="E18" s="249"/>
+      <ns0:c r="F18" s="249"/>
+      <ns0:c r="G18" s="249"/>
+      <ns0:c r="H18" s="249"/>
+      <ns0:c r="I18" s="249"/>
+      <ns0:c r="J18" s="249"/>
+      <ns0:c r="K18" s="249"/>
+    </ns0:row>
+    <ns0:row r="19" spans="1:11" ht="52" customHeight="1">
+      <ns0:c r="A19" s="231"/>
+      <ns0:c r="B19" s="231"/>
+      <ns0:c r="C19" s="231"/>
+      <ns0:c r="D19" s="249"/>
+      <ns0:c r="E19" s="249"/>
+      <ns0:c r="F19" s="249"/>
+      <ns0:c r="G19" s="249"/>
+      <ns0:c r="H19" s="249"/>
+      <ns0:c r="I19" s="249"/>
+      <ns0:c r="J19" s="249"/>
+      <ns0:c r="K19" s="249"/>
+    </ns0:row>
+    <ns0:row r="20" spans="1:11" ht="8" customHeight="1">
+      <ns0:c r="A20" s="231"/>
+      <ns0:c r="B20" s="231"/>
+      <ns0:c r="C20" s="231"/>
+      <ns0:c r="D20" s="230"/>
+      <ns0:c r="E20" s="230"/>
+      <ns0:c r="F20" s="230"/>
+      <ns0:c r="G20" s="230"/>
+      <ns0:c r="H20" s="230"/>
+      <ns0:c r="I20" s="230"/>
+      <ns0:c r="J20" s="230"/>
+      <ns0:c r="K20" s="230"/>
+    </ns0:row>
+    <ns0:row r="21" spans="1:11" ht="26" customHeight="1">
+      <ns0:c r="A21" s="231"/>
+      <ns0:c r="B21" s="231"/>
+      <ns0:c r="C21" s="231"/>
+      <ns0:c r="D21" s="250" t="inlineStr">
+        <ns0:is>
+          <ns0:t>使用方式</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E21" s="251"/>
+      <ns0:c r="F21" s="251"/>
+      <ns0:c r="G21" s="251"/>
+      <ns0:c r="H21" s="251"/>
+      <ns0:c r="I21" s="251"/>
+      <ns0:c r="J21" s="251"/>
+      <ns0:c r="K21" s="251"/>
+    </ns0:row>
+    <ns0:row r="22" spans="1:11" ht="62" customHeight="1">
+      <ns0:c r="A22" s="239" t="inlineStr">
+        <ns0:is>
+          <ns0:t>预览数据源</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" s="231"/>
+      <ns0:c r="C22" s="231"/>
+      <ns0:c r="D22" s="251" t="inlineStr">
+        <ns0:is>
+          <ns0:t>在左侧黄色输入框选择 day5 模板中的学生画像或姓名，右侧内容会自动更新。这个版式更适合导出 PDF 或截图发给家长。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E22" s="251"/>
+      <ns0:c r="F22" s="251"/>
+      <ns0:c r="G22" s="251"/>
+      <ns0:c r="H22" s="251"/>
+      <ns0:c r="I22" s="251"/>
+      <ns0:c r="J22" s="251"/>
+      <ns0:c r="K22" s="251"/>
+    </ns0:row>
+    <ns0:row r="23" spans="1:11" ht="62" customHeight="1">
+      <ns0:c r="A23" s="240" t="inlineStr">
+        <ns0:is>
+          <ns0:t>day5 模板页</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" s="231"/>
+      <ns0:c r="C23" s="231"/>
+      <ns0:c r="D23" s="251"/>
+      <ns0:c r="E23" s="251"/>
+      <ns0:c r="F23" s="251"/>
+      <ns0:c r="G23" s="251"/>
+      <ns0:c r="H23" s="251"/>
+      <ns0:c r="I23" s="251"/>
+      <ns0:c r="J23" s="251"/>
+      <ns0:c r="K23" s="251"/>
+    </ns0:row>
+    <ns0:row r="24" spans="1:11" ht="62" customHeight="1">
+      <ns0:c r="A24" s="231"/>
+      <ns0:c r="B24" s="231"/>
+      <ns0:c r="C24" s="231"/>
+      <ns0:c r="D24" s="251"/>
+      <ns0:c r="E24" s="251"/>
+      <ns0:c r="F24" s="251"/>
+      <ns0:c r="G24" s="251"/>
+      <ns0:c r="H24" s="251"/>
+      <ns0:c r="I24" s="251"/>
+      <ns0:c r="J24" s="251"/>
+      <ns0:c r="K24" s="251"/>
+    </ns0:row>
+    <ns0:row r="25" spans="1:11" ht="18" customHeight="1">
+      <ns0:c r="A25" s="231"/>
+      <ns0:c r="B25" s="231"/>
+      <ns0:c r="C25" s="231"/>
+      <ns0:c r="D25" s="230"/>
+      <ns0:c r="E25" s="230"/>
+      <ns0:c r="F25" s="230"/>
+      <ns0:c r="G25" s="230"/>
+      <ns0:c r="H25" s="230"/>
+      <ns0:c r="I25" s="230"/>
+      <ns0:c r="J25" s="230"/>
+      <ns0:c r="K25" s="230"/>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:mergeCells count="29">
+    <ns0:mergeCell ref="A1:C1"/>
+    <ns0:mergeCell ref="A2:C2"/>
+    <ns0:mergeCell ref="A3:C3"/>
+    <ns0:mergeCell ref="A5:C5"/>
+    <ns0:mergeCell ref="A6:C6"/>
+    <ns0:mergeCell ref="A8:C8"/>
+    <ns0:mergeCell ref="A9:C10"/>
+    <ns0:mergeCell ref="A11:C11"/>
+    <ns0:mergeCell ref="A12:C13"/>
+    <ns0:mergeCell ref="A14:C14"/>
+    <ns0:mergeCell ref="A15:C16"/>
+    <ns0:mergeCell ref="A17:C17"/>
+    <ns0:mergeCell ref="A18:C20"/>
+    <ns0:mergeCell ref="A22:C22"/>
+    <ns0:mergeCell ref="A23:C23"/>
+    <ns0:mergeCell ref="D1:K2"/>
+    <ns0:mergeCell ref="D3:K3"/>
+    <ns0:mergeCell ref="D5:K5"/>
+    <ns0:mergeCell ref="D6:K7"/>
+    <ns0:mergeCell ref="D9:K9"/>
+    <ns0:mergeCell ref="D10:K14"/>
+    <ns0:mergeCell ref="D16:F16"/>
+    <ns0:mergeCell ref="D17:F19"/>
+    <ns0:mergeCell ref="G16:H16"/>
+    <ns0:mergeCell ref="G17:H19"/>
+    <ns0:mergeCell ref="I16:K16"/>
+    <ns0:mergeCell ref="I17:K19"/>
+    <ns0:mergeCell ref="D21:K21"/>
+    <ns0:mergeCell ref="D22:K24"/>
+  </ns0:mergeCells>
+  <ns0:dataValidations count="1">
+    <ns0:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A6">
+      <ns0:formula1>'day5'!$B:$B</ns0:formula1>
+    </ns0:dataValidation>
+  </ns0:dataValidations>
+  <ns0:pageMargins left="0.25" right="0.25" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
+  <ns0:pageSetup orientation="portrait" paperSize="9"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>